<commit_message>
wip pertumbuhan balita, kpsp, m chat 1 dan 2
</commit_message>
<xml_diff>
--- a/dataset/anak.xlsx
+++ b/dataset/anak.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FED85201-F37D-3B41-BDB8-F583A1B5B6E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{941C8527-990D-0643-8DAE-55A5031FBC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4480" yWindow="-21000" windowWidth="36000" windowHeight="19540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
     <author>Microsoft Office User</author>
   </authors>
   <commentList>
-    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000016000000}">
+    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -40,7 +40,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000017000000}">
+    <comment ref="Q1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -55,7 +55,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000018000000}">
+    <comment ref="R1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -70,7 +70,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000019000000}">
+    <comment ref="W1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -85,7 +85,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BZ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001A000000}">
+    <comment ref="CC1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
       <text>
         <r>
           <rPr>
@@ -100,7 +100,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CC1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001B000000}">
+    <comment ref="CF1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -115,7 +115,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001C000000}">
+    <comment ref="CK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -130,7 +130,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001D000000}">
+    <comment ref="CN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -145,7 +145,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CR1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001E000000}">
+    <comment ref="CU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -160,7 +160,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CT1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001F000000}">
+    <comment ref="CW1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -175,7 +175,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000020000000}">
+    <comment ref="CX1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -190,7 +190,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000021000000}">
+    <comment ref="CY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
       <text>
         <r>
           <rPr>
@@ -205,7 +205,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CW1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000022000000}">
+    <comment ref="CZ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
       <text>
         <r>
           <rPr>
@@ -220,7 +220,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000023000000}">
+    <comment ref="DJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
       <text>
         <r>
           <rPr>
@@ -235,7 +235,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000024000000}">
+    <comment ref="EB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
       <text>
         <r>
           <rPr>
@@ -255,7 +255,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="238">
   <si>
     <t>batas_awal</t>
   </si>
@@ -272,18 +272,12 @@
     <t>disabilitas</t>
   </si>
   <si>
-    <t>periksa_gizi_laki</t>
-  </si>
-  <si>
     <t>berat_badan</t>
   </si>
   <si>
     <t>tinggi_badan</t>
   </si>
   <si>
-    <t>lingkar_perut</t>
-  </si>
-  <si>
     <t>periksa_gula_darah</t>
   </si>
   <si>
@@ -716,162 +710,171 @@
     <t>status</t>
   </si>
   <si>
+    <t>2026-05-18</t>
+  </si>
+  <si>
+    <t>2026-05-24</t>
+  </si>
+  <si>
+    <t>ARKANA NAUFAL</t>
+  </si>
+  <si>
+    <t>Non disabilitas</t>
+  </si>
+  <si>
+    <t>True</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>175</t>
+  </si>
+  <si>
+    <t>90</t>
+  </si>
+  <si>
+    <t>Ya</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>110</t>
+  </si>
+  <si>
+    <t>120</t>
+  </si>
+  <si>
+    <t>Benar semua</t>
+  </si>
+  <si>
+    <t>Tidak terkendali/tak teratur (perlu pencahar)</t>
+  </si>
+  <si>
+    <t>Kadang-kadang tak terkendali (hanya 1 x / 24 jam)</t>
+  </si>
+  <si>
+    <t>Mandiri</t>
+  </si>
+  <si>
+    <t>Bisa (pindah) dengan kursi roda</t>
+  </si>
+  <si>
+    <t>Sebagian dibantu (misalnya: mengancing baju)</t>
+  </si>
+  <si>
+    <t>Butuh pertolongan</t>
+  </si>
+  <si>
+    <t>SUDAH DITANYAKAN</t>
+  </si>
+  <si>
+    <t>Benar</t>
+  </si>
+  <si>
+    <t>Benar semua kata</t>
+  </si>
+  <si>
+    <t>Tidak, Berubah</t>
+  </si>
+  <si>
+    <t>Tidak Berubah</t>
+  </si>
+  <si>
+    <t>Tidak Tahu</t>
+  </si>
+  <si>
+    <t>Bertahan 10 detik</t>
+  </si>
+  <si>
+    <t>4.83 - 6.20 detik</t>
+  </si>
+  <si>
+    <t>&lt;11.19 detik</t>
+  </si>
+  <si>
+    <t>Nafsu Makan Yang Sangat Berkurang</t>
+  </si>
+  <si>
+    <t>Penurunan BB &gt; 3 Kg</t>
+  </si>
+  <si>
+    <t>Harus berbaring di tempat tidur atau menggunakan kursi roda</t>
+  </si>
+  <si>
+    <t>Dementia atau depresi berat</t>
+  </si>
+  <si>
+    <t>IMT &lt;19</t>
+  </si>
+  <si>
+    <t>&lt;31 cm</t>
+  </si>
+  <si>
+    <t>Tidak batuk</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Riwayat kontak serumah</t>
+  </si>
+  <si>
+    <t>Bakteriologis</t>
+  </si>
+  <si>
+    <t>TCM</t>
+  </si>
+  <si>
+    <t>Mtb not detected (Neg)</t>
+  </si>
+  <si>
+    <t>Suspek frambusia</t>
+  </si>
+  <si>
+    <t>Reaktif</t>
+  </si>
+  <si>
+    <t>Meragukan</t>
+  </si>
+  <si>
+    <t>Kusta</t>
+  </si>
+  <si>
+    <t>Tidak Ada</t>
+  </si>
+  <si>
+    <t>Tidak ada serumen impaksi</t>
+  </si>
+  <si>
+    <t>Tidak ada infeksi telinga</t>
+  </si>
+  <si>
+    <t>Curiga gangguan pendengaran</t>
+  </si>
+  <si>
+    <t>Gangguan Pendengaran</t>
+  </si>
+  <si>
+    <t>Curiga gangguan penglihatan (visus &lt;6/12)</t>
+  </si>
+  <si>
+    <t>Gangguan penglihatan ringan (visus &lt;6/12 - 6/18)</t>
+  </si>
+  <si>
+    <t>Visus membaik</t>
+  </si>
+  <si>
+    <t>Kelainan refraksi ringan (0.50 - 3.00 Dioptri)</t>
+  </si>
+  <si>
+    <t>Curiga katarak</t>
+  </si>
+  <si>
     <t>Tidak</t>
   </si>
   <si>
-    <t>Non disabilitas</t>
-  </si>
-  <si>
-    <t>Ya</t>
-  </si>
-  <si>
-    <t>True</t>
-  </si>
-  <si>
-    <t>80</t>
-  </si>
-  <si>
-    <t>175</t>
-  </si>
-  <si>
-    <t>90</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>110</t>
-  </si>
-  <si>
-    <t>120</t>
-  </si>
-  <si>
-    <t>Benar semua</t>
-  </si>
-  <si>
-    <t>Tidak terkendali/tak teratur (perlu pencahar)</t>
-  </si>
-  <si>
-    <t>Kadang-kadang tak terkendali (hanya 1 x / 24 jam)</t>
-  </si>
-  <si>
-    <t>Mandiri</t>
-  </si>
-  <si>
-    <t>Bisa (pindah) dengan kursi roda</t>
-  </si>
-  <si>
-    <t>Sebagian dibantu (misalnya: mengancing baju)</t>
-  </si>
-  <si>
-    <t>Butuh pertolongan</t>
-  </si>
-  <si>
-    <t>SUDAH DITANYAKAN</t>
-  </si>
-  <si>
-    <t>Benar</t>
-  </si>
-  <si>
-    <t>Benar semua kata</t>
-  </si>
-  <si>
-    <t>Tidak, Berubah</t>
-  </si>
-  <si>
-    <t>Tidak Berubah</t>
-  </si>
-  <si>
-    <t>Tidak Tahu</t>
-  </si>
-  <si>
-    <t>Bertahan 10 detik</t>
-  </si>
-  <si>
-    <t>4.83 - 6.20 detik</t>
-  </si>
-  <si>
-    <t>&lt;11.19 detik</t>
-  </si>
-  <si>
-    <t>Nafsu Makan Yang Sangat Berkurang</t>
-  </si>
-  <si>
-    <t>Penurunan BB &gt; 3 Kg</t>
-  </si>
-  <si>
-    <t>Harus berbaring di tempat tidur atau menggunakan kursi roda</t>
-  </si>
-  <si>
-    <t>Dementia atau depresi berat</t>
-  </si>
-  <si>
-    <t>IMT &lt;19</t>
-  </si>
-  <si>
-    <t>&lt;31 cm</t>
-  </si>
-  <si>
-    <t>Tidak batuk</t>
-  </si>
-  <si>
-    <t>Normal</t>
-  </si>
-  <si>
-    <t>Riwayat kontak serumah</t>
-  </si>
-  <si>
-    <t>Bakteriologis</t>
-  </si>
-  <si>
-    <t>TCM</t>
-  </si>
-  <si>
-    <t>Mtb not detected (Neg)</t>
-  </si>
-  <si>
-    <t>Suspek frambusia</t>
-  </si>
-  <si>
-    <t>Reaktif</t>
-  </si>
-  <si>
-    <t>Meragukan</t>
-  </si>
-  <si>
-    <t>Kusta</t>
-  </si>
-  <si>
-    <t>Tidak Ada</t>
-  </si>
-  <si>
-    <t>Tidak ada serumen impaksi</t>
-  </si>
-  <si>
-    <t>Tidak ada infeksi telinga</t>
-  </si>
-  <si>
-    <t>Curiga gangguan pendengaran</t>
-  </si>
-  <si>
-    <t>Gangguan Pendengaran</t>
-  </si>
-  <si>
-    <t>Curiga gangguan penglihatan (visus &lt;6/12)</t>
-  </si>
-  <si>
-    <t>Gangguan penglihatan ringan (visus &lt;6/12 - 6/18)</t>
-  </si>
-  <si>
-    <t>Visus membaik</t>
-  </si>
-  <si>
-    <t>Kelainan refraksi ringan (0.50 - 3.00 Dioptri)</t>
-  </si>
-  <si>
-    <t>Curiga katarak</t>
-  </si>
-  <si>
     <t>Iya</t>
   </si>
   <si>
@@ -944,16 +947,28 @@
     <t>Pernah didiagnosis tuberkulosis (TBC)</t>
   </si>
   <si>
-    <t>SUCCESS</t>
-  </si>
-  <si>
-    <t>ARKANA NAUFAL</t>
-  </si>
-  <si>
-    <t>2026-05-18</t>
-  </si>
-  <si>
-    <t>2026-05-24</t>
+    <t>posisi_pengukuran</t>
+  </si>
+  <si>
+    <t>Berdiri</t>
+  </si>
+  <si>
+    <t>status_lingkar_kepala</t>
+  </si>
+  <si>
+    <t>Makrosefali</t>
+  </si>
+  <si>
+    <t>hasil_kpsp</t>
+  </si>
+  <si>
+    <t>Perkembangan sesuai usia</t>
+  </si>
+  <si>
+    <t>m_chat_1</t>
+  </si>
+  <si>
+    <t>m_chat_2</t>
   </si>
 </sst>
 </file>
@@ -985,7 +1000,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="1" tint="0.14993743705557422"/>
+        <fgColor theme="1" tint="0.14990691854609822"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -1356,7 +1371,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:EX2"/>
+  <dimension ref="A1:FA2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -1365,119 +1380,121 @@
     <col min="4" max="4" width="10.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="14.33203125" customWidth="1"/>
-    <col min="11" max="11" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="17.1640625" customWidth="1"/>
-    <col min="18" max="18" width="12" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.83203125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="21" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="18" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="21.83203125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="21.1640625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="42.1640625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="38" max="39" width="18.1640625" customWidth="1"/>
-    <col min="40" max="40" width="27.1640625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="40" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="16" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="16" customWidth="1"/>
-    <col min="44" max="44" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="47" max="50" width="15.83203125" customWidth="1"/>
-    <col min="51" max="70" width="10.5" customWidth="1"/>
-    <col min="71" max="71" width="16" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="25" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="14.83203125" customWidth="1"/>
-    <col min="79" max="79" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="22.83203125" customWidth="1"/>
-    <col min="84" max="84" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="16.1640625" customWidth="1"/>
-    <col min="86" max="86" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="88" max="89" width="12.33203125" customWidth="1"/>
-    <col min="90" max="90" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="14.1640625" customWidth="1"/>
-    <col min="92" max="92" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="23.6640625" customWidth="1"/>
-    <col min="95" max="95" width="26" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="26" customWidth="1"/>
-    <col min="97" max="97" width="36.1640625" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="41.5" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="29" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="102" max="103" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="104" max="105" width="12.83203125" customWidth="1"/>
-    <col min="106" max="106" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="17.5" customWidth="1"/>
-    <col min="109" max="109" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="13" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="112" max="112" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="113" max="115" width="19.5" customWidth="1"/>
-    <col min="116" max="116" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="117" max="117" width="9.83203125" customWidth="1"/>
-    <col min="118" max="118" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="119" max="122" width="11.5" customWidth="1"/>
-    <col min="123" max="123" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="124" max="124" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="125" max="125" width="9" bestFit="1" customWidth="1"/>
-    <col min="126" max="126" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="18.1640625" customWidth="1"/>
-    <col min="130" max="130" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="131" max="131" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="132" max="134" width="8.33203125" customWidth="1"/>
-    <col min="135" max="135" width="22" bestFit="1" customWidth="1"/>
-    <col min="136" max="136" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="137" max="137" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="138" max="138" width="14" bestFit="1" customWidth="1"/>
-    <col min="139" max="139" width="14" customWidth="1"/>
-    <col min="140" max="140" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="141" max="141" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="142" max="142" width="18.1640625" customWidth="1"/>
-    <col min="143" max="143" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="144" max="144" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="145" max="145" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="146" max="148" width="18.1640625" customWidth="1"/>
-    <col min="149" max="149" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="150" max="150" width="35" bestFit="1" customWidth="1"/>
-    <col min="151" max="151" width="43.1640625" bestFit="1" customWidth="1"/>
-    <col min="152" max="152" width="18.1640625" customWidth="1"/>
-    <col min="153" max="153" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="154" max="154" width="10.83203125" customWidth="1"/>
+    <col min="7" max="8" width="14.33203125" customWidth="1"/>
+    <col min="9" max="9" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="19" customWidth="1"/>
+    <col min="14" max="14" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="17.1640625" customWidth="1"/>
+    <col min="21" max="21" width="12" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="8" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="16" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="21" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="18" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="21.83203125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="11" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="42.1640625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="41" max="42" width="18.1640625" customWidth="1"/>
+    <col min="43" max="43" width="27.1640625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="40" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="16" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="16" customWidth="1"/>
+    <col min="47" max="47" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="50" max="53" width="15.83203125" customWidth="1"/>
+    <col min="54" max="73" width="10.5" customWidth="1"/>
+    <col min="74" max="74" width="16" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="25" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="14.83203125" customWidth="1"/>
+    <col min="82" max="82" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="22.83203125" customWidth="1"/>
+    <col min="87" max="87" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="16.1640625" customWidth="1"/>
+    <col min="89" max="89" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="91" max="92" width="12.33203125" customWidth="1"/>
+    <col min="93" max="93" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="14.1640625" customWidth="1"/>
+    <col min="95" max="95" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="23.6640625" customWidth="1"/>
+    <col min="98" max="98" width="26" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="26" customWidth="1"/>
+    <col min="100" max="100" width="36.1640625" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="41.5" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="29" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="105" max="106" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="107" max="108" width="12.83203125" customWidth="1"/>
+    <col min="109" max="109" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="110" max="110" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="17.5" customWidth="1"/>
+    <col min="112" max="112" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="13" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="115" max="115" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="116" max="118" width="19.5" customWidth="1"/>
+    <col min="119" max="119" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="9.83203125" customWidth="1"/>
+    <col min="121" max="121" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="122" max="125" width="11.5" customWidth="1"/>
+    <col min="126" max="126" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="127" max="127" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="128" max="128" width="9" bestFit="1" customWidth="1"/>
+    <col min="129" max="129" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="130" max="130" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="131" max="131" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="132" max="132" width="18.1640625" customWidth="1"/>
+    <col min="133" max="133" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="134" max="134" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="135" max="137" width="8.33203125" customWidth="1"/>
+    <col min="138" max="138" width="22" bestFit="1" customWidth="1"/>
+    <col min="139" max="139" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="140" max="140" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="141" max="141" width="14" bestFit="1" customWidth="1"/>
+    <col min="142" max="142" width="14" customWidth="1"/>
+    <col min="143" max="143" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="144" max="144" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="145" max="145" width="18.1640625" customWidth="1"/>
+    <col min="146" max="146" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="147" max="147" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="148" max="148" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="149" max="151" width="18.1640625" customWidth="1"/>
+    <col min="152" max="152" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="153" max="153" width="35" bestFit="1" customWidth="1"/>
+    <col min="154" max="154" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="155" max="155" width="18.1640625" customWidth="1"/>
+    <col min="156" max="156" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="157" max="157" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:154" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:157" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1500,453 +1517,462 @@
         <v>6</v>
       </c>
       <c r="I1" t="s">
+        <v>230</v>
+      </c>
+      <c r="J1" t="s">
+        <v>232</v>
+      </c>
+      <c r="K1" t="s">
+        <v>234</v>
+      </c>
+      <c r="L1" t="s">
+        <v>236</v>
+      </c>
+      <c r="M1" t="s">
+        <v>237</v>
+      </c>
+      <c r="N1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="O1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+      <c r="P1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="Q1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" t="s">
+      <c r="R1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" t="s">
+      <c r="S1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" t="s">
+      <c r="T1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" t="s">
+      <c r="U1" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="V1" t="s">
         <v>15</v>
       </c>
-      <c r="R1" t="s">
+      <c r="W1" t="s">
         <v>16</v>
       </c>
-      <c r="S1" t="s">
+      <c r="X1" t="s">
         <v>17</v>
       </c>
-      <c r="T1" t="s">
+      <c r="Y1" t="s">
         <v>18</v>
       </c>
-      <c r="U1" t="s">
+      <c r="Z1" t="s">
         <v>19</v>
       </c>
-      <c r="V1" t="s">
+      <c r="AA1" t="s">
         <v>20</v>
       </c>
-      <c r="W1" t="s">
+      <c r="AB1" t="s">
         <v>21</v>
       </c>
-      <c r="X1" t="s">
+      <c r="AC1" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="AD1" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AE1" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AF1" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AG1" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AH1" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AI1" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AJ1" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AK1" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AL1" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AM1" t="s">
         <v>32</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AN1" t="s">
         <v>33</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AO1" t="s">
         <v>34</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AP1" t="s">
         <v>35</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AQ1" t="s">
         <v>36</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AR1" t="s">
         <v>37</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AS1" t="s">
         <v>38</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AT1" t="s">
         <v>39</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AU1" t="s">
         <v>40</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AV1" t="s">
         <v>41</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AW1" t="s">
         <v>42</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AX1" t="s">
         <v>43</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AY1" t="s">
         <v>44</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AZ1" t="s">
         <v>45</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="BA1" t="s">
         <v>46</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="BB1" t="s">
         <v>47</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="BC1" t="s">
         <v>48</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="BD1" t="s">
         <v>49</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BE1" t="s">
         <v>50</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BF1" t="s">
         <v>51</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BG1" t="s">
         <v>52</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BH1" t="s">
         <v>53</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BI1" t="s">
         <v>54</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BJ1" t="s">
         <v>55</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BK1" t="s">
         <v>56</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BL1" t="s">
         <v>57</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BM1" t="s">
         <v>58</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BN1" t="s">
         <v>59</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BO1" t="s">
         <v>60</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BP1" t="s">
         <v>61</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BQ1" t="s">
         <v>62</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BR1" t="s">
         <v>63</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BS1" t="s">
         <v>64</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BT1" t="s">
         <v>65</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BU1" t="s">
         <v>66</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BV1" t="s">
         <v>67</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BW1" t="s">
         <v>68</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BX1" t="s">
         <v>69</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BY1" t="s">
         <v>70</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BZ1" t="s">
         <v>71</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="CA1" t="s">
         <v>72</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="CB1" t="s">
         <v>73</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CC1" t="s">
         <v>74</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CD1" t="s">
         <v>75</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CE1" t="s">
         <v>76</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CF1" t="s">
         <v>77</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CG1" t="s">
         <v>78</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CH1" t="s">
         <v>79</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CI1" t="s">
         <v>80</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CJ1" t="s">
         <v>81</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CK1" t="s">
         <v>82</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CL1" t="s">
         <v>83</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CM1" t="s">
         <v>84</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CN1" t="s">
         <v>85</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CO1" t="s">
         <v>86</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CP1" t="s">
         <v>87</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CQ1" t="s">
         <v>88</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CR1" t="s">
         <v>89</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CS1" t="s">
         <v>90</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CT1" t="s">
         <v>91</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="CU1" t="s">
         <v>92</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="CV1" t="s">
         <v>93</v>
       </c>
-      <c r="CR1" t="s">
+      <c r="CW1" t="s">
         <v>94</v>
       </c>
-      <c r="CS1" t="s">
+      <c r="CX1" t="s">
         <v>95</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="CY1" t="s">
         <v>96</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="CZ1" t="s">
         <v>97</v>
       </c>
-      <c r="CV1" t="s">
+      <c r="DA1" t="s">
         <v>98</v>
       </c>
-      <c r="CW1" t="s">
+      <c r="DB1" t="s">
         <v>99</v>
       </c>
-      <c r="CX1" t="s">
+      <c r="DC1" t="s">
         <v>100</v>
       </c>
-      <c r="CY1" t="s">
+      <c r="DD1" t="s">
         <v>101</v>
       </c>
-      <c r="CZ1" t="s">
+      <c r="DE1" t="s">
         <v>102</v>
       </c>
-      <c r="DA1" t="s">
+      <c r="DF1" t="s">
         <v>103</v>
       </c>
-      <c r="DB1" t="s">
+      <c r="DG1" t="s">
         <v>104</v>
       </c>
-      <c r="DC1" t="s">
+      <c r="DH1" t="s">
         <v>105</v>
       </c>
-      <c r="DD1" t="s">
+      <c r="DI1" t="s">
         <v>106</v>
       </c>
-      <c r="DE1" t="s">
+      <c r="DJ1" t="s">
         <v>107</v>
       </c>
-      <c r="DF1" t="s">
+      <c r="DK1" t="s">
         <v>108</v>
       </c>
-      <c r="DG1" t="s">
+      <c r="DL1" t="s">
         <v>109</v>
       </c>
-      <c r="DH1" t="s">
+      <c r="DM1" t="s">
         <v>110</v>
       </c>
-      <c r="DI1" t="s">
+      <c r="DN1" t="s">
         <v>111</v>
       </c>
-      <c r="DJ1" t="s">
+      <c r="DO1" t="s">
         <v>112</v>
       </c>
-      <c r="DK1" t="s">
+      <c r="DP1" t="s">
         <v>113</v>
       </c>
-      <c r="DL1" t="s">
+      <c r="DQ1" t="s">
         <v>114</v>
       </c>
-      <c r="DM1" t="s">
+      <c r="DR1" t="s">
         <v>115</v>
       </c>
-      <c r="DN1" t="s">
+      <c r="DS1" t="s">
         <v>116</v>
       </c>
-      <c r="DO1" t="s">
+      <c r="DT1" t="s">
         <v>117</v>
       </c>
-      <c r="DP1" t="s">
+      <c r="DU1" t="s">
         <v>118</v>
       </c>
-      <c r="DQ1" t="s">
+      <c r="DV1" t="s">
         <v>119</v>
       </c>
-      <c r="DR1" t="s">
+      <c r="DW1" t="s">
         <v>120</v>
       </c>
-      <c r="DS1" t="s">
+      <c r="DX1" t="s">
         <v>121</v>
       </c>
-      <c r="DT1" t="s">
+      <c r="DY1" t="s">
         <v>122</v>
       </c>
-      <c r="DU1" t="s">
+      <c r="DZ1" t="s">
         <v>123</v>
       </c>
-      <c r="DV1" t="s">
+      <c r="EA1" t="s">
         <v>124</v>
       </c>
-      <c r="DW1" t="s">
+      <c r="EB1" t="s">
         <v>125</v>
       </c>
-      <c r="DX1" t="s">
+      <c r="EC1" t="s">
         <v>126</v>
       </c>
-      <c r="DY1" t="s">
+      <c r="ED1" t="s">
         <v>127</v>
       </c>
-      <c r="DZ1" t="s">
+      <c r="EE1" t="s">
         <v>128</v>
       </c>
-      <c r="EA1" t="s">
+      <c r="EF1" t="s">
         <v>129</v>
       </c>
-      <c r="EB1" t="s">
+      <c r="EG1" t="s">
         <v>130</v>
       </c>
-      <c r="EC1" t="s">
+      <c r="EH1" t="s">
         <v>131</v>
       </c>
-      <c r="ED1" t="s">
+      <c r="EI1" t="s">
         <v>132</v>
       </c>
-      <c r="EE1" t="s">
+      <c r="EJ1" t="s">
         <v>133</v>
       </c>
-      <c r="EF1" t="s">
+      <c r="EK1" t="s">
         <v>134</v>
       </c>
-      <c r="EG1" t="s">
+      <c r="EL1" t="s">
         <v>135</v>
       </c>
-      <c r="EH1" t="s">
+      <c r="EM1" t="s">
         <v>136</v>
       </c>
-      <c r="EI1" t="s">
+      <c r="EN1" t="s">
         <v>137</v>
       </c>
-      <c r="EJ1" t="s">
+      <c r="EO1" t="s">
         <v>138</v>
       </c>
-      <c r="EK1" t="s">
+      <c r="EP1" t="s">
         <v>139</v>
       </c>
-      <c r="EL1" t="s">
+      <c r="EQ1" t="s">
         <v>140</v>
       </c>
-      <c r="EM1" t="s">
+      <c r="ER1" t="s">
         <v>141</v>
       </c>
-      <c r="EN1" t="s">
+      <c r="ES1" t="s">
         <v>142</v>
       </c>
-      <c r="EO1" t="s">
+      <c r="ET1" t="s">
         <v>143</v>
       </c>
-      <c r="EP1" t="s">
+      <c r="EU1" t="s">
         <v>144</v>
       </c>
-      <c r="EQ1" t="s">
+      <c r="EV1" t="s">
         <v>145</v>
       </c>
-      <c r="ER1" t="s">
+      <c r="EW1" t="s">
         <v>146</v>
       </c>
-      <c r="ES1" t="s">
+      <c r="EX1" t="s">
         <v>147</v>
       </c>
-      <c r="ET1" t="s">
+      <c r="EY1" t="s">
         <v>148</v>
       </c>
-      <c r="EU1" t="s">
+      <c r="EZ1" t="s">
         <v>149</v>
       </c>
-      <c r="EV1" t="s">
+      <c r="FA1" t="s">
         <v>150</v>
       </c>
-      <c r="EW1" t="s">
+    </row>
+    <row r="2" spans="1:157" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="EX1" t="s">
+      <c r="B2" s="1" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="2" spans="1:154" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>232</v>
-      </c>
       <c r="C2" t="s">
-        <v>230</v>
+        <v>153</v>
       </c>
       <c r="E2" t="s">
         <v>154</v>
@@ -1958,124 +1984,124 @@
         <v>157</v>
       </c>
       <c r="I2" t="s">
+        <v>231</v>
+      </c>
+      <c r="J2" t="s">
+        <v>233</v>
+      </c>
+      <c r="K2" t="s">
+        <v>235</v>
+      </c>
+      <c r="L2" t="s">
+        <v>159</v>
+      </c>
+      <c r="M2">
+        <v>10</v>
+      </c>
+      <c r="N2" t="s">
+        <v>155</v>
+      </c>
+      <c r="O2" t="s">
+        <v>159</v>
+      </c>
+      <c r="P2" t="s">
+        <v>160</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>161</v>
+      </c>
+      <c r="S2" t="s">
         <v>158</v>
       </c>
-      <c r="J2" t="s">
-        <v>159</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="U2" t="s">
+        <v>155</v>
+      </c>
+      <c r="V2" t="s">
+        <v>159</v>
+      </c>
+      <c r="W2" t="s">
+        <v>160</v>
+      </c>
+      <c r="X2" t="s">
+        <v>162</v>
+      </c>
+      <c r="Y2" t="s">
         <v>156</v>
       </c>
-      <c r="L2" t="s">
-        <v>155</v>
-      </c>
-      <c r="M2" t="s">
-        <v>160</v>
-      </c>
-      <c r="N2" t="s">
-        <v>161</v>
-      </c>
-      <c r="P2" t="s">
-        <v>159</v>
-      </c>
-      <c r="R2" t="s">
-        <v>156</v>
-      </c>
-      <c r="S2" t="s">
-        <v>155</v>
-      </c>
-      <c r="T2" t="s">
-        <v>160</v>
-      </c>
-      <c r="U2" t="s">
-        <v>162</v>
-      </c>
-      <c r="V2" t="s">
-        <v>157</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>155</v>
-      </c>
-      <c r="Z2" t="s">
+      <c r="AB2" t="s">
+        <v>159</v>
+      </c>
+      <c r="AC2" t="s">
         <v>163</v>
       </c>
-      <c r="AA2" t="s">
-        <v>155</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>155</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>155</v>
-      </c>
       <c r="AD2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="AE2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="AF2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="AG2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="AH2" t="s">
+        <v>159</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>159</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>159</v>
+      </c>
+      <c r="AK2" t="s">
         <v>164</v>
       </c>
-      <c r="AI2" t="s">
+      <c r="AL2" t="s">
         <v>165</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>166</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>166</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>166</v>
       </c>
       <c r="AM2" t="s">
         <v>166</v>
       </c>
       <c r="AN2" t="s">
+        <v>166</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>166</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>166</v>
+      </c>
+      <c r="AQ2" t="s">
         <v>167</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AR2" t="s">
         <v>168</v>
       </c>
-      <c r="AP2" t="s">
+      <c r="AS2" t="s">
         <v>169</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="AT2" t="s">
         <v>166</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="AU2" t="s">
         <v>170</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AV2" t="s">
         <v>171</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="AW2" t="s">
         <v>172</v>
       </c>
-      <c r="AU2" t="s">
+      <c r="AX2" t="s">
         <v>173</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="AY2" t="s">
         <v>174</v>
       </c>
-      <c r="AW2" t="s">
+      <c r="AZ2" t="s">
         <v>174</v>
-      </c>
-      <c r="AX2" t="s">
-        <v>175</v>
-      </c>
-      <c r="AY2" t="s">
-        <v>175</v>
-      </c>
-      <c r="AZ2" t="s">
-        <v>175</v>
       </c>
       <c r="BA2" t="s">
         <v>175</v>
@@ -2084,485 +2110,500 @@
         <v>175</v>
       </c>
       <c r="BC2" t="s">
+        <v>175</v>
+      </c>
+      <c r="BD2" t="s">
+        <v>175</v>
+      </c>
+      <c r="BE2" t="s">
+        <v>175</v>
+      </c>
+      <c r="BF2" t="s">
         <v>176</v>
       </c>
-      <c r="BD2" t="s">
+      <c r="BG2" t="s">
         <v>176</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BH2" t="s">
         <v>176</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BI2" t="s">
         <v>177</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BJ2" t="s">
         <v>178</v>
       </c>
-      <c r="BH2" t="s">
+      <c r="BK2" t="s">
         <v>179</v>
       </c>
-      <c r="BI2" t="s">
+      <c r="BL2" t="s">
         <v>180</v>
       </c>
-      <c r="BJ2" t="s">
+      <c r="BM2" t="s">
         <v>181</v>
       </c>
-      <c r="BK2" t="s">
-        <v>155</v>
-      </c>
-      <c r="BL2" t="s">
+      <c r="BN2" t="s">
+        <v>159</v>
+      </c>
+      <c r="BO2" t="s">
         <v>182</v>
       </c>
-      <c r="BM2" t="s">
+      <c r="BP2" t="s">
         <v>183</v>
       </c>
-      <c r="BN2" t="s">
+      <c r="BQ2" t="s">
         <v>184</v>
       </c>
-      <c r="BO2" t="s">
-        <v>155</v>
-      </c>
-      <c r="BP2" t="s">
-        <v>155</v>
-      </c>
-      <c r="BQ2" t="s">
-        <v>155</v>
-      </c>
       <c r="BR2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="BS2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="BT2" t="s">
-        <v>185</v>
+        <v>159</v>
       </c>
       <c r="BU2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="BV2" t="s">
         <v>155</v>
       </c>
       <c r="BW2" t="s">
+        <v>185</v>
+      </c>
+      <c r="BX2" t="s">
+        <v>159</v>
+      </c>
+      <c r="BY2" t="s">
+        <v>159</v>
+      </c>
+      <c r="BZ2" t="s">
+        <v>159</v>
+      </c>
+      <c r="CA2" t="s">
+        <v>159</v>
+      </c>
+      <c r="CB2" t="s">
+        <v>159</v>
+      </c>
+      <c r="CC2" t="s">
+        <v>186</v>
+      </c>
+      <c r="CD2" t="s">
         <v>155</v>
       </c>
-      <c r="BX2" t="s">
+      <c r="CE2" t="s">
+        <v>187</v>
+      </c>
+      <c r="CF2" t="s">
+        <v>188</v>
+      </c>
+      <c r="CG2" t="s">
+        <v>189</v>
+      </c>
+      <c r="CH2" t="s">
+        <v>190</v>
+      </c>
+      <c r="CI2" t="s">
         <v>155</v>
       </c>
-      <c r="BY2" t="s">
+      <c r="CJ2" t="s">
+        <v>191</v>
+      </c>
+      <c r="CK2" t="s">
+        <v>192</v>
+      </c>
+      <c r="CL2" t="s">
         <v>155</v>
       </c>
-      <c r="BZ2" t="s">
+      <c r="CM2" t="s">
+        <v>193</v>
+      </c>
+      <c r="CN2" t="s">
+        <v>194</v>
+      </c>
+      <c r="CO2" t="s">
+        <v>155</v>
+      </c>
+      <c r="CP2" t="s">
+        <v>195</v>
+      </c>
+      <c r="CQ2" t="s">
+        <v>155</v>
+      </c>
+      <c r="CR2" t="s">
+        <v>196</v>
+      </c>
+      <c r="CS2" t="s">
+        <v>197</v>
+      </c>
+      <c r="CT2" t="s">
+        <v>198</v>
+      </c>
+      <c r="CU2" t="s">
+        <v>199</v>
+      </c>
+      <c r="CV2" t="s">
+        <v>200</v>
+      </c>
+      <c r="CW2" t="s">
+        <v>201</v>
+      </c>
+      <c r="CX2" t="s">
+        <v>202</v>
+      </c>
+      <c r="CY2" t="s">
+        <v>203</v>
+      </c>
+      <c r="CZ2" t="s">
         <v>186</v>
       </c>
-      <c r="CA2" t="s">
-        <v>156</v>
-      </c>
-      <c r="CB2" t="s">
-        <v>187</v>
-      </c>
-      <c r="CC2" t="s">
-        <v>188</v>
-      </c>
-      <c r="CD2" t="s">
-        <v>189</v>
-      </c>
-      <c r="CE2" t="s">
-        <v>190</v>
-      </c>
-      <c r="CF2" t="s">
-        <v>156</v>
-      </c>
-      <c r="CG2" t="s">
-        <v>191</v>
-      </c>
-      <c r="CH2" t="s">
-        <v>192</v>
-      </c>
-      <c r="CI2" t="s">
-        <v>156</v>
-      </c>
-      <c r="CJ2" t="s">
-        <v>193</v>
-      </c>
-      <c r="CK2" t="s">
-        <v>194</v>
-      </c>
-      <c r="CL2" t="s">
-        <v>156</v>
-      </c>
-      <c r="CM2" t="s">
-        <v>195</v>
-      </c>
-      <c r="CN2" t="s">
-        <v>156</v>
-      </c>
-      <c r="CO2" t="s">
-        <v>196</v>
-      </c>
-      <c r="CP2" t="s">
-        <v>197</v>
-      </c>
-      <c r="CQ2" t="s">
-        <v>198</v>
-      </c>
-      <c r="CR2" t="s">
-        <v>199</v>
-      </c>
-      <c r="CS2" t="s">
-        <v>200</v>
-      </c>
-      <c r="CT2" t="s">
-        <v>201</v>
-      </c>
-      <c r="CU2" t="s">
-        <v>202</v>
-      </c>
-      <c r="CV2" t="s">
-        <v>203</v>
-      </c>
-      <c r="CW2" t="s">
-        <v>186</v>
-      </c>
-      <c r="CX2" t="s">
+      <c r="DA2" t="s">
         <v>204</v>
       </c>
-      <c r="CY2" t="s">
-        <v>156</v>
-      </c>
-      <c r="CZ2" t="s">
+      <c r="DB2" t="s">
         <v>155</v>
       </c>
-      <c r="DA2" t="s">
-        <v>153</v>
-      </c>
-      <c r="DB2" t="s">
-        <v>156</v>
-      </c>
       <c r="DC2" t="s">
+        <v>159</v>
+      </c>
+      <c r="DD2" t="s">
+        <v>205</v>
+      </c>
+      <c r="DE2" t="s">
         <v>155</v>
       </c>
-      <c r="DD2" t="s">
-        <v>155</v>
-      </c>
-      <c r="DE2" t="s">
-        <v>156</v>
-      </c>
       <c r="DF2" t="s">
-        <v>205</v>
+        <v>159</v>
       </c>
       <c r="DG2" t="s">
-        <v>206</v>
+        <v>159</v>
       </c>
       <c r="DH2" t="s">
         <v>155</v>
       </c>
       <c r="DI2" t="s">
+        <v>206</v>
+      </c>
+      <c r="DJ2" t="s">
+        <v>207</v>
+      </c>
+      <c r="DK2" t="s">
+        <v>159</v>
+      </c>
+      <c r="DL2" t="s">
+        <v>159</v>
+      </c>
+      <c r="DM2" t="s">
+        <v>159</v>
+      </c>
+      <c r="DN2" t="s">
+        <v>159</v>
+      </c>
+      <c r="DO2" t="s">
         <v>155</v>
       </c>
-      <c r="DJ2" t="s">
+      <c r="DP2" t="s">
+        <v>158</v>
+      </c>
+      <c r="DQ2" t="s">
         <v>155</v>
       </c>
-      <c r="DK2" t="s">
+      <c r="DR2" t="s">
+        <v>208</v>
+      </c>
+      <c r="DS2" t="s">
+        <v>208</v>
+      </c>
+      <c r="DT2" t="s">
+        <v>209</v>
+      </c>
+      <c r="DU2" t="s">
+        <v>210</v>
+      </c>
+      <c r="DV2" t="s">
         <v>155</v>
       </c>
-      <c r="DL2" t="s">
-        <v>156</v>
-      </c>
-      <c r="DM2" t="s">
-        <v>159</v>
-      </c>
-      <c r="DN2" t="s">
-        <v>156</v>
-      </c>
-      <c r="DO2" t="s">
-        <v>207</v>
-      </c>
-      <c r="DP2" t="s">
-        <v>207</v>
-      </c>
-      <c r="DQ2" t="s">
-        <v>208</v>
-      </c>
-      <c r="DR2" t="s">
-        <v>209</v>
-      </c>
-      <c r="DS2" t="s">
-        <v>156</v>
-      </c>
-      <c r="DT2" t="s">
-        <v>210</v>
-      </c>
-      <c r="DU2" t="s">
+      <c r="DW2" t="s">
         <v>211</v>
       </c>
-      <c r="DV2" t="s">
-        <v>156</v>
-      </c>
-      <c r="DW2" t="s">
+      <c r="DX2" t="s">
         <v>212</v>
       </c>
-      <c r="DX2" t="s">
+      <c r="DY2" t="s">
+        <v>155</v>
+      </c>
+      <c r="DZ2" t="s">
         <v>213</v>
       </c>
-      <c r="DY2" t="s">
+      <c r="EA2" t="s">
         <v>214</v>
       </c>
-      <c r="DZ2" t="s">
-        <v>156</v>
-      </c>
-      <c r="EA2" t="s">
+      <c r="EB2" t="s">
         <v>215</v>
       </c>
-      <c r="EB2" t="s">
-        <v>207</v>
-      </c>
       <c r="EC2" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="ED2" t="s">
         <v>216</v>
       </c>
       <c r="EE2" t="s">
-        <v>156</v>
+        <v>208</v>
       </c>
       <c r="EF2" t="s">
-        <v>216</v>
+        <v>158</v>
       </c>
       <c r="EG2" t="s">
         <v>217</v>
       </c>
       <c r="EH2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="EI2" t="s">
-        <v>186</v>
+        <v>217</v>
       </c>
       <c r="EJ2" t="s">
         <v>218</v>
       </c>
       <c r="EK2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="EL2" t="s">
+        <v>186</v>
+      </c>
+      <c r="EM2" t="s">
         <v>219</v>
       </c>
-      <c r="EM2" t="s">
+      <c r="EN2" t="s">
+        <v>155</v>
+      </c>
+      <c r="EO2" t="s">
         <v>220</v>
       </c>
-      <c r="EN2" t="s">
+      <c r="EP2" t="s">
         <v>221</v>
       </c>
-      <c r="EO2" t="s">
-        <v>156</v>
-      </c>
-      <c r="EP2" t="s">
+      <c r="EQ2" t="s">
         <v>222</v>
       </c>
-      <c r="EQ2" t="s">
+      <c r="ER2" t="s">
+        <v>155</v>
+      </c>
+      <c r="ES2" t="s">
         <v>223</v>
       </c>
-      <c r="ER2" t="s">
+      <c r="ET2" t="s">
         <v>224</v>
       </c>
-      <c r="ES2" t="s">
+      <c r="EU2" t="s">
         <v>225</v>
       </c>
-      <c r="ET2" t="s">
+      <c r="EV2" t="s">
         <v>226</v>
       </c>
-      <c r="EU2" t="s">
+      <c r="EW2" t="s">
         <v>227</v>
       </c>
-      <c r="EV2" t="s">
+      <c r="EX2" t="s">
         <v>228</v>
       </c>
-      <c r="EW2" t="s">
+      <c r="EY2" t="s">
+        <v>229</v>
+      </c>
+      <c r="EZ2" t="s">
         <v>186</v>
-      </c>
-      <c r="EX2" t="s">
-        <v>229</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="60">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2 S2 Y2 AA2:AG2 BK2 BO2:BR2 BU2:BY2 CZ2:DA2 DC2:DD2 DH2:DK2" xr:uid="{00000000-0002-0000-0000-000001000000}">
+  <dataValidations count="63">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2 V2 AB2 AD2:AJ2 BN2 BR2:BU2 BX2:CB2 DC2:DD2 DF2:DG2 DK2:DN2 L2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BT2 CE2 ES2 EV2 BJ2 BF2:BG2 AU2:BB2" xr:uid="{00000000-0002-0000-0000-000003000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2 K2 Q2:R2 BS2 CA2 CF2 CI2 CL2 CN2 CY2 DB2 DE2 DL2 DN2 DS2 DV2 DZ2 EE2 EH2 EK2 EO2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX2:BE2 BI2:BJ2 BM2 BW2 CH2 EV2 EY2" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2 T2:U2 BV2 CD2 CI2 CL2 CO2 CQ2 DB2 DE2 DH2 DO2 DQ2 DV2 DY2 EC2 EH2 EK2 EN2 ER2" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CE2" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Normal,Curiga gangguan pendengaran"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CU2" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Gangguan Pendengaran"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2" xr:uid="{00000000-0002-0000-0000-000014000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Normal (visus 6/6 - 6/12),Curiga gangguan penglihatan (visus &lt;6/12)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CW2" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"Normal (visus 6/6 - 6/12),Gangguan penglihatan ringan (visus &lt;6/12 - 6/18),Gangguan penglihatan sedang (&lt;6/18 - 6/60),Gangguan penglihatan berat (&lt;6/60 - 3/60),Buta (&lt;3/60)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CU2" xr:uid="{00000000-0002-0000-0000-000016000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CX2" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"Visus membaik,Visus tidak membaik (visus tetap)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CY2" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"Kelainan refraksi ringan (0.50 - 3.00 Dioptri),Kelainan refraksi sedang (3.00 - 6.00 Dioptri),Kelainan refraksi berat (&gt;6.00 Dioptri)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CW2" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CZ2" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CX2" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DA2" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"Curiga katarak,Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DF2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DI2" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DG2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DJ2" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DW2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DX2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EA2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DY2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EB2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EI2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EL2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EJ2" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EM2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EL2" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EO2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EM2" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EP2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EN2" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EQ2" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EP2" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ES2" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EQ2" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ET2" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ER2" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EU2" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ET2" xr:uid="{00000000-0002-0000-0000-000027000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EW2" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EU2" xr:uid="{00000000-0002-0000-0000-000028000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EX2" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EW2" xr:uid="{00000000-0002-0000-0000-000029000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EZ2" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Z2" xr:uid="{00000000-0002-0000-0000-00002A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AC2" xr:uid="{00000000-0002-0000-0000-000027000000}">
       <formula1>"Benar semua,Salah satu/Dua,Tidak Tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH2" xr:uid="{00000000-0002-0000-0000-00002B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2" xr:uid="{00000000-0002-0000-0000-000028000000}">
       <formula1>"Tidak terkendali/tak teratur (perlu pencahar),Kadang-kadang tak terkendali (1 x / minggu),Terkendali teratur"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2" xr:uid="{00000000-0002-0000-0000-00002C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"Tak terkendali atau pakai kateter,Kadang-kadang tak terkendali (hanya 1 x / 24 jam),Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2" xr:uid="{00000000-0002-0000-0000-00002D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM2" xr:uid="{00000000-0002-0000-0000-00002A000000}">
       <formula1>"Mandiri,Butuh pertolongan orang lain"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2" xr:uid="{00000000-0002-0000-0000-00002E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2" xr:uid="{00000000-0002-0000-0000-00002B000000}">
       <formula1>"Tergantung pertolongan orang lain,Perlu pertolongan pada beberapa kegiatan tetapi dapat mengerjakan sendiri beberapa kegiatan yang lain,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-00002F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2" xr:uid="{00000000-0002-0000-0000-00002C000000}">
       <formula1>"Tidak mampu,Perlu ditolong memotong makanan,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM2" xr:uid="{00000000-0002-0000-0000-000030000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AP2" xr:uid="{00000000-0002-0000-0000-00002D000000}">
       <formula1>"Tidak mampu,Perlu banyak bantuan untuk bias duduk (2 orang),Bantuan minimal 1 orang,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2" xr:uid="{00000000-0002-0000-0000-000031000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2" xr:uid="{00000000-0002-0000-0000-00002E000000}">
       <formula1>"Tidak mampu,Bisa (pindah) dengan kursi roda,Bantuan minimal 1 orang,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2" xr:uid="{00000000-0002-0000-0000-000032000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AR2" xr:uid="{00000000-0002-0000-0000-00002F000000}">
       <formula1>"Tergantung orang lain,Sebagian dibantu (misalnya: mengancing baju),Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AP2" xr:uid="{00000000-0002-0000-0000-000033000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AS2" xr:uid="{00000000-0002-0000-0000-000030000000}">
       <formula1>"Tidak mampu,Butuh pertolongan,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2" xr:uid="{00000000-0002-0000-0000-000034000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AT2" xr:uid="{00000000-0002-0000-0000-000031000000}">
       <formula1>"Tergantung orang lain,Mandiri"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AR2" xr:uid="{00000000-0002-0000-0000-000035000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2" xr:uid="{00000000-0002-0000-0000-000032000000}">
       <formula1>"SUDAH DITANYAKAN"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AS2" xr:uid="{00000000-0002-0000-0000-000036000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2" xr:uid="{00000000-0002-0000-0000-000033000000}">
       <formula1>"Benar,Salah"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AT2" xr:uid="{00000000-0002-0000-0000-000037000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW2" xr:uid="{00000000-0002-0000-0000-000034000000}">
       <formula1>"Benar 1 kata,Benar 2 Kata,Benar semua kata,Tidak dapat mengingat/mengulang kata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BC2:BD2" xr:uid="{00000000-0002-0000-0000-00003A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BF2:BG2" xr:uid="{00000000-0002-0000-0000-000035000000}">
       <formula1>"Bertahan 10 detik,Tidak bertahan 10 detik,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2" xr:uid="{00000000-0002-0000-0000-00003B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH2" xr:uid="{00000000-0002-0000-0000-000036000000}">
       <formula1>"Bertahan 10 detik,Bertahan 3 - 9.99 detik,Bertahan &lt; 3 detik"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH2" xr:uid="{00000000-0002-0000-0000-00003E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK2" xr:uid="{00000000-0002-0000-0000-000037000000}">
       <formula1>"Nafsu Makan Yang Sangat Berkurang,Nafsu Makan Sedikit Berkurang,Nafsu Makan Biasa saja"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2" xr:uid="{00000000-0002-0000-0000-00003F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2" xr:uid="{00000000-0002-0000-0000-000038000000}">
       <formula1>"Penurunan BB &gt; 3 Kg,Tidak Tahu,Penurunan BB antara 1 - 3 Kg"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2" xr:uid="{00000000-0002-0000-0000-000041000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2" xr:uid="{00000000-0002-0000-0000-000039000000}">
       <formula1>"Dementia atau depresi berat,Demensia/kepikunan ringan,Tidak ada masalah psikologis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BM2" xr:uid="{00000000-0002-0000-0000-000042000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2" xr:uid="{00000000-0002-0000-0000-00003A000000}">
       <formula1>"IMT &lt;19,IMT 19 - &lt;21,IMT 21 - &lt;23,IMT &gt;= 23"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BN2" xr:uid="{00000000-0002-0000-0000-000043000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ2" xr:uid="{00000000-0002-0000-0000-00003B000000}">
       <formula1>"&lt;31 cm,&gt;= 31 cm"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{0739CCB7-0531-A140-9A86-D8E33CA4DE7A}">
+      <formula1>"Berdiri,Telentang"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2" xr:uid="{CFE5A940-B719-944C-A4F2-7D7AAD4869A6}">
+      <formula1>"Makrosefali,Normal,Mikrosefali"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2" xr:uid="{418FF0C6-4714-6B4F-B204-3DD4B6B23A44}">
+      <formula1>"Perkembangan sesuai usia,Perkembangan meragukan,Perkembangan curiga adanya penyimpangan"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
wip risiko tb anak
</commit_message>
<xml_diff>
--- a/dataset/anak.xlsx
+++ b/dataset/anak.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{941C8527-990D-0643-8DAE-55A5031FBC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF1CE0CC-D728-4547-82FF-E9D24A2E1323}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4480" yWindow="-21000" windowWidth="36000" windowHeight="19540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,67 +25,7 @@
     <author>Microsoft Office User</author>
   </authors>
   <commentList>
-    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Microsoft Office User:
-wajib diisi apabila pernah_diabetes Ya</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">Microsoft Office User:
-wajib diisi apabila pernah_diabetes Ya </t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Microsoft Office User:
-wajib diisi apabila pernah_diabetes Tidak</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="W1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="12"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>Microsoft Office User:
-wajib diisi apabila pernah_hipertensi Ya</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="CC1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="T1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
       <text>
         <r>
           <rPr>
@@ -100,7 +40,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CF1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="W1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -115,7 +55,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="AB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -130,7 +70,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="AE1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -145,7 +85,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="AL1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -160,7 +100,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CW1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="AN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -175,7 +115,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CX1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="AO1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -190,7 +130,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
+    <comment ref="AP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
       <text>
         <r>
           <rPr>
@@ -205,7 +145,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CZ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
+    <comment ref="AQ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
       <text>
         <r>
           <rPr>
@@ -220,7 +160,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="DJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
+    <comment ref="BA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
       <text>
         <r>
           <rPr>
@@ -235,7 +175,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="EB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
+    <comment ref="BS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
       <text>
         <r>
           <rPr>
@@ -255,7 +195,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="152">
   <si>
     <t>batas_awal</t>
   </si>
@@ -278,189 +218,6 @@
     <t>tinggi_badan</t>
   </si>
   <si>
-    <t>periksa_gula_darah</t>
-  </si>
-  <si>
-    <t>pernah_diabetes</t>
-  </si>
-  <si>
-    <t>total_bulan_diabetes</t>
-  </si>
-  <si>
-    <t>gula_darah_sewaktu</t>
-  </si>
-  <si>
-    <t>gula_darah_sewaktu_2</t>
-  </si>
-  <si>
-    <t>gula_darah_puasa</t>
-  </si>
-  <si>
-    <t>gula_darah_pp</t>
-  </si>
-  <si>
-    <t>periksa_tensi</t>
-  </si>
-  <si>
-    <t>pernah_hipertensi</t>
-  </si>
-  <si>
-    <t>total_bulan_hipertensi</t>
-  </si>
-  <si>
-    <t>sistolik</t>
-  </si>
-  <si>
-    <t>diastolik</t>
-  </si>
-  <si>
-    <t>sistolik_2</t>
-  </si>
-  <si>
-    <t>diastolik_2</t>
-  </si>
-  <si>
-    <t>mengingat_3_kata</t>
-  </si>
-  <si>
-    <t>tanggal_berapa_dimana</t>
-  </si>
-  <si>
-    <t>ulangi_3_kata_sebelumnya</t>
-  </si>
-  <si>
-    <t>berdiri_di_kursi</t>
-  </si>
-  <si>
-    <t>berat_badan_berkurang</t>
-  </si>
-  <si>
-    <t>hilang_nafsu_makan</t>
-  </si>
-  <si>
-    <t>lila_kurang_21cm</t>
-  </si>
-  <si>
-    <t>2_minggu_terakhir_sedih</t>
-  </si>
-  <si>
-    <t>2_minggu_sedikit_minat</t>
-  </si>
-  <si>
-    <t>kendali_bab</t>
-  </si>
-  <si>
-    <t>kendali_bak</t>
-  </si>
-  <si>
-    <t>membersihkan_diri</t>
-  </si>
-  <si>
-    <t>penggunaan_jamban</t>
-  </si>
-  <si>
-    <t>makan_minum</t>
-  </si>
-  <si>
-    <t>berubah_sikap</t>
-  </si>
-  <si>
-    <t>berpindah</t>
-  </si>
-  <si>
-    <t>memakai_baju</t>
-  </si>
-  <si>
-    <t>naik_turun_tangga</t>
-  </si>
-  <si>
-    <t>mandi</t>
-  </si>
-  <si>
-    <t>mini_cog_1</t>
-  </si>
-  <si>
-    <t>mini_cog_2</t>
-  </si>
-  <si>
-    <t>mini_cog_3</t>
-  </si>
-  <si>
-    <t>ina_1</t>
-  </si>
-  <si>
-    <t>ina_2</t>
-  </si>
-  <si>
-    <t>ina_3</t>
-  </si>
-  <si>
-    <t>ina_4</t>
-  </si>
-  <si>
-    <t>ina_5</t>
-  </si>
-  <si>
-    <t>ina_6</t>
-  </si>
-  <si>
-    <t>ina_7</t>
-  </si>
-  <si>
-    <t>ina_8</t>
-  </si>
-  <si>
-    <t>sppb_1</t>
-  </si>
-  <si>
-    <t>sppb_2</t>
-  </si>
-  <si>
-    <t>sppb_3</t>
-  </si>
-  <si>
-    <t>sppb_4</t>
-  </si>
-  <si>
-    <t>sppb_5</t>
-  </si>
-  <si>
-    <t>mna_sf_1</t>
-  </si>
-  <si>
-    <t>mna_sf_2</t>
-  </si>
-  <si>
-    <t>mna_sf_3</t>
-  </si>
-  <si>
-    <t>mna_sf_4</t>
-  </si>
-  <si>
-    <t>mna_sf_5</t>
-  </si>
-  <si>
-    <t>mna_sf_6</t>
-  </si>
-  <si>
-    <t>mna_sf_7</t>
-  </si>
-  <si>
-    <t>depresi_lanjutan_1</t>
-  </si>
-  <si>
-    <t>depresi_lanjutan_2</t>
-  </si>
-  <si>
-    <t>depresi_lanjutan_3</t>
-  </si>
-  <si>
-    <t>depresi_lanjutan_4</t>
-  </si>
-  <si>
-    <t>periksa_risiko_tbc</t>
-  </si>
-  <si>
     <t>pernah_batuk_tidak_sembuh</t>
   </si>
   <si>
@@ -470,9 +227,6 @@
     <t>demam_hilang_timbul</t>
   </si>
   <si>
-    <t>berkeringat_malam</t>
-  </si>
-  <si>
     <t>pembesaran_getah_bening</t>
   </si>
   <si>
@@ -737,81 +491,6 @@
     <t>Ya</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>110</t>
-  </si>
-  <si>
-    <t>120</t>
-  </si>
-  <si>
-    <t>Benar semua</t>
-  </si>
-  <si>
-    <t>Tidak terkendali/tak teratur (perlu pencahar)</t>
-  </si>
-  <si>
-    <t>Kadang-kadang tak terkendali (hanya 1 x / 24 jam)</t>
-  </si>
-  <si>
-    <t>Mandiri</t>
-  </si>
-  <si>
-    <t>Bisa (pindah) dengan kursi roda</t>
-  </si>
-  <si>
-    <t>Sebagian dibantu (misalnya: mengancing baju)</t>
-  </si>
-  <si>
-    <t>Butuh pertolongan</t>
-  </si>
-  <si>
-    <t>SUDAH DITANYAKAN</t>
-  </si>
-  <si>
-    <t>Benar</t>
-  </si>
-  <si>
-    <t>Benar semua kata</t>
-  </si>
-  <si>
-    <t>Tidak, Berubah</t>
-  </si>
-  <si>
-    <t>Tidak Berubah</t>
-  </si>
-  <si>
-    <t>Tidak Tahu</t>
-  </si>
-  <si>
-    <t>Bertahan 10 detik</t>
-  </si>
-  <si>
-    <t>4.83 - 6.20 detik</t>
-  </si>
-  <si>
-    <t>&lt;11.19 detik</t>
-  </si>
-  <si>
-    <t>Nafsu Makan Yang Sangat Berkurang</t>
-  </si>
-  <si>
-    <t>Penurunan BB &gt; 3 Kg</t>
-  </si>
-  <si>
-    <t>Harus berbaring di tempat tidur atau menggunakan kursi roda</t>
-  </si>
-  <si>
-    <t>Dementia atau depresi berat</t>
-  </si>
-  <si>
-    <t>IMT &lt;19</t>
-  </si>
-  <si>
-    <t>&lt;31 cm</t>
-  </si>
-  <si>
     <t>Tidak batuk</t>
   </si>
   <si>
@@ -969,6 +648,9 @@
   </si>
   <si>
     <t>m_chat_2</t>
+  </si>
+  <si>
+    <t>lesu</t>
   </si>
 </sst>
 </file>
@@ -1371,7 +1053,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:FA2"/>
+  <dimension ref="A1:CR2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -1384,117 +1066,80 @@
     <col min="9" max="9" width="16.5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19" bestFit="1" customWidth="1"/>
     <col min="11" max="13" width="19" customWidth="1"/>
-    <col min="14" max="14" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="17.1640625" customWidth="1"/>
-    <col min="21" max="21" width="12" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="8" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.83203125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="16" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="21" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="18" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="21.83203125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="21.1640625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="11" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="42.1640625" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="41" max="42" width="18.1640625" customWidth="1"/>
-    <col min="43" max="43" width="27.1640625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="40" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="16" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="16" customWidth="1"/>
-    <col min="47" max="47" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="50" max="53" width="15.83203125" customWidth="1"/>
-    <col min="54" max="73" width="10.5" customWidth="1"/>
-    <col min="74" max="74" width="16" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="25" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="14.83203125" customWidth="1"/>
-    <col min="82" max="82" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="22.83203125" customWidth="1"/>
-    <col min="87" max="87" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="16.1640625" customWidth="1"/>
-    <col min="89" max="89" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="91" max="92" width="12.33203125" customWidth="1"/>
-    <col min="93" max="93" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="14.1640625" customWidth="1"/>
-    <col min="95" max="95" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="23.6640625" customWidth="1"/>
-    <col min="98" max="98" width="26" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="26" customWidth="1"/>
-    <col min="100" max="100" width="36.1640625" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="41.5" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="29" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="105" max="106" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="107" max="108" width="12.83203125" customWidth="1"/>
-    <col min="109" max="109" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="17.5" customWidth="1"/>
-    <col min="112" max="112" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="113" max="113" width="13" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="115" max="115" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="116" max="118" width="19.5" customWidth="1"/>
-    <col min="119" max="119" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="9.83203125" customWidth="1"/>
-    <col min="121" max="121" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="122" max="125" width="11.5" customWidth="1"/>
-    <col min="126" max="126" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="9" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="130" max="130" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="131" max="131" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="132" max="132" width="18.1640625" customWidth="1"/>
-    <col min="133" max="133" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="134" max="134" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="135" max="137" width="8.33203125" customWidth="1"/>
-    <col min="138" max="138" width="22" bestFit="1" customWidth="1"/>
-    <col min="139" max="139" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="140" max="140" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="141" max="141" width="14" bestFit="1" customWidth="1"/>
-    <col min="142" max="142" width="14" customWidth="1"/>
-    <col min="143" max="143" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="144" max="144" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="145" max="145" width="18.1640625" customWidth="1"/>
-    <col min="146" max="146" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="147" max="147" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="148" max="148" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="149" max="151" width="18.1640625" customWidth="1"/>
-    <col min="152" max="152" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="153" max="153" width="35" bestFit="1" customWidth="1"/>
-    <col min="154" max="154" width="43.1640625" bestFit="1" customWidth="1"/>
-    <col min="155" max="155" width="18.1640625" customWidth="1"/>
-    <col min="156" max="156" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="157" max="157" width="10.83203125" customWidth="1"/>
+    <col min="14" max="14" width="25" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.83203125" customWidth="1"/>
+    <col min="21" max="21" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="22.83203125" customWidth="1"/>
+    <col min="26" max="26" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="16.1640625" customWidth="1"/>
+    <col min="28" max="28" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="30" max="31" width="12.33203125" customWidth="1"/>
+    <col min="32" max="32" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.1640625" customWidth="1"/>
+    <col min="34" max="34" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="23.6640625" customWidth="1"/>
+    <col min="37" max="37" width="26" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="26" customWidth="1"/>
+    <col min="39" max="39" width="36.1640625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="41.5" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="29" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="44" max="45" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="46" max="47" width="12.83203125" customWidth="1"/>
+    <col min="48" max="48" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="17.5" customWidth="1"/>
+    <col min="51" max="51" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="13" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="55" max="57" width="19.5" customWidth="1"/>
+    <col min="58" max="58" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="9.83203125" customWidth="1"/>
+    <col min="60" max="60" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="61" max="64" width="11.5" customWidth="1"/>
+    <col min="65" max="65" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="9" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="18.1640625" customWidth="1"/>
+    <col min="72" max="72" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="74" max="76" width="8.33203125" customWidth="1"/>
+    <col min="77" max="77" width="22" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="14" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="14" customWidth="1"/>
+    <col min="82" max="82" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="18.1640625" customWidth="1"/>
+    <col min="85" max="85" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="88" max="90" width="18.1640625" customWidth="1"/>
+    <col min="91" max="91" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="35" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="18.1640625" customWidth="1"/>
+    <col min="95" max="95" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:157" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1517,19 +1162,19 @@
         <v>6</v>
       </c>
       <c r="I1" t="s">
-        <v>230</v>
+        <v>143</v>
       </c>
       <c r="J1" t="s">
-        <v>232</v>
+        <v>145</v>
       </c>
       <c r="K1" t="s">
-        <v>234</v>
+        <v>147</v>
       </c>
       <c r="L1" t="s">
-        <v>236</v>
+        <v>149</v>
       </c>
       <c r="M1" t="s">
-        <v>237</v>
+        <v>150</v>
       </c>
       <c r="N1" t="s">
         <v>7</v>
@@ -1541,1060 +1186,643 @@
         <v>9</v>
       </c>
       <c r="Q1" t="s">
+        <v>151</v>
+      </c>
+      <c r="R1" t="s">
         <v>10</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>11</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>12</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>13</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>14</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>15</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>16</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>17</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>18</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>19</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>20</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>21</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>22</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>23</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>24</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>25</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>26</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>27</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
         <v>28</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AK1" t="s">
         <v>29</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AL1" t="s">
         <v>30</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AM1" t="s">
         <v>31</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AN1" t="s">
         <v>32</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AO1" t="s">
         <v>33</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AP1" t="s">
         <v>34</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AQ1" t="s">
         <v>35</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AR1" t="s">
         <v>36</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AS1" t="s">
         <v>37</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AT1" t="s">
         <v>38</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AU1" t="s">
         <v>39</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AV1" t="s">
         <v>40</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AW1" t="s">
         <v>41</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AX1" t="s">
         <v>42</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AY1" t="s">
         <v>43</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AZ1" t="s">
         <v>44</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BA1" t="s">
         <v>45</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BB1" t="s">
         <v>46</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BC1" t="s">
         <v>47</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BD1" t="s">
         <v>48</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BE1" t="s">
         <v>49</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BF1" t="s">
         <v>50</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BG1" t="s">
         <v>51</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BH1" t="s">
         <v>52</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BI1" t="s">
         <v>53</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BJ1" t="s">
         <v>54</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BK1" t="s">
         <v>55</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BL1" t="s">
         <v>56</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BM1" t="s">
         <v>57</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BN1" t="s">
         <v>58</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BO1" t="s">
         <v>59</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BP1" t="s">
         <v>60</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BQ1" t="s">
         <v>61</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BR1" t="s">
         <v>62</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BS1" t="s">
         <v>63</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BT1" t="s">
         <v>64</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BU1" t="s">
         <v>65</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BV1" t="s">
         <v>66</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="BW1" t="s">
         <v>67</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="BX1" t="s">
         <v>68</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="BY1" t="s">
         <v>69</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="BZ1" t="s">
         <v>70</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CA1" t="s">
         <v>71</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CB1" t="s">
         <v>72</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CC1" t="s">
         <v>73</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CD1" t="s">
         <v>74</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CE1" t="s">
         <v>75</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CF1" t="s">
         <v>76</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CG1" t="s">
         <v>77</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CH1" t="s">
         <v>78</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CI1" t="s">
         <v>79</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CJ1" t="s">
         <v>80</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CK1" t="s">
         <v>81</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CL1" t="s">
         <v>82</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CM1" t="s">
         <v>83</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CN1" t="s">
         <v>84</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CO1" t="s">
         <v>85</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CP1" t="s">
         <v>86</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="CQ1" t="s">
         <v>87</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="CR1" t="s">
         <v>88</v>
       </c>
-      <c r="CR1" t="s">
+    </row>
+    <row r="2" spans="1:96" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="CS1" t="s">
+      <c r="B2" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="C2" t="s">
         <v>91</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="E2" t="s">
         <v>92</v>
       </c>
-      <c r="CV1" t="s">
-        <v>93</v>
-      </c>
-      <c r="CW1" t="s">
+      <c r="G2" t="s">
         <v>94</v>
       </c>
-      <c r="CX1" t="s">
+      <c r="H2" t="s">
         <v>95</v>
       </c>
-      <c r="CY1" t="s">
-        <v>96</v>
-      </c>
-      <c r="CZ1" t="s">
+      <c r="I2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J2" t="s">
+        <v>146</v>
+      </c>
+      <c r="K2" t="s">
+        <v>148</v>
+      </c>
+      <c r="L2" t="s">
         <v>97</v>
-      </c>
-      <c r="DA1" t="s">
-        <v>98</v>
-      </c>
-      <c r="DB1" t="s">
-        <v>99</v>
-      </c>
-      <c r="DC1" t="s">
-        <v>100</v>
-      </c>
-      <c r="DD1" t="s">
-        <v>101</v>
-      </c>
-      <c r="DE1" t="s">
-        <v>102</v>
-      </c>
-      <c r="DF1" t="s">
-        <v>103</v>
-      </c>
-      <c r="DG1" t="s">
-        <v>104</v>
-      </c>
-      <c r="DH1" t="s">
-        <v>105</v>
-      </c>
-      <c r="DI1" t="s">
-        <v>106</v>
-      </c>
-      <c r="DJ1" t="s">
-        <v>107</v>
-      </c>
-      <c r="DK1" t="s">
-        <v>108</v>
-      </c>
-      <c r="DL1" t="s">
-        <v>109</v>
-      </c>
-      <c r="DM1" t="s">
-        <v>110</v>
-      </c>
-      <c r="DN1" t="s">
-        <v>111</v>
-      </c>
-      <c r="DO1" t="s">
-        <v>112</v>
-      </c>
-      <c r="DP1" t="s">
-        <v>113</v>
-      </c>
-      <c r="DQ1" t="s">
-        <v>114</v>
-      </c>
-      <c r="DR1" t="s">
-        <v>115</v>
-      </c>
-      <c r="DS1" t="s">
-        <v>116</v>
-      </c>
-      <c r="DT1" t="s">
-        <v>117</v>
-      </c>
-      <c r="DU1" t="s">
-        <v>118</v>
-      </c>
-      <c r="DV1" t="s">
-        <v>119</v>
-      </c>
-      <c r="DW1" t="s">
-        <v>120</v>
-      </c>
-      <c r="DX1" t="s">
-        <v>121</v>
-      </c>
-      <c r="DY1" t="s">
-        <v>122</v>
-      </c>
-      <c r="DZ1" t="s">
-        <v>123</v>
-      </c>
-      <c r="EA1" t="s">
-        <v>124</v>
-      </c>
-      <c r="EB1" t="s">
-        <v>125</v>
-      </c>
-      <c r="EC1" t="s">
-        <v>126</v>
-      </c>
-      <c r="ED1" t="s">
-        <v>127</v>
-      </c>
-      <c r="EE1" t="s">
-        <v>128</v>
-      </c>
-      <c r="EF1" t="s">
-        <v>129</v>
-      </c>
-      <c r="EG1" t="s">
-        <v>130</v>
-      </c>
-      <c r="EH1" t="s">
-        <v>131</v>
-      </c>
-      <c r="EI1" t="s">
-        <v>132</v>
-      </c>
-      <c r="EJ1" t="s">
-        <v>133</v>
-      </c>
-      <c r="EK1" t="s">
-        <v>134</v>
-      </c>
-      <c r="EL1" t="s">
-        <v>135</v>
-      </c>
-      <c r="EM1" t="s">
-        <v>136</v>
-      </c>
-      <c r="EN1" t="s">
-        <v>137</v>
-      </c>
-      <c r="EO1" t="s">
-        <v>138</v>
-      </c>
-      <c r="EP1" t="s">
-        <v>139</v>
-      </c>
-      <c r="EQ1" t="s">
-        <v>140</v>
-      </c>
-      <c r="ER1" t="s">
-        <v>141</v>
-      </c>
-      <c r="ES1" t="s">
-        <v>142</v>
-      </c>
-      <c r="ET1" t="s">
-        <v>143</v>
-      </c>
-      <c r="EU1" t="s">
-        <v>144</v>
-      </c>
-      <c r="EV1" t="s">
-        <v>145</v>
-      </c>
-      <c r="EW1" t="s">
-        <v>146</v>
-      </c>
-      <c r="EX1" t="s">
-        <v>147</v>
-      </c>
-      <c r="EY1" t="s">
-        <v>148</v>
-      </c>
-      <c r="EZ1" t="s">
-        <v>149</v>
-      </c>
-      <c r="FA1" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="2" spans="1:157" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C2" t="s">
-        <v>153</v>
-      </c>
-      <c r="E2" t="s">
-        <v>154</v>
-      </c>
-      <c r="G2" t="s">
-        <v>156</v>
-      </c>
-      <c r="H2" t="s">
-        <v>157</v>
-      </c>
-      <c r="I2" t="s">
-        <v>231</v>
-      </c>
-      <c r="J2" t="s">
-        <v>233</v>
-      </c>
-      <c r="K2" t="s">
-        <v>235</v>
-      </c>
-      <c r="L2" t="s">
-        <v>159</v>
       </c>
       <c r="M2">
         <v>10</v>
       </c>
       <c r="N2" t="s">
-        <v>155</v>
+        <v>98</v>
       </c>
       <c r="O2" t="s">
-        <v>159</v>
+        <v>97</v>
       </c>
       <c r="P2" t="s">
-        <v>160</v>
+        <v>97</v>
       </c>
       <c r="Q2" t="s">
-        <v>161</v>
+        <v>97</v>
+      </c>
+      <c r="R2" t="s">
+        <v>97</v>
       </c>
       <c r="S2" t="s">
-        <v>158</v>
+        <v>97</v>
+      </c>
+      <c r="T2" t="s">
+        <v>99</v>
       </c>
       <c r="U2" t="s">
-        <v>155</v>
+        <v>93</v>
       </c>
       <c r="V2" t="s">
-        <v>159</v>
+        <v>100</v>
       </c>
       <c r="W2" t="s">
-        <v>160</v>
+        <v>101</v>
       </c>
       <c r="X2" t="s">
-        <v>162</v>
+        <v>102</v>
       </c>
       <c r="Y2" t="s">
-        <v>156</v>
+        <v>103</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>93</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>104</v>
       </c>
       <c r="AB2" t="s">
-        <v>159</v>
+        <v>105</v>
       </c>
       <c r="AC2" t="s">
-        <v>163</v>
+        <v>93</v>
       </c>
       <c r="AD2" t="s">
-        <v>159</v>
+        <v>106</v>
       </c>
       <c r="AE2" t="s">
-        <v>159</v>
+        <v>107</v>
       </c>
       <c r="AF2" t="s">
-        <v>159</v>
+        <v>93</v>
       </c>
       <c r="AG2" t="s">
-        <v>159</v>
+        <v>108</v>
       </c>
       <c r="AH2" t="s">
-        <v>159</v>
+        <v>93</v>
       </c>
       <c r="AI2" t="s">
-        <v>159</v>
+        <v>109</v>
       </c>
       <c r="AJ2" t="s">
-        <v>159</v>
+        <v>110</v>
       </c>
       <c r="AK2" t="s">
-        <v>164</v>
+        <v>111</v>
       </c>
       <c r="AL2" t="s">
-        <v>165</v>
+        <v>112</v>
       </c>
       <c r="AM2" t="s">
-        <v>166</v>
+        <v>113</v>
       </c>
       <c r="AN2" t="s">
-        <v>166</v>
+        <v>114</v>
       </c>
       <c r="AO2" t="s">
-        <v>166</v>
+        <v>115</v>
       </c>
       <c r="AP2" t="s">
-        <v>166</v>
+        <v>116</v>
       </c>
       <c r="AQ2" t="s">
-        <v>167</v>
+        <v>99</v>
       </c>
       <c r="AR2" t="s">
-        <v>168</v>
+        <v>117</v>
       </c>
       <c r="AS2" t="s">
-        <v>169</v>
+        <v>93</v>
       </c>
       <c r="AT2" t="s">
-        <v>166</v>
+        <v>97</v>
       </c>
       <c r="AU2" t="s">
-        <v>170</v>
+        <v>118</v>
       </c>
       <c r="AV2" t="s">
-        <v>171</v>
+        <v>93</v>
       </c>
       <c r="AW2" t="s">
-        <v>172</v>
+        <v>97</v>
       </c>
       <c r="AX2" t="s">
-        <v>173</v>
+        <v>97</v>
       </c>
       <c r="AY2" t="s">
-        <v>174</v>
+        <v>93</v>
       </c>
       <c r="AZ2" t="s">
-        <v>174</v>
+        <v>119</v>
       </c>
       <c r="BA2" t="s">
-        <v>175</v>
+        <v>120</v>
       </c>
       <c r="BB2" t="s">
-        <v>175</v>
+        <v>97</v>
       </c>
       <c r="BC2" t="s">
-        <v>175</v>
+        <v>97</v>
       </c>
       <c r="BD2" t="s">
-        <v>175</v>
+        <v>97</v>
       </c>
       <c r="BE2" t="s">
-        <v>175</v>
+        <v>97</v>
       </c>
       <c r="BF2" t="s">
-        <v>176</v>
+        <v>93</v>
       </c>
       <c r="BG2" t="s">
-        <v>176</v>
+        <v>96</v>
       </c>
       <c r="BH2" t="s">
-        <v>176</v>
+        <v>93</v>
       </c>
       <c r="BI2" t="s">
-        <v>177</v>
+        <v>121</v>
       </c>
       <c r="BJ2" t="s">
-        <v>178</v>
+        <v>121</v>
       </c>
       <c r="BK2" t="s">
-        <v>179</v>
+        <v>122</v>
       </c>
       <c r="BL2" t="s">
-        <v>180</v>
+        <v>123</v>
       </c>
       <c r="BM2" t="s">
-        <v>181</v>
+        <v>93</v>
       </c>
       <c r="BN2" t="s">
-        <v>159</v>
+        <v>124</v>
       </c>
       <c r="BO2" t="s">
-        <v>182</v>
+        <v>125</v>
       </c>
       <c r="BP2" t="s">
-        <v>183</v>
+        <v>93</v>
       </c>
       <c r="BQ2" t="s">
-        <v>184</v>
+        <v>126</v>
       </c>
       <c r="BR2" t="s">
-        <v>159</v>
+        <v>127</v>
       </c>
       <c r="BS2" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="BT2" t="s">
-        <v>159</v>
+        <v>93</v>
       </c>
       <c r="BU2" t="s">
-        <v>159</v>
+        <v>129</v>
       </c>
       <c r="BV2" t="s">
-        <v>155</v>
+        <v>121</v>
       </c>
       <c r="BW2" t="s">
-        <v>185</v>
+        <v>96</v>
       </c>
       <c r="BX2" t="s">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="BY2" t="s">
-        <v>159</v>
+        <v>93</v>
       </c>
       <c r="BZ2" t="s">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="CA2" t="s">
-        <v>159</v>
+        <v>131</v>
       </c>
       <c r="CB2" t="s">
-        <v>159</v>
+        <v>93</v>
       </c>
       <c r="CC2" t="s">
-        <v>186</v>
+        <v>99</v>
       </c>
       <c r="CD2" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="CE2" t="s">
-        <v>187</v>
+        <v>93</v>
       </c>
       <c r="CF2" t="s">
-        <v>188</v>
+        <v>133</v>
       </c>
       <c r="CG2" t="s">
-        <v>189</v>
+        <v>134</v>
       </c>
       <c r="CH2" t="s">
-        <v>190</v>
+        <v>135</v>
       </c>
       <c r="CI2" t="s">
-        <v>155</v>
+        <v>93</v>
       </c>
       <c r="CJ2" t="s">
-        <v>191</v>
+        <v>136</v>
       </c>
       <c r="CK2" t="s">
-        <v>192</v>
+        <v>137</v>
       </c>
       <c r="CL2" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="CM2" t="s">
-        <v>193</v>
+        <v>139</v>
       </c>
       <c r="CN2" t="s">
-        <v>194</v>
+        <v>140</v>
       </c>
       <c r="CO2" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="CP2" t="s">
-        <v>195</v>
+        <v>142</v>
       </c>
       <c r="CQ2" t="s">
-        <v>155</v>
-      </c>
-      <c r="CR2" t="s">
-        <v>196</v>
-      </c>
-      <c r="CS2" t="s">
-        <v>197</v>
-      </c>
-      <c r="CT2" t="s">
-        <v>198</v>
-      </c>
-      <c r="CU2" t="s">
-        <v>199</v>
-      </c>
-      <c r="CV2" t="s">
-        <v>200</v>
-      </c>
-      <c r="CW2" t="s">
-        <v>201</v>
-      </c>
-      <c r="CX2" t="s">
-        <v>202</v>
-      </c>
-      <c r="CY2" t="s">
-        <v>203</v>
-      </c>
-      <c r="CZ2" t="s">
-        <v>186</v>
-      </c>
-      <c r="DA2" t="s">
-        <v>204</v>
-      </c>
-      <c r="DB2" t="s">
-        <v>155</v>
-      </c>
-      <c r="DC2" t="s">
-        <v>159</v>
-      </c>
-      <c r="DD2" t="s">
-        <v>205</v>
-      </c>
-      <c r="DE2" t="s">
-        <v>155</v>
-      </c>
-      <c r="DF2" t="s">
-        <v>159</v>
-      </c>
-      <c r="DG2" t="s">
-        <v>159</v>
-      </c>
-      <c r="DH2" t="s">
-        <v>155</v>
-      </c>
-      <c r="DI2" t="s">
-        <v>206</v>
-      </c>
-      <c r="DJ2" t="s">
-        <v>207</v>
-      </c>
-      <c r="DK2" t="s">
-        <v>159</v>
-      </c>
-      <c r="DL2" t="s">
-        <v>159</v>
-      </c>
-      <c r="DM2" t="s">
-        <v>159</v>
-      </c>
-      <c r="DN2" t="s">
-        <v>159</v>
-      </c>
-      <c r="DO2" t="s">
-        <v>155</v>
-      </c>
-      <c r="DP2" t="s">
-        <v>158</v>
-      </c>
-      <c r="DQ2" t="s">
-        <v>155</v>
-      </c>
-      <c r="DR2" t="s">
-        <v>208</v>
-      </c>
-      <c r="DS2" t="s">
-        <v>208</v>
-      </c>
-      <c r="DT2" t="s">
-        <v>209</v>
-      </c>
-      <c r="DU2" t="s">
-        <v>210</v>
-      </c>
-      <c r="DV2" t="s">
-        <v>155</v>
-      </c>
-      <c r="DW2" t="s">
-        <v>211</v>
-      </c>
-      <c r="DX2" t="s">
-        <v>212</v>
-      </c>
-      <c r="DY2" t="s">
-        <v>155</v>
-      </c>
-      <c r="DZ2" t="s">
-        <v>213</v>
-      </c>
-      <c r="EA2" t="s">
-        <v>214</v>
-      </c>
-      <c r="EB2" t="s">
-        <v>215</v>
-      </c>
-      <c r="EC2" t="s">
-        <v>155</v>
-      </c>
-      <c r="ED2" t="s">
-        <v>216</v>
-      </c>
-      <c r="EE2" t="s">
-        <v>208</v>
-      </c>
-      <c r="EF2" t="s">
-        <v>158</v>
-      </c>
-      <c r="EG2" t="s">
-        <v>217</v>
-      </c>
-      <c r="EH2" t="s">
-        <v>155</v>
-      </c>
-      <c r="EI2" t="s">
-        <v>217</v>
-      </c>
-      <c r="EJ2" t="s">
-        <v>218</v>
-      </c>
-      <c r="EK2" t="s">
-        <v>155</v>
-      </c>
-      <c r="EL2" t="s">
-        <v>186</v>
-      </c>
-      <c r="EM2" t="s">
-        <v>219</v>
-      </c>
-      <c r="EN2" t="s">
-        <v>155</v>
-      </c>
-      <c r="EO2" t="s">
-        <v>220</v>
-      </c>
-      <c r="EP2" t="s">
-        <v>221</v>
-      </c>
-      <c r="EQ2" t="s">
-        <v>222</v>
-      </c>
-      <c r="ER2" t="s">
-        <v>155</v>
-      </c>
-      <c r="ES2" t="s">
-        <v>223</v>
-      </c>
-      <c r="ET2" t="s">
-        <v>224</v>
-      </c>
-      <c r="EU2" t="s">
-        <v>225</v>
-      </c>
-      <c r="EV2" t="s">
-        <v>226</v>
-      </c>
-      <c r="EW2" t="s">
-        <v>227</v>
-      </c>
-      <c r="EX2" t="s">
-        <v>228</v>
-      </c>
-      <c r="EY2" t="s">
-        <v>229</v>
-      </c>
-      <c r="EZ2" t="s">
-        <v>186</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="63">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2 V2 AB2 AD2:AJ2 BN2 BR2:BU2 BX2:CB2 DC2:DD2 DF2:DG2 DK2:DN2 L2" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="42">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:S2 AT2:AU2 AW2:AX2 BB2:BE2 L2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX2:BE2 BI2:BJ2 BM2 BW2 CH2 EV2 EY2" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2 T2:U2 BV2 CD2 CI2 CL2 CO2 CQ2 DB2 DE2 DH2 DO2 DQ2 DV2 DY2 EC2 EH2 EK2 EN2 ER2" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2 Y2 CM2 CP2" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2 Z2 AC2 AF2 AH2 AS2 AV2 AY2 BF2 BH2 BM2 BP2 BT2 BY2 CB2 CE2 CI2" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CE2" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA2" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AB2" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AD2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AE2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AG2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Normal,Curiga gangguan pendengaran"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CU2" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Gangguan Pendengaran"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM2" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Normal (visus 6/6 - 6/12),Curiga gangguan penglihatan (visus &lt;6/12)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CW2" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"Normal (visus 6/6 - 6/12),Gangguan penglihatan ringan (visus &lt;6/12 - 6/18),Gangguan penglihatan sedang (&lt;6/18 - 6/60),Gangguan penglihatan berat (&lt;6/60 - 3/60),Buta (&lt;3/60)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CX2" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"Visus membaik,Visus tidak membaik (visus tetap)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CY2" xr:uid="{00000000-0002-0000-0000-000014000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AP2" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"Kelainan refraksi ringan (0.50 - 3.00 Dioptri),Kelainan refraksi sedang (3.00 - 6.00 Dioptri),Kelainan refraksi berat (&gt;6.00 Dioptri)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CZ2" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DA2" xr:uid="{00000000-0002-0000-0000-000016000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AR2" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"Curiga katarak,Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DI2" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AZ2" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DJ2" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BA2" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ2" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EA2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EB2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BS2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EL2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EM2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EO2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EP2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EQ2" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ES2" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="ET2" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EU2" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EW2" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EX2" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EZ2" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AC2" xr:uid="{00000000-0002-0000-0000-000027000000}">
-      <formula1>"Benar semua,Salah satu/Dua,Tidak Tahu"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2" xr:uid="{00000000-0002-0000-0000-000028000000}">
-      <formula1>"Tidak terkendali/tak teratur (perlu pencahar),Kadang-kadang tak terkendali (1 x / minggu),Terkendali teratur"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-000029000000}">
-      <formula1>"Tak terkendali atau pakai kateter,Kadang-kadang tak terkendali (hanya 1 x / 24 jam),Mandiri"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM2" xr:uid="{00000000-0002-0000-0000-00002A000000}">
-      <formula1>"Mandiri,Butuh pertolongan orang lain"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2" xr:uid="{00000000-0002-0000-0000-00002B000000}">
-      <formula1>"Tergantung pertolongan orang lain,Perlu pertolongan pada beberapa kegiatan tetapi dapat mengerjakan sendiri beberapa kegiatan yang lain,Mandiri"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2" xr:uid="{00000000-0002-0000-0000-00002C000000}">
-      <formula1>"Tidak mampu,Perlu ditolong memotong makanan,Mandiri"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AP2" xr:uid="{00000000-0002-0000-0000-00002D000000}">
-      <formula1>"Tidak mampu,Perlu banyak bantuan untuk bias duduk (2 orang),Bantuan minimal 1 orang,Mandiri"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2" xr:uid="{00000000-0002-0000-0000-00002E000000}">
-      <formula1>"Tidak mampu,Bisa (pindah) dengan kursi roda,Bantuan minimal 1 orang,Mandiri"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AR2" xr:uid="{00000000-0002-0000-0000-00002F000000}">
-      <formula1>"Tergantung orang lain,Sebagian dibantu (misalnya: mengancing baju),Mandiri"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AS2" xr:uid="{00000000-0002-0000-0000-000030000000}">
-      <formula1>"Tidak mampu,Butuh pertolongan,Mandiri"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AT2" xr:uid="{00000000-0002-0000-0000-000031000000}">
-      <formula1>"Tergantung orang lain,Mandiri"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2" xr:uid="{00000000-0002-0000-0000-000032000000}">
-      <formula1>"SUDAH DITANYAKAN"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2" xr:uid="{00000000-0002-0000-0000-000033000000}">
-      <formula1>"Benar,Salah"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW2" xr:uid="{00000000-0002-0000-0000-000034000000}">
-      <formula1>"Benar 1 kata,Benar 2 Kata,Benar semua kata,Tidak dapat mengingat/mengulang kata"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BF2:BG2" xr:uid="{00000000-0002-0000-0000-000035000000}">
-      <formula1>"Bertahan 10 detik,Tidak bertahan 10 detik,Tidak dilakukan"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH2" xr:uid="{00000000-0002-0000-0000-000036000000}">
-      <formula1>"Bertahan 10 detik,Bertahan 3 - 9.99 detik,Bertahan &lt; 3 detik"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK2" xr:uid="{00000000-0002-0000-0000-000037000000}">
-      <formula1>"Nafsu Makan Yang Sangat Berkurang,Nafsu Makan Sedikit Berkurang,Nafsu Makan Biasa saja"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2" xr:uid="{00000000-0002-0000-0000-000038000000}">
-      <formula1>"Penurunan BB &gt; 3 Kg,Tidak Tahu,Penurunan BB antara 1 - 3 Kg"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2" xr:uid="{00000000-0002-0000-0000-000039000000}">
-      <formula1>"Dementia atau depresi berat,Demensia/kepikunan ringan,Tidak ada masalah psikologis"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2" xr:uid="{00000000-0002-0000-0000-00003A000000}">
-      <formula1>"IMT &lt;19,IMT 19 - &lt;21,IMT 21 - &lt;23,IMT &gt;= 23"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ2" xr:uid="{00000000-0002-0000-0000-00003B000000}">
-      <formula1>"&lt;31 cm,&gt;= 31 cm"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{0739CCB7-0531-A140-9A86-D8E33CA4DE7A}">
       <formula1>"Berdiri,Telentang"</formula1>

</xml_diff>

<commit_message>
do jantung bawaan, berat lahir, dan riwayat imunisasi hepatitis B
</commit_message>
<xml_diff>
--- a/dataset/anak.xlsx
+++ b/dataset/anak.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ABC4917-D04E-E147-BFFC-CECC50C12AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26B9198C-6645-2644-B5B5-614EEE7EBC1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4480" yWindow="-21000" windowWidth="36000" windowHeight="19520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="AB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -55,7 +55,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="AG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -70,7 +70,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="AJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -85,7 +85,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="BA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -100,7 +100,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="BS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="145">
   <si>
     <t>batas_awal</t>
   </si>
@@ -537,6 +537,24 @@
   </si>
   <si>
     <t>Tidak ada</t>
+  </si>
+  <si>
+    <t>mendapat_imunisasi_hepatitis_b</t>
+  </si>
+  <si>
+    <t>Sudah</t>
+  </si>
+  <si>
+    <t>berat_lahir</t>
+  </si>
+  <si>
+    <t>berat_sekarang</t>
+  </si>
+  <si>
+    <t>pjb_tangan_kanan</t>
+  </si>
+  <si>
+    <t>pjb_kaki</t>
   </si>
 </sst>
 </file>
@@ -939,7 +957,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CM2"/>
+  <dimension ref="A1:CR2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -959,70 +977,75 @@
     <col min="18" max="18" width="23.5" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="14.83203125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="14.83203125" customWidth="1"/>
-    <col min="21" max="21" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="22.83203125" customWidth="1"/>
-    <col min="26" max="26" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="16.1640625" customWidth="1"/>
-    <col min="28" max="28" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="30" max="31" width="12.33203125" customWidth="1"/>
-    <col min="32" max="32" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.1640625" customWidth="1"/>
-    <col min="34" max="34" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="23.6640625" customWidth="1"/>
-    <col min="37" max="37" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="12.83203125" customWidth="1"/>
-    <col min="43" max="43" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="17.5" customWidth="1"/>
-    <col min="46" max="46" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="13" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="50" max="52" width="19.5" customWidth="1"/>
-    <col min="53" max="53" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="9.83203125" customWidth="1"/>
-    <col min="55" max="55" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="56" max="59" width="11.5" customWidth="1"/>
-    <col min="60" max="60" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="9" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="18.1640625" customWidth="1"/>
-    <col min="67" max="67" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="69" max="71" width="8.33203125" customWidth="1"/>
-    <col min="72" max="72" width="22" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="14" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="14" customWidth="1"/>
-    <col min="77" max="77" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="18.1640625" customWidth="1"/>
-    <col min="80" max="80" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="83" max="85" width="18.1640625" customWidth="1"/>
-    <col min="86" max="86" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="35" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="43.1640625" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="18.1640625" customWidth="1"/>
-    <col min="90" max="90" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="10.83203125" customWidth="1"/>
+    <col min="21" max="21" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="13.6640625" customWidth="1"/>
+    <col min="26" max="26" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="22.83203125" customWidth="1"/>
+    <col min="31" max="31" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="16.1640625" customWidth="1"/>
+    <col min="33" max="33" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="12.33203125" customWidth="1"/>
+    <col min="37" max="37" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="14.1640625" customWidth="1"/>
+    <col min="39" max="39" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="23.6640625" customWidth="1"/>
+    <col min="42" max="42" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="12.83203125" customWidth="1"/>
+    <col min="48" max="48" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="17.5" customWidth="1"/>
+    <col min="51" max="51" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="13" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="55" max="57" width="19.5" customWidth="1"/>
+    <col min="58" max="58" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="9.83203125" customWidth="1"/>
+    <col min="60" max="60" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="61" max="64" width="11.5" customWidth="1"/>
+    <col min="65" max="65" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="9" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="18.1640625" customWidth="1"/>
+    <col min="72" max="72" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="74" max="76" width="8.33203125" customWidth="1"/>
+    <col min="77" max="77" width="22" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="14" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="14" customWidth="1"/>
+    <col min="82" max="82" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="18.1640625" customWidth="1"/>
+    <col min="85" max="85" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="88" max="90" width="18.1640625" customWidth="1"/>
+    <col min="91" max="91" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="35" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="18.1640625" customWidth="1"/>
+    <col min="95" max="95" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:91" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1081,220 +1104,235 @@
         <v>18</v>
       </c>
       <c r="U1" t="s">
+        <v>139</v>
+      </c>
+      <c r="V1" t="s">
+        <v>141</v>
+      </c>
+      <c r="W1" t="s">
+        <v>142</v>
+      </c>
+      <c r="X1" t="s">
+        <v>143</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>144</v>
+      </c>
+      <c r="Z1" t="s">
         <v>19</v>
       </c>
-      <c r="V1" t="s">
+      <c r="AA1" t="s">
         <v>20</v>
       </c>
-      <c r="W1" t="s">
+      <c r="AB1" t="s">
         <v>21</v>
       </c>
-      <c r="X1" t="s">
+      <c r="AC1" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="AD1" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AE1" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AF1" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AG1" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AH1" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AI1" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AJ1" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AK1" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AL1" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AM1" t="s">
         <v>32</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AN1" t="s">
         <v>33</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AO1" t="s">
         <v>34</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AP1" t="s">
         <v>132</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AQ1" t="s">
         <v>134</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AR1" t="s">
         <v>135</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AS1" t="s">
         <v>136</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AT1" t="s">
         <v>137</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AU1" t="s">
         <v>35</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AV1" t="s">
         <v>36</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AW1" t="s">
         <v>37</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AX1" t="s">
         <v>38</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AY1" t="s">
         <v>39</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AZ1" t="s">
         <v>40</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="BA1" t="s">
         <v>41</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="BB1" t="s">
         <v>42</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="BC1" t="s">
         <v>43</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="BD1" t="s">
         <v>44</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BE1" t="s">
         <v>45</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BF1" t="s">
         <v>46</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BG1" t="s">
         <v>47</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BH1" t="s">
         <v>48</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BI1" t="s">
         <v>49</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BJ1" t="s">
         <v>50</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BK1" t="s">
         <v>51</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BL1" t="s">
         <v>52</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BM1" t="s">
         <v>53</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BN1" t="s">
         <v>54</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BO1" t="s">
         <v>55</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BP1" t="s">
         <v>56</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BQ1" t="s">
         <v>57</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BR1" t="s">
         <v>58</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BS1" t="s">
         <v>59</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BT1" t="s">
         <v>60</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BU1" t="s">
         <v>61</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BV1" t="s">
         <v>62</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BW1" t="s">
         <v>63</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BX1" t="s">
         <v>64</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BY1" t="s">
         <v>65</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BZ1" t="s">
         <v>66</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="CA1" t="s">
         <v>67</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="CB1" t="s">
         <v>68</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CC1" t="s">
         <v>69</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CD1" t="s">
         <v>70</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CE1" t="s">
         <v>71</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CF1" t="s">
         <v>72</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CG1" t="s">
         <v>73</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CH1" t="s">
         <v>74</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CI1" t="s">
         <v>75</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CJ1" t="s">
         <v>76</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CK1" t="s">
         <v>77</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CL1" t="s">
         <v>78</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CM1" t="s">
         <v>79</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CN1" t="s">
         <v>80</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CO1" t="s">
         <v>81</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CP1" t="s">
         <v>82</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CQ1" t="s">
         <v>83</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CR1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:91" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:96" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>85</v>
       </c>
@@ -1350,88 +1388,88 @@
         <v>93</v>
       </c>
       <c r="U2" t="s">
-        <v>94</v>
-      </c>
-      <c r="V2" t="s">
-        <v>95</v>
-      </c>
-      <c r="W2" t="s">
-        <v>96</v>
-      </c>
-      <c r="X2" t="s">
-        <v>97</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>98</v>
+        <v>140</v>
+      </c>
+      <c r="V2">
+        <v>2900</v>
+      </c>
+      <c r="W2">
+        <v>6000</v>
+      </c>
+      <c r="X2">
+        <v>80</v>
+      </c>
+      <c r="Y2">
+        <v>90</v>
       </c>
       <c r="Z2" t="s">
         <v>94</v>
       </c>
       <c r="AA2" t="s">
+        <v>95</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>96</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>97</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AF2" t="s">
         <v>99</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AG2" t="s">
         <v>100</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>94</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>101</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>102</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>94</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>103</v>
       </c>
       <c r="AH2" t="s">
         <v>94</v>
       </c>
       <c r="AI2" t="s">
+        <v>101</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN2" t="s">
         <v>104</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AO2" t="s">
         <v>105</v>
       </c>
-      <c r="AK2" t="s">
+      <c r="AP2" t="s">
         <v>133</v>
       </c>
-      <c r="AL2" t="s">
+      <c r="AQ2" t="s">
         <v>93</v>
       </c>
-      <c r="AM2" t="s">
+      <c r="AR2" t="s">
         <v>93</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AS2" t="s">
         <v>94</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AT2" t="s">
         <v>138</v>
       </c>
-      <c r="AP2" t="s">
+      <c r="AU2" t="s">
         <v>106</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="AV2" t="s">
         <v>94</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AS2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AT2" t="s">
-        <v>94</v>
-      </c>
-      <c r="AU2" t="s">
-        <v>107</v>
-      </c>
-      <c r="AV2" t="s">
-        <v>108</v>
       </c>
       <c r="AW2" t="s">
         <v>91</v>
@@ -1440,226 +1478,241 @@
         <v>91</v>
       </c>
       <c r="AY2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AZ2" t="s">
+        <v>107</v>
+      </c>
+      <c r="BA2" t="s">
+        <v>108</v>
+      </c>
+      <c r="BB2" t="s">
         <v>91</v>
       </c>
-      <c r="AZ2" t="s">
+      <c r="BC2" t="s">
         <v>91</v>
       </c>
-      <c r="BA2" t="s">
+      <c r="BD2" t="s">
+        <v>91</v>
+      </c>
+      <c r="BE2" t="s">
+        <v>91</v>
+      </c>
+      <c r="BF2" t="s">
         <v>94</v>
       </c>
-      <c r="BB2" t="s">
+      <c r="BG2" t="s">
         <v>109</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>94</v>
-      </c>
-      <c r="BD2" t="s">
-        <v>110</v>
-      </c>
-      <c r="BE2" t="s">
-        <v>110</v>
-      </c>
-      <c r="BF2" t="s">
-        <v>111</v>
-      </c>
-      <c r="BG2" t="s">
-        <v>112</v>
       </c>
       <c r="BH2" t="s">
         <v>94</v>
       </c>
       <c r="BI2" t="s">
+        <v>110</v>
+      </c>
+      <c r="BJ2" t="s">
+        <v>110</v>
+      </c>
+      <c r="BK2" t="s">
+        <v>111</v>
+      </c>
+      <c r="BL2" t="s">
+        <v>112</v>
+      </c>
+      <c r="BM2" t="s">
+        <v>94</v>
+      </c>
+      <c r="BN2" t="s">
         <v>113</v>
       </c>
-      <c r="BJ2" t="s">
+      <c r="BO2" t="s">
         <v>114</v>
       </c>
-      <c r="BK2" t="s">
+      <c r="BP2" t="s">
         <v>94</v>
       </c>
-      <c r="BL2" t="s">
+      <c r="BQ2" t="s">
         <v>115</v>
       </c>
-      <c r="BM2" t="s">
+      <c r="BR2" t="s">
         <v>116</v>
       </c>
-      <c r="BN2" t="s">
+      <c r="BS2" t="s">
         <v>117</v>
-      </c>
-      <c r="BO2" t="s">
-        <v>94</v>
-      </c>
-      <c r="BP2" t="s">
-        <v>118</v>
-      </c>
-      <c r="BQ2" t="s">
-        <v>110</v>
-      </c>
-      <c r="BR2" t="s">
-        <v>109</v>
-      </c>
-      <c r="BS2" t="s">
-        <v>119</v>
       </c>
       <c r="BT2" t="s">
         <v>94</v>
       </c>
       <c r="BU2" t="s">
+        <v>118</v>
+      </c>
+      <c r="BV2" t="s">
+        <v>110</v>
+      </c>
+      <c r="BW2" t="s">
+        <v>109</v>
+      </c>
+      <c r="BX2" t="s">
         <v>119</v>
       </c>
-      <c r="BV2" t="s">
+      <c r="BY2" t="s">
+        <v>94</v>
+      </c>
+      <c r="BZ2" t="s">
+        <v>119</v>
+      </c>
+      <c r="CA2" t="s">
         <v>120</v>
       </c>
-      <c r="BW2" t="s">
+      <c r="CB2" t="s">
         <v>94</v>
       </c>
-      <c r="BX2" t="s">
+      <c r="CC2" t="s">
         <v>93</v>
       </c>
-      <c r="BY2" t="s">
+      <c r="CD2" t="s">
         <v>121</v>
       </c>
-      <c r="BZ2" t="s">
+      <c r="CE2" t="s">
         <v>94</v>
       </c>
-      <c r="CA2" t="s">
+      <c r="CF2" t="s">
         <v>122</v>
       </c>
-      <c r="CB2" t="s">
+      <c r="CG2" t="s">
         <v>123</v>
       </c>
-      <c r="CC2" t="s">
+      <c r="CH2" t="s">
         <v>124</v>
       </c>
-      <c r="CD2" t="s">
+      <c r="CI2" t="s">
         <v>94</v>
       </c>
-      <c r="CE2" t="s">
+      <c r="CJ2" t="s">
         <v>125</v>
       </c>
-      <c r="CF2" t="s">
+      <c r="CK2" t="s">
         <v>126</v>
       </c>
-      <c r="CG2" t="s">
+      <c r="CL2" t="s">
         <v>127</v>
       </c>
-      <c r="CH2" t="s">
+      <c r="CM2" t="s">
         <v>128</v>
       </c>
-      <c r="CI2" t="s">
+      <c r="CN2" t="s">
         <v>129</v>
       </c>
-      <c r="CJ2" t="s">
+      <c r="CO2" t="s">
         <v>130</v>
       </c>
-      <c r="CK2" t="s">
+      <c r="CP2" t="s">
         <v>131</v>
       </c>
-      <c r="CL2" t="s">
+      <c r="CQ2" t="s">
         <v>93</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="39">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2 O2:S2 AW2:AZ2 AR2:AS2 AP2" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="40">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2 O2:S2 BB2:BE2 AW2:AX2 AU2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2 CK2 CH2" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2 Z2 AC2 AF2 AH2 AN2 AQ2 AT2 BA2 BC2 BH2 BK2 BO2 BT2 BW2 BZ2 CD2" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2 CP2 CM2" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Z2 AE2 AH2 AK2 AM2 AS2 AV2 AY2 BF2 BH2 BM2 BP2 BT2 BY2 CB2 CE2 CI2" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA2" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AB2" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AC2" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA2" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AF2" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AB2" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AG2" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AD2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AE2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AG2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AP2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Sesuai Umur,Ada kemungkinan penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM2" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AR2" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Normal,Curiga kelainan pupil putih pada anak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AZ2" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BA2" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ2" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BM2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BN2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BS2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BY2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CE2" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{00000000-0002-0000-0000-000027000000}">
@@ -1671,7 +1724,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"Perkembangan sesuai usia,Perkembangan meragukan,Perkembangan curiga adanya penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y2" xr:uid="{8CF71D70-E85F-9946-A33A-2D9580913A62}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AD2" xr:uid="{8CF71D70-E85F-9946-A33A-2D9580913A62}">
       <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
         <mc:Choice Requires="x12ac">
           <x12ac:list>Mtb not detected (Neg),"Mtb detected, Rif resistance not detected (Rif Sen)","Mtb detected, Rif resistance detected (Rif Res)","MTB detected, Rif Resistance Indeterminate (Rif Indet)",Invalid,Error,No Result</x12ac:list>
@@ -1681,8 +1734,11 @@
         </mc:Fallback>
       </mc:AlternateContent>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2" xr:uid="{6581135A-9ACF-CC48-9D5E-ECD150302CDE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AT2" xr:uid="{6581135A-9ACF-CC48-9D5E-ECD150302CDE}">
       <formula1>"Tidak ada,1,2,3,&gt;3"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2" xr:uid="{C8F9D09B-6ED1-1641-81FF-EFC972969A8B}">
+      <formula1>"Sudah,Belum"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
wip SHK, darah tumit, and konfirmasi SHK
</commit_message>
<xml_diff>
--- a/dataset/anak.xlsx
+++ b/dataset/anak.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26B9198C-6645-2644-B5B5-614EEE7EBC1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{615E66AB-C2C4-EC49-8BEC-62283C351191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4480" yWindow="-21000" windowWidth="36000" windowHeight="19520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="AG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -55,7 +55,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="AL1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -70,7 +70,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="AO1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -85,7 +85,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="BF1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -100,7 +100,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BS1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="BX1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="150">
   <si>
     <t>batas_awal</t>
   </si>
@@ -555,6 +555,21 @@
   </si>
   <si>
     <t>pjb_kaki</t>
+  </si>
+  <si>
+    <t>darah_tumit</t>
+  </si>
+  <si>
+    <t>shk</t>
+  </si>
+  <si>
+    <t>g6pd</t>
+  </si>
+  <si>
+    <t>hak</t>
+  </si>
+  <si>
+    <t>dilakukan_konfirmasi_shk</t>
   </si>
 </sst>
 </file>
@@ -957,7 +972,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CR2"/>
+  <dimension ref="A1:CW2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -981,71 +996,73 @@
     <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="16" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.6640625" customWidth="1"/>
-    <col min="26" max="26" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="22.83203125" customWidth="1"/>
-    <col min="31" max="31" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="16.1640625" customWidth="1"/>
-    <col min="33" max="33" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="12.33203125" customWidth="1"/>
-    <col min="37" max="37" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="14.1640625" customWidth="1"/>
-    <col min="39" max="39" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="23.6640625" customWidth="1"/>
-    <col min="42" max="42" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="12.83203125" customWidth="1"/>
-    <col min="48" max="48" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="17.5" customWidth="1"/>
-    <col min="51" max="51" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="13" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="55" max="57" width="19.5" customWidth="1"/>
-    <col min="58" max="58" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="9.83203125" customWidth="1"/>
-    <col min="60" max="60" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="61" max="64" width="11.5" customWidth="1"/>
-    <col min="65" max="65" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="9" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="18.1640625" customWidth="1"/>
-    <col min="72" max="72" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="74" max="76" width="8.33203125" customWidth="1"/>
-    <col min="77" max="77" width="22" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="14" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="14" customWidth="1"/>
-    <col min="82" max="82" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="18.1640625" customWidth="1"/>
-    <col min="85" max="85" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="88" max="90" width="18.1640625" customWidth="1"/>
-    <col min="91" max="91" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="35" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="43.1640625" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="18.1640625" customWidth="1"/>
-    <col min="95" max="95" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="10.83203125" customWidth="1"/>
+    <col min="25" max="26" width="13.6640625" customWidth="1"/>
+    <col min="27" max="27" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="30" width="13.6640625" customWidth="1"/>
+    <col min="31" max="31" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="22.83203125" customWidth="1"/>
+    <col min="36" max="36" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="16.1640625" customWidth="1"/>
+    <col min="38" max="38" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="40" max="41" width="12.33203125" customWidth="1"/>
+    <col min="42" max="42" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="14.1640625" customWidth="1"/>
+    <col min="44" max="44" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="23.6640625" customWidth="1"/>
+    <col min="47" max="47" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="12.83203125" customWidth="1"/>
+    <col min="53" max="53" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="17.5" customWidth="1"/>
+    <col min="56" max="56" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="13" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="60" max="62" width="19.5" customWidth="1"/>
+    <col min="63" max="63" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="9.83203125" customWidth="1"/>
+    <col min="65" max="65" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="66" max="69" width="11.5" customWidth="1"/>
+    <col min="70" max="70" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="9" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="18.1640625" customWidth="1"/>
+    <col min="77" max="77" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="79" max="81" width="8.33203125" customWidth="1"/>
+    <col min="82" max="82" width="22" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="14" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="14" customWidth="1"/>
+    <col min="87" max="87" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="18.1640625" customWidth="1"/>
+    <col min="90" max="90" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="93" max="95" width="18.1640625" customWidth="1"/>
+    <col min="96" max="96" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="35" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="18.1640625" customWidth="1"/>
+    <col min="100" max="100" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:96" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:101" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1119,220 +1136,235 @@
         <v>144</v>
       </c>
       <c r="Z1" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>146</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>147</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>148</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>149</v>
+      </c>
+      <c r="AE1" t="s">
         <v>19</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AF1" t="s">
         <v>20</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AG1" t="s">
         <v>21</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AH1" t="s">
         <v>22</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AI1" t="s">
         <v>23</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AJ1" t="s">
         <v>24</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AK1" t="s">
         <v>25</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AL1" t="s">
         <v>26</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AM1" t="s">
         <v>27</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AN1" t="s">
         <v>28</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AO1" t="s">
         <v>29</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AP1" t="s">
         <v>30</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AQ1" t="s">
         <v>31</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AR1" t="s">
         <v>32</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AS1" t="s">
         <v>33</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AT1" t="s">
         <v>34</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AU1" t="s">
         <v>132</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AV1" t="s">
         <v>134</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AW1" t="s">
         <v>135</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AX1" t="s">
         <v>136</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AY1" t="s">
         <v>137</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AZ1" t="s">
         <v>35</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="BA1" t="s">
         <v>36</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="BB1" t="s">
         <v>37</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="BC1" t="s">
         <v>38</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="BD1" t="s">
         <v>39</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BE1" t="s">
         <v>40</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BF1" t="s">
         <v>41</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BG1" t="s">
         <v>42</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BH1" t="s">
         <v>43</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BI1" t="s">
         <v>44</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BJ1" t="s">
         <v>45</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BK1" t="s">
         <v>46</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BL1" t="s">
         <v>47</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BM1" t="s">
         <v>48</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BN1" t="s">
         <v>49</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BO1" t="s">
         <v>50</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BP1" t="s">
         <v>51</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BQ1" t="s">
         <v>52</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BR1" t="s">
         <v>53</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BS1" t="s">
         <v>54</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BT1" t="s">
         <v>55</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BU1" t="s">
         <v>56</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BV1" t="s">
         <v>57</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BW1" t="s">
         <v>58</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BX1" t="s">
         <v>59</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BY1" t="s">
         <v>60</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BZ1" t="s">
         <v>61</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="CA1" t="s">
         <v>62</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="CB1" t="s">
         <v>63</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CC1" t="s">
         <v>64</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CD1" t="s">
         <v>65</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CE1" t="s">
         <v>66</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CF1" t="s">
         <v>67</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CG1" t="s">
         <v>68</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CH1" t="s">
         <v>69</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CI1" t="s">
         <v>70</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CJ1" t="s">
         <v>71</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CK1" t="s">
         <v>72</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CL1" t="s">
         <v>73</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CM1" t="s">
         <v>74</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CN1" t="s">
         <v>75</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CO1" t="s">
         <v>76</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CP1" t="s">
         <v>77</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CQ1" t="s">
         <v>78</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CR1" t="s">
         <v>79</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CS1" t="s">
         <v>80</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CT1" t="s">
         <v>81</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="CU1" t="s">
         <v>82</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="CV1" t="s">
         <v>83</v>
       </c>
-      <c r="CR1" t="s">
+      <c r="CW1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:96" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:101" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>85</v>
       </c>
@@ -1403,88 +1435,88 @@
         <v>90</v>
       </c>
       <c r="Z2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="AA2" t="s">
-        <v>95</v>
+        <v>124</v>
       </c>
       <c r="AB2" t="s">
-        <v>96</v>
+        <v>124</v>
       </c>
       <c r="AC2" t="s">
-        <v>97</v>
+        <v>124</v>
       </c>
       <c r="AD2" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="AE2" t="s">
         <v>94</v>
       </c>
       <c r="AF2" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>96</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>97</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>98</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AK2" t="s">
         <v>99</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AL2" t="s">
         <v>100</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>94</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>101</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>102</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>94</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>103</v>
       </c>
       <c r="AM2" t="s">
         <v>94</v>
       </c>
       <c r="AN2" t="s">
+        <v>101</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AS2" t="s">
         <v>104</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AT2" t="s">
         <v>105</v>
       </c>
-      <c r="AP2" t="s">
+      <c r="AU2" t="s">
         <v>133</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="AV2" t="s">
         <v>93</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="AW2" t="s">
         <v>93</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AX2" t="s">
         <v>94</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="AY2" t="s">
         <v>138</v>
       </c>
-      <c r="AU2" t="s">
+      <c r="AZ2" t="s">
         <v>106</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="BA2" t="s">
         <v>94</v>
-      </c>
-      <c r="AW2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AX2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AY2" t="s">
-        <v>94</v>
-      </c>
-      <c r="AZ2" t="s">
-        <v>107</v>
-      </c>
-      <c r="BA2" t="s">
-        <v>108</v>
       </c>
       <c r="BB2" t="s">
         <v>91</v>
@@ -1493,226 +1525,241 @@
         <v>91</v>
       </c>
       <c r="BD2" t="s">
+        <v>94</v>
+      </c>
+      <c r="BE2" t="s">
+        <v>107</v>
+      </c>
+      <c r="BF2" t="s">
+        <v>108</v>
+      </c>
+      <c r="BG2" t="s">
         <v>91</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BH2" t="s">
         <v>91</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BI2" t="s">
+        <v>91</v>
+      </c>
+      <c r="BJ2" t="s">
+        <v>91</v>
+      </c>
+      <c r="BK2" t="s">
         <v>94</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BL2" t="s">
         <v>109</v>
-      </c>
-      <c r="BH2" t="s">
-        <v>94</v>
-      </c>
-      <c r="BI2" t="s">
-        <v>110</v>
-      </c>
-      <c r="BJ2" t="s">
-        <v>110</v>
-      </c>
-      <c r="BK2" t="s">
-        <v>111</v>
-      </c>
-      <c r="BL2" t="s">
-        <v>112</v>
       </c>
       <c r="BM2" t="s">
         <v>94</v>
       </c>
       <c r="BN2" t="s">
+        <v>110</v>
+      </c>
+      <c r="BO2" t="s">
+        <v>110</v>
+      </c>
+      <c r="BP2" t="s">
+        <v>111</v>
+      </c>
+      <c r="BQ2" t="s">
+        <v>112</v>
+      </c>
+      <c r="BR2" t="s">
+        <v>94</v>
+      </c>
+      <c r="BS2" t="s">
         <v>113</v>
       </c>
-      <c r="BO2" t="s">
+      <c r="BT2" t="s">
         <v>114</v>
       </c>
-      <c r="BP2" t="s">
+      <c r="BU2" t="s">
         <v>94</v>
       </c>
-      <c r="BQ2" t="s">
+      <c r="BV2" t="s">
         <v>115</v>
       </c>
-      <c r="BR2" t="s">
+      <c r="BW2" t="s">
         <v>116</v>
       </c>
-      <c r="BS2" t="s">
+      <c r="BX2" t="s">
         <v>117</v>
-      </c>
-      <c r="BT2" t="s">
-        <v>94</v>
-      </c>
-      <c r="BU2" t="s">
-        <v>118</v>
-      </c>
-      <c r="BV2" t="s">
-        <v>110</v>
-      </c>
-      <c r="BW2" t="s">
-        <v>109</v>
-      </c>
-      <c r="BX2" t="s">
-        <v>119</v>
       </c>
       <c r="BY2" t="s">
         <v>94</v>
       </c>
       <c r="BZ2" t="s">
+        <v>118</v>
+      </c>
+      <c r="CA2" t="s">
+        <v>110</v>
+      </c>
+      <c r="CB2" t="s">
+        <v>109</v>
+      </c>
+      <c r="CC2" t="s">
         <v>119</v>
       </c>
-      <c r="CA2" t="s">
+      <c r="CD2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CE2" t="s">
+        <v>119</v>
+      </c>
+      <c r="CF2" t="s">
         <v>120</v>
       </c>
-      <c r="CB2" t="s">
+      <c r="CG2" t="s">
         <v>94</v>
       </c>
-      <c r="CC2" t="s">
+      <c r="CH2" t="s">
         <v>93</v>
       </c>
-      <c r="CD2" t="s">
+      <c r="CI2" t="s">
         <v>121</v>
       </c>
-      <c r="CE2" t="s">
+      <c r="CJ2" t="s">
         <v>94</v>
       </c>
-      <c r="CF2" t="s">
+      <c r="CK2" t="s">
         <v>122</v>
       </c>
-      <c r="CG2" t="s">
+      <c r="CL2" t="s">
         <v>123</v>
       </c>
-      <c r="CH2" t="s">
+      <c r="CM2" t="s">
         <v>124</v>
       </c>
-      <c r="CI2" t="s">
+      <c r="CN2" t="s">
         <v>94</v>
       </c>
-      <c r="CJ2" t="s">
+      <c r="CO2" t="s">
         <v>125</v>
       </c>
-      <c r="CK2" t="s">
+      <c r="CP2" t="s">
         <v>126</v>
       </c>
-      <c r="CL2" t="s">
+      <c r="CQ2" t="s">
         <v>127</v>
       </c>
-      <c r="CM2" t="s">
+      <c r="CR2" t="s">
         <v>128</v>
       </c>
-      <c r="CN2" t="s">
+      <c r="CS2" t="s">
         <v>129</v>
       </c>
-      <c r="CO2" t="s">
+      <c r="CT2" t="s">
         <v>130</v>
       </c>
-      <c r="CP2" t="s">
+      <c r="CU2" t="s">
         <v>131</v>
       </c>
-      <c r="CQ2" t="s">
+      <c r="CV2" t="s">
         <v>93</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="40">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2 O2:S2 BB2:BE2 AW2:AX2 AU2" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="41">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2 O2:S2 BG2:BJ2 BB2:BC2 AZ2 Z2 AD2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2 CP2 CM2" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Z2 AE2 AH2 AK2 AM2 AS2 AV2 AY2 BF2 BH2 BM2 BP2 BT2 BY2 CB2 CE2 CI2" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2 CU2 CR2" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AE2 AJ2 AM2 AP2 AR2 AX2 BA2 BD2 BK2 BM2 BR2 BU2 BY2 CD2 CG2 CJ2 CN2" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA2" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AF2" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AB2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AG2" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AC2" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH2" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AF2" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AG2" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AS2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AT2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AP2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Sesuai Umur,Ada kemungkinan penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AR2" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW2" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Normal,Curiga kelainan pupil putih pada anak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AZ2" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BA2" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BF2" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ2" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BV2" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BW2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BS2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{00000000-0002-0000-0000-000027000000}">
@@ -1724,7 +1771,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"Perkembangan sesuai usia,Perkembangan meragukan,Perkembangan curiga adanya penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AD2" xr:uid="{8CF71D70-E85F-9946-A33A-2D9580913A62}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2" xr:uid="{8CF71D70-E85F-9946-A33A-2D9580913A62}">
       <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
         <mc:Choice Requires="x12ac">
           <x12ac:list>Mtb not detected (Neg),"Mtb detected, Rif resistance not detected (Rif Sen)","Mtb detected, Rif resistance detected (Rif Res)","MTB detected, Rif Resistance Indeterminate (Rif Indet)",Invalid,Error,No Result</x12ac:list>
@@ -1734,11 +1781,14 @@
         </mc:Fallback>
       </mc:AlternateContent>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AT2" xr:uid="{6581135A-9ACF-CC48-9D5E-ECD150302CDE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AY2" xr:uid="{6581135A-9ACF-CC48-9D5E-ECD150302CDE}">
       <formula1>"Tidak ada,1,2,3,&gt;3"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2" xr:uid="{C8F9D09B-6ED1-1641-81FF-EFC972969A8B}">
       <formula1>"Sudah,Belum"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA2:AC2" xr:uid="{8053A0D4-04B2-4C40-B539-974DDB07ADD7}">
+      <formula1>"Positif,Negatif"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
do konfirmasi SHK, warna kulit dan tinja, hasil kramer, warna kulit dan tinja 28 hari
</commit_message>
<xml_diff>
--- a/dataset/anak.xlsx
+++ b/dataset/anak.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{615E66AB-C2C4-EC49-8BEC-62283C351191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFC5F5B1-DBF2-C54E-B461-FF8CD7436F9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4480" yWindow="-21000" windowWidth="36000" windowHeight="19520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="19520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="AQ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -55,7 +55,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AL1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="AV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -70,7 +70,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AO1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="AY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -85,7 +85,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BF1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="BP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -100,7 +100,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BX1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="CH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="162">
   <si>
     <t>batas_awal</t>
   </si>
@@ -570,6 +570,42 @@
   </si>
   <si>
     <t>dilakukan_konfirmasi_shk</t>
+  </si>
+  <si>
+    <t>hasil_konfirm_shk</t>
+  </si>
+  <si>
+    <t>dilakukan_konfirmasi_g6pd</t>
+  </si>
+  <si>
+    <t>hasil_konfirm_g6pd</t>
+  </si>
+  <si>
+    <t>dilakukan_konfirmasi_hak</t>
+  </si>
+  <si>
+    <t>hasil_konfirm_hak</t>
+  </si>
+  <si>
+    <t>dilakukan_edukasi_warna_kulit_dan_tinja</t>
+  </si>
+  <si>
+    <t>nilai_hasil_kramer</t>
+  </si>
+  <si>
+    <t>Bayi Kuning Kramer 1-3</t>
+  </si>
+  <si>
+    <t>tgl_pemeriksaan_kramer</t>
+  </si>
+  <si>
+    <t>kramer_bayi_kuning</t>
+  </si>
+  <si>
+    <t>derajat_warna_tinja</t>
+  </si>
+  <si>
+    <t>&gt;3 Normal</t>
   </si>
 </sst>
 </file>
@@ -972,7 +1008,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CW2"/>
+  <dimension ref="A1:DG2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -998,71 +1034,75 @@
     <col min="24" max="24" width="16" bestFit="1" customWidth="1"/>
     <col min="25" max="26" width="13.6640625" customWidth="1"/>
     <col min="27" max="27" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="28" max="30" width="13.6640625" customWidth="1"/>
-    <col min="31" max="31" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="22.83203125" customWidth="1"/>
-    <col min="36" max="36" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="16.1640625" customWidth="1"/>
-    <col min="38" max="38" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="40" max="41" width="12.33203125" customWidth="1"/>
-    <col min="42" max="42" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="14.1640625" customWidth="1"/>
-    <col min="44" max="44" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="23.6640625" customWidth="1"/>
-    <col min="47" max="47" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="12.83203125" customWidth="1"/>
-    <col min="53" max="53" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="17.5" customWidth="1"/>
-    <col min="56" max="56" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="13" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="60" max="62" width="19.5" customWidth="1"/>
-    <col min="63" max="63" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="9.83203125" customWidth="1"/>
-    <col min="65" max="65" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="66" max="69" width="11.5" customWidth="1"/>
-    <col min="70" max="70" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="9" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="18.1640625" customWidth="1"/>
-    <col min="77" max="77" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="79" max="81" width="8.33203125" customWidth="1"/>
-    <col min="82" max="82" width="22" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="14" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="14" customWidth="1"/>
-    <col min="87" max="87" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="18.1640625" customWidth="1"/>
-    <col min="90" max="90" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="93" max="95" width="18.1640625" customWidth="1"/>
-    <col min="96" max="96" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="35" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="29" width="13.6640625" customWidth="1"/>
+    <col min="30" max="30" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="31" max="35" width="22.5" customWidth="1"/>
+    <col min="36" max="36" width="35.83203125" bestFit="1" customWidth="1"/>
+    <col min="37" max="40" width="22.5" customWidth="1"/>
+    <col min="41" max="41" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="22.83203125" customWidth="1"/>
+    <col min="46" max="46" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="16.1640625" customWidth="1"/>
+    <col min="48" max="48" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="50" max="51" width="12.33203125" customWidth="1"/>
+    <col min="52" max="52" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="14.1640625" customWidth="1"/>
+    <col min="54" max="54" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="23.6640625" customWidth="1"/>
+    <col min="57" max="57" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="12.83203125" customWidth="1"/>
+    <col min="63" max="63" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="17.5" customWidth="1"/>
+    <col min="66" max="66" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="13" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="70" max="72" width="19.5" customWidth="1"/>
+    <col min="73" max="73" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="9.83203125" customWidth="1"/>
+    <col min="75" max="75" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="76" max="79" width="11.5" customWidth="1"/>
+    <col min="80" max="80" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="9" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="18.1640625" customWidth="1"/>
+    <col min="87" max="87" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="89" max="91" width="8.33203125" customWidth="1"/>
+    <col min="92" max="92" width="22" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="14" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="14" customWidth="1"/>
+    <col min="97" max="97" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="18.1640625" bestFit="1" customWidth="1"/>
     <col min="99" max="99" width="18.1640625" customWidth="1"/>
-    <col min="100" max="100" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="10.83203125" customWidth="1"/>
+    <col min="100" max="100" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="103" max="105" width="18.1640625" customWidth="1"/>
+    <col min="106" max="106" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="35" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="109" max="109" width="18.1640625" customWidth="1"/>
+    <col min="110" max="110" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:101" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1151,220 +1191,250 @@
         <v>149</v>
       </c>
       <c r="AE1" t="s">
+        <v>150</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>151</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>152</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>153</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>154</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>155</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>156</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>158</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>159</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>160</v>
+      </c>
+      <c r="AO1" t="s">
         <v>19</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AP1" t="s">
         <v>20</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AQ1" t="s">
         <v>21</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AR1" t="s">
         <v>22</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AS1" t="s">
         <v>23</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AT1" t="s">
         <v>24</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AU1" t="s">
         <v>25</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AV1" t="s">
         <v>26</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AW1" t="s">
         <v>27</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AX1" t="s">
         <v>28</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AY1" t="s">
         <v>29</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AZ1" t="s">
         <v>30</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="BA1" t="s">
         <v>31</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="BB1" t="s">
         <v>32</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="BC1" t="s">
         <v>33</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="BD1" t="s">
         <v>34</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="BE1" t="s">
         <v>132</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="BF1" t="s">
         <v>134</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="BG1" t="s">
         <v>135</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="BH1" t="s">
         <v>136</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="BI1" t="s">
         <v>137</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BJ1" t="s">
         <v>35</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BK1" t="s">
         <v>36</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BL1" t="s">
         <v>37</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BM1" t="s">
         <v>38</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BN1" t="s">
         <v>39</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BO1" t="s">
         <v>40</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BP1" t="s">
         <v>41</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BQ1" t="s">
         <v>42</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BR1" t="s">
         <v>43</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BS1" t="s">
         <v>44</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BT1" t="s">
         <v>45</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BU1" t="s">
         <v>46</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BV1" t="s">
         <v>47</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BW1" t="s">
         <v>48</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BX1" t="s">
         <v>49</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BY1" t="s">
         <v>50</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BZ1" t="s">
         <v>51</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="CA1" t="s">
         <v>52</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="CB1" t="s">
         <v>53</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="CC1" t="s">
         <v>54</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="CD1" t="s">
         <v>55</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="CE1" t="s">
         <v>56</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="CF1" t="s">
         <v>57</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="CG1" t="s">
         <v>58</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CH1" t="s">
         <v>59</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CI1" t="s">
         <v>60</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CJ1" t="s">
         <v>61</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CK1" t="s">
         <v>62</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CL1" t="s">
         <v>63</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CM1" t="s">
         <v>64</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CN1" t="s">
         <v>65</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CO1" t="s">
         <v>66</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CP1" t="s">
         <v>67</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CQ1" t="s">
         <v>68</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CR1" t="s">
         <v>69</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CS1" t="s">
         <v>70</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CT1" t="s">
         <v>71</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CU1" t="s">
         <v>72</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CV1" t="s">
         <v>73</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CW1" t="s">
         <v>74</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CX1" t="s">
         <v>75</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CY1" t="s">
         <v>76</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="CZ1" t="s">
         <v>77</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="DA1" t="s">
         <v>78</v>
       </c>
-      <c r="CR1" t="s">
+      <c r="DB1" t="s">
         <v>79</v>
       </c>
-      <c r="CS1" t="s">
+      <c r="DC1" t="s">
         <v>80</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="DD1" t="s">
         <v>81</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="DE1" t="s">
         <v>82</v>
       </c>
-      <c r="CV1" t="s">
+      <c r="DF1" t="s">
         <v>83</v>
       </c>
-      <c r="CW1" t="s">
+      <c r="DG1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:101" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>85</v>
       </c>
@@ -1447,319 +1517,349 @@
         <v>124</v>
       </c>
       <c r="AD2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>124</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>124</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>124</v>
+      </c>
+      <c r="AJ2" t="s">
         <v>106</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AK2" t="s">
+        <v>157</v>
+      </c>
+      <c r="AL2">
+        <v>30122025</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>93</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>161</v>
+      </c>
+      <c r="AO2" t="s">
         <v>94</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AP2" t="s">
         <v>95</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AQ2" t="s">
         <v>96</v>
       </c>
-      <c r="AH2" t="s">
+      <c r="AR2" t="s">
         <v>97</v>
       </c>
-      <c r="AI2" t="s">
+      <c r="AS2" t="s">
         <v>98</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AT2" t="s">
         <v>94</v>
       </c>
-      <c r="AK2" t="s">
+      <c r="AU2" t="s">
         <v>99</v>
       </c>
-      <c r="AL2" t="s">
+      <c r="AV2" t="s">
         <v>100</v>
       </c>
-      <c r="AM2" t="s">
+      <c r="AW2" t="s">
         <v>94</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AX2" t="s">
         <v>101</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AY2" t="s">
         <v>102</v>
       </c>
-      <c r="AP2" t="s">
+      <c r="AZ2" t="s">
         <v>94</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="BA2" t="s">
         <v>103</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="BB2" t="s">
         <v>94</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="BC2" t="s">
         <v>104</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="BD2" t="s">
         <v>105</v>
       </c>
-      <c r="AU2" t="s">
+      <c r="BE2" t="s">
         <v>133</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="BF2" t="s">
         <v>93</v>
       </c>
-      <c r="AW2" t="s">
+      <c r="BG2" t="s">
         <v>93</v>
       </c>
-      <c r="AX2" t="s">
+      <c r="BH2" t="s">
         <v>94</v>
       </c>
-      <c r="AY2" t="s">
+      <c r="BI2" t="s">
         <v>138</v>
       </c>
-      <c r="AZ2" t="s">
+      <c r="BJ2" t="s">
         <v>106</v>
-      </c>
-      <c r="BA2" t="s">
-        <v>94</v>
-      </c>
-      <c r="BB2" t="s">
-        <v>91</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>91</v>
-      </c>
-      <c r="BD2" t="s">
-        <v>94</v>
-      </c>
-      <c r="BE2" t="s">
-        <v>107</v>
-      </c>
-      <c r="BF2" t="s">
-        <v>108</v>
-      </c>
-      <c r="BG2" t="s">
-        <v>91</v>
-      </c>
-      <c r="BH2" t="s">
-        <v>91</v>
-      </c>
-      <c r="BI2" t="s">
-        <v>91</v>
-      </c>
-      <c r="BJ2" t="s">
-        <v>91</v>
       </c>
       <c r="BK2" t="s">
         <v>94</v>
       </c>
       <c r="BL2" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="BM2" t="s">
+        <v>91</v>
+      </c>
+      <c r="BN2" t="s">
         <v>94</v>
       </c>
-      <c r="BN2" t="s">
-        <v>110</v>
-      </c>
       <c r="BO2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="BP2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="BQ2" t="s">
-        <v>112</v>
+        <v>91</v>
       </c>
       <c r="BR2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="BS2" t="s">
-        <v>113</v>
+        <v>91</v>
       </c>
       <c r="BT2" t="s">
-        <v>114</v>
+        <v>91</v>
       </c>
       <c r="BU2" t="s">
         <v>94</v>
       </c>
       <c r="BV2" t="s">
+        <v>109</v>
+      </c>
+      <c r="BW2" t="s">
+        <v>94</v>
+      </c>
+      <c r="BX2" t="s">
+        <v>110</v>
+      </c>
+      <c r="BY2" t="s">
+        <v>110</v>
+      </c>
+      <c r="BZ2" t="s">
+        <v>111</v>
+      </c>
+      <c r="CA2" t="s">
+        <v>112</v>
+      </c>
+      <c r="CB2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CC2" t="s">
+        <v>113</v>
+      </c>
+      <c r="CD2" t="s">
+        <v>114</v>
+      </c>
+      <c r="CE2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CF2" t="s">
         <v>115</v>
       </c>
-      <c r="BW2" t="s">
+      <c r="CG2" t="s">
         <v>116</v>
       </c>
-      <c r="BX2" t="s">
+      <c r="CH2" t="s">
         <v>117</v>
       </c>
-      <c r="BY2" t="s">
+      <c r="CI2" t="s">
         <v>94</v>
       </c>
-      <c r="BZ2" t="s">
+      <c r="CJ2" t="s">
         <v>118</v>
       </c>
-      <c r="CA2" t="s">
+      <c r="CK2" t="s">
         <v>110</v>
       </c>
-      <c r="CB2" t="s">
+      <c r="CL2" t="s">
         <v>109</v>
       </c>
-      <c r="CC2" t="s">
+      <c r="CM2" t="s">
         <v>119</v>
-      </c>
-      <c r="CD2" t="s">
-        <v>94</v>
-      </c>
-      <c r="CE2" t="s">
-        <v>119</v>
-      </c>
-      <c r="CF2" t="s">
-        <v>120</v>
-      </c>
-      <c r="CG2" t="s">
-        <v>94</v>
-      </c>
-      <c r="CH2" t="s">
-        <v>93</v>
-      </c>
-      <c r="CI2" t="s">
-        <v>121</v>
-      </c>
-      <c r="CJ2" t="s">
-        <v>94</v>
-      </c>
-      <c r="CK2" t="s">
-        <v>122</v>
-      </c>
-      <c r="CL2" t="s">
-        <v>123</v>
-      </c>
-      <c r="CM2" t="s">
-        <v>124</v>
       </c>
       <c r="CN2" t="s">
         <v>94</v>
       </c>
       <c r="CO2" t="s">
+        <v>119</v>
+      </c>
+      <c r="CP2" t="s">
+        <v>120</v>
+      </c>
+      <c r="CQ2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CR2" t="s">
+        <v>93</v>
+      </c>
+      <c r="CS2" t="s">
+        <v>121</v>
+      </c>
+      <c r="CT2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CU2" t="s">
+        <v>122</v>
+      </c>
+      <c r="CV2" t="s">
+        <v>123</v>
+      </c>
+      <c r="CW2" t="s">
+        <v>124</v>
+      </c>
+      <c r="CX2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CY2" t="s">
         <v>125</v>
       </c>
-      <c r="CP2" t="s">
+      <c r="CZ2" t="s">
         <v>126</v>
       </c>
-      <c r="CQ2" t="s">
+      <c r="DA2" t="s">
         <v>127</v>
       </c>
-      <c r="CR2" t="s">
+      <c r="DB2" t="s">
         <v>128</v>
       </c>
-      <c r="CS2" t="s">
+      <c r="DC2" t="s">
         <v>129</v>
       </c>
-      <c r="CT2" t="s">
+      <c r="DD2" t="s">
         <v>130</v>
       </c>
-      <c r="CU2" t="s">
+      <c r="DE2" t="s">
         <v>131</v>
       </c>
-      <c r="CV2" t="s">
+      <c r="DF2" t="s">
         <v>93</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="41">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2 O2:S2 BG2:BJ2 BB2:BC2 AZ2 Z2 AD2" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="44">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2 O2:S2 BQ2:BT2 BL2:BM2 BJ2 Z2 AD2 AF2 AH2 AJ2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2 CU2 CR2" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AE2 AJ2 AM2 AP2 AR2 AX2 BA2 BD2 BK2 BM2 BR2 BU2 BY2 CD2 CG2 CJ2 CN2" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2 DE2 DB2" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2 AT2 AW2 AZ2 BB2 BH2 BK2 BN2 BU2 BW2 CB2 CE2 CI2 CN2 CQ2 CT2 CX2" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AF2" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AP2" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AG2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH2" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AR2" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AY2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BA2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AS2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BC2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AT2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BD2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Sesuai Umur,Ada kemungkinan penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BF2" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW2" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BG2" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Normal,Curiga kelainan pupil putih pada anak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BF2" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BV2" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BW2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CU2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CW2" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CY2" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CZ2" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DA2" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DC2" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DD2" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DF2" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{00000000-0002-0000-0000-000027000000}">
@@ -1771,7 +1871,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"Perkembangan sesuai usia,Perkembangan meragukan,Perkembangan curiga adanya penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2" xr:uid="{8CF71D70-E85F-9946-A33A-2D9580913A62}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AS2" xr:uid="{8CF71D70-E85F-9946-A33A-2D9580913A62}">
       <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
         <mc:Choice Requires="x12ac">
           <x12ac:list>Mtb not detected (Neg),"Mtb detected, Rif resistance not detected (Rif Sen)","Mtb detected, Rif resistance detected (Rif Res)","MTB detected, Rif Resistance Indeterminate (Rif Indet)",Invalid,Error,No Result</x12ac:list>
@@ -1781,14 +1881,23 @@
         </mc:Fallback>
       </mc:AlternateContent>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AY2" xr:uid="{6581135A-9ACF-CC48-9D5E-ECD150302CDE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2" xr:uid="{6581135A-9ACF-CC48-9D5E-ECD150302CDE}">
       <formula1>"Tidak ada,1,2,3,&gt;3"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2" xr:uid="{C8F9D09B-6ED1-1641-81FF-EFC972969A8B}">
       <formula1>"Sudah,Belum"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA2:AC2" xr:uid="{8053A0D4-04B2-4C40-B539-974DDB07ADD7}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA2:AC2 AE2 AG2 AI2" xr:uid="{8053A0D4-04B2-4C40-B539-974DDB07ADD7}">
       <formula1>"Positif,Negatif"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2" xr:uid="{268DC933-A25C-DE45-9BA6-2A40B37E78EB}">
+      <formula1>"Normal,Bayi Kuning Kramer 1-3,Bayi Kuning Kramer &gt;3"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM2" xr:uid="{CB08F77E-49BC-544C-8574-4FEDEA492356}">
+      <formula1>"Normal,Bayi Kuning Kramer 1,Bayi Kuning Kramer 2,Bayi Kuning Kramer 3,Bayi Kuning Kramer 4,Bayi Kuning Kramer 5"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2" xr:uid="{D7812175-EA41-8345-9FD2-DBDE71A78328}">
+      <formula1>"&gt;3 Normal,&lt;=3 Pucat"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
wip risiko gula darah anak
</commit_message>
<xml_diff>
--- a/dataset/anak.xlsx
+++ b/dataset/anak.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFC5F5B1-DBF2-C54E-B461-FF8CD7436F9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAA99FB2-B904-A041-B1F2-517DE9579951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="19520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,172 @@
     <author>Microsoft Office User</author>
   </authors>
   <commentList>
-    <comment ref="T1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{4E68458D-00F6-2449-BE73-7974FEBDE11C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Microsoft Office User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>diisi jika pernah_kencing_manis Ya</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{FBAFFD93-F95D-C44F-BE39-B9E95005DE70}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Microsoft Office User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>diisi jika pernah_kencing_manis Tidak</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{E7636830-21DF-9D4C-945F-544CF8F76894}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Microsoft Office User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>diisi jika pernah_kencing_manis Tidak</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{1763EDAD-7DCB-CD41-827C-6BBEF78B6BD3}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Microsoft Office User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>diisi jika pernah_kencing_manis Tidak</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0" xr:uid="{99F7BF8B-E64C-4F4E-9536-282AF2583775}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Microsoft Office User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>diisi jika pernah_kencing_manis Tidak</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -40,7 +205,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AQ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="AV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -55,7 +220,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AV1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="BA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -70,7 +235,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AY1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="BD1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -85,7 +250,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BP1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="BU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -100,7 +265,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CH1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="CM1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -120,7 +285,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="169">
   <si>
     <t>batas_awal</t>
   </si>
@@ -606,13 +771,34 @@
   </si>
   <si>
     <t>&gt;3 Normal</t>
+  </si>
+  <si>
+    <t>AFIFUDDIN MUHAJIR</t>
+  </si>
+  <si>
+    <t>pernah_kencing_manis</t>
+  </si>
+  <si>
+    <t>berapa_bulan_diabetes</t>
+  </si>
+  <si>
+    <t>sering_lapar</t>
+  </si>
+  <si>
+    <t>sering_haus</t>
+  </si>
+  <si>
+    <t>penurunan_berat_badan</t>
+  </si>
+  <si>
+    <t>anggota_keluarga_diabetes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -626,6 +812,25 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF343434"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -670,9 +875,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Dark Mode" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -1008,7 +1214,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:DG2"/>
+  <dimension ref="A1:DL3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -1016,93 +1222,95 @@
     <col min="3" max="3" width="11.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.83203125" customWidth="1"/>
-    <col min="7" max="8" width="14.33203125" customWidth="1"/>
-    <col min="9" max="9" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="19" customWidth="1"/>
-    <col min="14" max="14" width="25" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.83203125" customWidth="1"/>
-    <col min="21" max="21" width="28.83203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="13.6640625" customWidth="1"/>
-    <col min="27" max="27" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="28" max="29" width="13.6640625" customWidth="1"/>
-    <col min="30" max="30" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="31" max="35" width="22.5" customWidth="1"/>
-    <col min="36" max="36" width="35.83203125" bestFit="1" customWidth="1"/>
-    <col min="37" max="40" width="22.5" customWidth="1"/>
-    <col min="41" max="41" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="22.83203125" customWidth="1"/>
-    <col min="46" max="46" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="16.1640625" customWidth="1"/>
-    <col min="48" max="48" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="50" max="51" width="12.33203125" customWidth="1"/>
-    <col min="52" max="52" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="14.1640625" customWidth="1"/>
-    <col min="54" max="54" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="23.6640625" customWidth="1"/>
-    <col min="57" max="57" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="12.83203125" customWidth="1"/>
-    <col min="63" max="63" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="17.5" customWidth="1"/>
-    <col min="66" max="66" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="13" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="70" max="72" width="19.5" customWidth="1"/>
-    <col min="73" max="73" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="9.83203125" customWidth="1"/>
-    <col min="75" max="75" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="76" max="79" width="11.5" customWidth="1"/>
-    <col min="80" max="80" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="9" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="16.1640625" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="18.1640625" customWidth="1"/>
-    <col min="87" max="87" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="89" max="91" width="8.33203125" customWidth="1"/>
-    <col min="92" max="92" width="22" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="14" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="14" customWidth="1"/>
-    <col min="97" max="97" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="18.1640625" customWidth="1"/>
-    <col min="100" max="100" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="103" max="105" width="18.1640625" customWidth="1"/>
-    <col min="106" max="106" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="35" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="43.1640625" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="18.1640625" customWidth="1"/>
-    <col min="110" max="110" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="11" width="13.83203125" customWidth="1"/>
+    <col min="12" max="13" width="14.33203125" customWidth="1"/>
+    <col min="14" max="14" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19" bestFit="1" customWidth="1"/>
+    <col min="16" max="18" width="19" customWidth="1"/>
+    <col min="19" max="19" width="25" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="14.83203125" customWidth="1"/>
+    <col min="26" max="26" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="16" bestFit="1" customWidth="1"/>
+    <col min="30" max="31" width="13.6640625" customWidth="1"/>
+    <col min="32" max="32" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="34" width="13.6640625" customWidth="1"/>
+    <col min="35" max="35" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="36" max="40" width="22.5" customWidth="1"/>
+    <col min="41" max="41" width="35.83203125" bestFit="1" customWidth="1"/>
+    <col min="42" max="45" width="22.5" customWidth="1"/>
+    <col min="46" max="46" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="22.83203125" customWidth="1"/>
+    <col min="51" max="51" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="16.1640625" customWidth="1"/>
+    <col min="53" max="53" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="55" max="56" width="12.33203125" customWidth="1"/>
+    <col min="57" max="57" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="14.1640625" customWidth="1"/>
+    <col min="59" max="59" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="23.6640625" customWidth="1"/>
+    <col min="62" max="62" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="12.83203125" customWidth="1"/>
+    <col min="68" max="68" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="17.5" customWidth="1"/>
+    <col min="71" max="71" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="13" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="75" max="77" width="19.5" customWidth="1"/>
+    <col min="78" max="78" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="9.83203125" customWidth="1"/>
+    <col min="80" max="80" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="81" max="84" width="11.5" customWidth="1"/>
+    <col min="85" max="85" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="9" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="18.1640625" customWidth="1"/>
+    <col min="92" max="92" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="94" max="96" width="8.33203125" customWidth="1"/>
+    <col min="97" max="97" width="22" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="14" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="14" customWidth="1"/>
+    <col min="102" max="102" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="18.1640625" customWidth="1"/>
+    <col min="105" max="105" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="108" max="110" width="18.1640625" customWidth="1"/>
+    <col min="111" max="111" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="35" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="18.1640625" customWidth="1"/>
+    <col min="115" max="115" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="116" max="116" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:111" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:116" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1118,323 +1326,341 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>163</v>
+      </c>
       <c r="G1" t="s">
+        <v>164</v>
+      </c>
+      <c r="H1" t="s">
+        <v>165</v>
+      </c>
+      <c r="I1" t="s">
+        <v>166</v>
+      </c>
+      <c r="J1" t="s">
+        <v>167</v>
+      </c>
+      <c r="K1" t="s">
+        <v>168</v>
+      </c>
+      <c r="L1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="M1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="N1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="O1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+      <c r="P1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="Q1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" t="s">
+      <c r="R1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" t="s">
+      <c r="S1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" t="s">
+      <c r="T1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" t="s">
+      <c r="U1" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="V1" t="s">
         <v>15</v>
       </c>
-      <c r="R1" t="s">
+      <c r="W1" t="s">
         <v>16</v>
       </c>
-      <c r="S1" t="s">
+      <c r="X1" t="s">
         <v>17</v>
       </c>
-      <c r="T1" t="s">
+      <c r="Y1" t="s">
         <v>18</v>
       </c>
-      <c r="U1" t="s">
+      <c r="Z1" t="s">
         <v>139</v>
       </c>
-      <c r="V1" t="s">
+      <c r="AA1" t="s">
         <v>141</v>
       </c>
-      <c r="W1" t="s">
+      <c r="AB1" t="s">
         <v>142</v>
       </c>
-      <c r="X1" t="s">
+      <c r="AC1" t="s">
         <v>143</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="AD1" t="s">
         <v>144</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AE1" t="s">
         <v>145</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AF1" t="s">
         <v>146</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AG1" t="s">
         <v>147</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AH1" t="s">
         <v>148</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AI1" t="s">
         <v>149</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AJ1" t="s">
         <v>150</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AK1" t="s">
         <v>151</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AL1" t="s">
         <v>152</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AM1" t="s">
         <v>153</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AN1" t="s">
         <v>154</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AO1" t="s">
         <v>155</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AP1" t="s">
         <v>156</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AQ1" t="s">
         <v>158</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AR1" t="s">
         <v>159</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AS1" t="s">
         <v>160</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AT1" t="s">
         <v>19</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AU1" t="s">
         <v>20</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AV1" t="s">
         <v>21</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AW1" t="s">
         <v>22</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AX1" t="s">
         <v>23</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AY1" t="s">
         <v>24</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AZ1" t="s">
         <v>25</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="BA1" t="s">
         <v>26</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="BB1" t="s">
         <v>27</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="BC1" t="s">
         <v>28</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="BD1" t="s">
         <v>29</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BE1" t="s">
         <v>30</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BF1" t="s">
         <v>31</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BG1" t="s">
         <v>32</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BH1" t="s">
         <v>33</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BI1" t="s">
         <v>34</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BJ1" t="s">
         <v>132</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BK1" t="s">
         <v>134</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BL1" t="s">
         <v>135</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BM1" t="s">
         <v>136</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BN1" t="s">
         <v>137</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BO1" t="s">
         <v>35</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BP1" t="s">
         <v>36</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BQ1" t="s">
         <v>37</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BR1" t="s">
         <v>38</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BS1" t="s">
         <v>39</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BT1" t="s">
         <v>40</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BU1" t="s">
         <v>41</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BV1" t="s">
         <v>42</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BW1" t="s">
         <v>43</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BX1" t="s">
         <v>44</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BY1" t="s">
         <v>45</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BZ1" t="s">
         <v>46</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="CA1" t="s">
         <v>47</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="CB1" t="s">
         <v>48</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CC1" t="s">
         <v>49</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CD1" t="s">
         <v>50</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CE1" t="s">
         <v>51</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CF1" t="s">
         <v>52</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CG1" t="s">
         <v>53</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CH1" t="s">
         <v>54</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CI1" t="s">
         <v>55</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CJ1" t="s">
         <v>56</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CK1" t="s">
         <v>57</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CL1" t="s">
         <v>58</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CM1" t="s">
         <v>59</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CN1" t="s">
         <v>60</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CO1" t="s">
         <v>61</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CP1" t="s">
         <v>62</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CQ1" t="s">
         <v>63</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CR1" t="s">
         <v>64</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CS1" t="s">
         <v>65</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CT1" t="s">
         <v>66</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="CU1" t="s">
         <v>67</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="CV1" t="s">
         <v>68</v>
       </c>
-      <c r="CR1" t="s">
+      <c r="CW1" t="s">
         <v>69</v>
       </c>
-      <c r="CS1" t="s">
+      <c r="CX1" t="s">
         <v>70</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="CY1" t="s">
         <v>71</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="CZ1" t="s">
         <v>72</v>
       </c>
-      <c r="CV1" t="s">
+      <c r="DA1" t="s">
         <v>73</v>
       </c>
-      <c r="CW1" t="s">
+      <c r="DB1" t="s">
         <v>74</v>
       </c>
-      <c r="CX1" t="s">
+      <c r="DC1" t="s">
         <v>75</v>
       </c>
-      <c r="CY1" t="s">
+      <c r="DD1" t="s">
         <v>76</v>
       </c>
-      <c r="CZ1" t="s">
+      <c r="DE1" t="s">
         <v>77</v>
       </c>
-      <c r="DA1" t="s">
+      <c r="DF1" t="s">
         <v>78</v>
       </c>
-      <c r="DB1" t="s">
+      <c r="DG1" t="s">
         <v>79</v>
       </c>
-      <c r="DC1" t="s">
+      <c r="DH1" t="s">
         <v>80</v>
       </c>
-      <c r="DD1" t="s">
+      <c r="DI1" t="s">
         <v>81</v>
       </c>
-      <c r="DE1" t="s">
+      <c r="DJ1" t="s">
         <v>82</v>
       </c>
-      <c r="DF1" t="s">
+      <c r="DK1" t="s">
         <v>83</v>
       </c>
-      <c r="DG1" t="s">
+      <c r="DL1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:111" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:116" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>85</v>
       </c>
@@ -1447,431 +1673,787 @@
       <c r="E2" t="s">
         <v>88</v>
       </c>
-      <c r="G2">
+      <c r="F2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H2" t="s">
+        <v>106</v>
+      </c>
+      <c r="I2" t="s">
+        <v>106</v>
+      </c>
+      <c r="J2" t="s">
+        <v>106</v>
+      </c>
+      <c r="K2" t="s">
+        <v>106</v>
+      </c>
+      <c r="L2">
         <v>30</v>
       </c>
-      <c r="H2">
+      <c r="M2">
         <v>100</v>
       </c>
-      <c r="I2" t="s">
+      <c r="N2" t="s">
         <v>89</v>
       </c>
-      <c r="J2" t="s">
+      <c r="O2" t="s">
         <v>93</v>
       </c>
-      <c r="K2" t="s">
+      <c r="P2" t="s">
         <v>90</v>
       </c>
-      <c r="L2" t="s">
-        <v>91</v>
-      </c>
-      <c r="M2">
+      <c r="Q2" t="s">
+        <v>91</v>
+      </c>
+      <c r="R2">
         <v>10</v>
       </c>
-      <c r="N2" t="s">
+      <c r="S2" t="s">
         <v>92</v>
       </c>
-      <c r="O2" t="s">
-        <v>91</v>
-      </c>
-      <c r="P2" t="s">
-        <v>91</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>91</v>
-      </c>
-      <c r="R2" t="s">
-        <v>91</v>
-      </c>
-      <c r="S2" t="s">
-        <v>91</v>
-      </c>
       <c r="T2" t="s">
+        <v>91</v>
+      </c>
+      <c r="U2" t="s">
+        <v>91</v>
+      </c>
+      <c r="V2" t="s">
+        <v>91</v>
+      </c>
+      <c r="W2" t="s">
+        <v>91</v>
+      </c>
+      <c r="X2" t="s">
+        <v>91</v>
+      </c>
+      <c r="Y2" t="s">
         <v>93</v>
       </c>
-      <c r="U2" t="s">
+      <c r="Z2" t="s">
         <v>140</v>
       </c>
-      <c r="V2">
+      <c r="AA2">
         <v>2900</v>
       </c>
-      <c r="W2">
+      <c r="AB2">
         <v>6000</v>
       </c>
-      <c r="X2">
+      <c r="AC2">
         <v>80</v>
       </c>
-      <c r="Y2">
+      <c r="AD2">
         <v>90</v>
       </c>
-      <c r="Z2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AA2" t="s">
+      <c r="AE2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AF2" t="s">
         <v>124</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>124</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>124</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>124</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>91</v>
       </c>
       <c r="AG2" t="s">
         <v>124</v>
       </c>
       <c r="AH2" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="AI2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AJ2" t="s">
         <v>124</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AK2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>124</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>124</v>
+      </c>
+      <c r="AO2" t="s">
         <v>106</v>
       </c>
-      <c r="AK2" t="s">
+      <c r="AP2" t="s">
         <v>157</v>
       </c>
-      <c r="AL2">
+      <c r="AQ2">
         <v>30122025</v>
       </c>
-      <c r="AM2" t="s">
+      <c r="AR2" t="s">
         <v>93</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AS2" t="s">
         <v>161</v>
       </c>
-      <c r="AO2" t="s">
-        <v>94</v>
-      </c>
-      <c r="AP2" t="s">
+      <c r="AT2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AU2" t="s">
         <v>95</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="AV2" t="s">
         <v>96</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="AW2" t="s">
         <v>97</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AX2" t="s">
         <v>98</v>
       </c>
-      <c r="AT2" t="s">
-        <v>94</v>
-      </c>
-      <c r="AU2" t="s">
+      <c r="AY2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AZ2" t="s">
         <v>99</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="BA2" t="s">
         <v>100</v>
       </c>
-      <c r="AW2" t="s">
-        <v>94</v>
-      </c>
-      <c r="AX2" t="s">
+      <c r="BB2" t="s">
+        <v>94</v>
+      </c>
+      <c r="BC2" t="s">
         <v>101</v>
       </c>
-      <c r="AY2" t="s">
+      <c r="BD2" t="s">
         <v>102</v>
       </c>
-      <c r="AZ2" t="s">
-        <v>94</v>
-      </c>
-      <c r="BA2" t="s">
+      <c r="BE2" t="s">
+        <v>94</v>
+      </c>
+      <c r="BF2" t="s">
         <v>103</v>
       </c>
-      <c r="BB2" t="s">
-        <v>94</v>
-      </c>
-      <c r="BC2" t="s">
+      <c r="BG2" t="s">
+        <v>94</v>
+      </c>
+      <c r="BH2" t="s">
         <v>104</v>
       </c>
-      <c r="BD2" t="s">
+      <c r="BI2" t="s">
         <v>105</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BJ2" t="s">
         <v>133</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BK2" t="s">
         <v>93</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BL2" t="s">
         <v>93</v>
       </c>
-      <c r="BH2" t="s">
-        <v>94</v>
-      </c>
-      <c r="BI2" t="s">
+      <c r="BM2" t="s">
+        <v>94</v>
+      </c>
+      <c r="BN2" t="s">
         <v>138</v>
       </c>
-      <c r="BJ2" t="s">
+      <c r="BO2" t="s">
         <v>106</v>
       </c>
-      <c r="BK2" t="s">
-        <v>94</v>
-      </c>
-      <c r="BL2" t="s">
-        <v>91</v>
-      </c>
-      <c r="BM2" t="s">
-        <v>91</v>
-      </c>
-      <c r="BN2" t="s">
-        <v>94</v>
-      </c>
-      <c r="BO2" t="s">
+      <c r="BP2" t="s">
+        <v>94</v>
+      </c>
+      <c r="BQ2" t="s">
+        <v>91</v>
+      </c>
+      <c r="BR2" t="s">
+        <v>91</v>
+      </c>
+      <c r="BS2" t="s">
+        <v>94</v>
+      </c>
+      <c r="BT2" t="s">
         <v>107</v>
       </c>
-      <c r="BP2" t="s">
+      <c r="BU2" t="s">
         <v>108</v>
       </c>
-      <c r="BQ2" t="s">
-        <v>91</v>
-      </c>
-      <c r="BR2" t="s">
-        <v>91</v>
-      </c>
-      <c r="BS2" t="s">
-        <v>91</v>
-      </c>
-      <c r="BT2" t="s">
-        <v>91</v>
-      </c>
-      <c r="BU2" t="s">
-        <v>94</v>
-      </c>
       <c r="BV2" t="s">
+        <v>91</v>
+      </c>
+      <c r="BW2" t="s">
+        <v>91</v>
+      </c>
+      <c r="BX2" t="s">
+        <v>91</v>
+      </c>
+      <c r="BY2" t="s">
+        <v>91</v>
+      </c>
+      <c r="BZ2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CA2" t="s">
         <v>109</v>
       </c>
-      <c r="BW2" t="s">
-        <v>94</v>
-      </c>
-      <c r="BX2" t="s">
+      <c r="CB2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CC2" t="s">
         <v>110</v>
       </c>
-      <c r="BY2" t="s">
+      <c r="CD2" t="s">
         <v>110</v>
       </c>
-      <c r="BZ2" t="s">
+      <c r="CE2" t="s">
         <v>111</v>
       </c>
-      <c r="CA2" t="s">
+      <c r="CF2" t="s">
         <v>112</v>
       </c>
-      <c r="CB2" t="s">
-        <v>94</v>
-      </c>
-      <c r="CC2" t="s">
+      <c r="CG2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CH2" t="s">
         <v>113</v>
       </c>
-      <c r="CD2" t="s">
+      <c r="CI2" t="s">
         <v>114</v>
       </c>
-      <c r="CE2" t="s">
-        <v>94</v>
-      </c>
-      <c r="CF2" t="s">
+      <c r="CJ2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CK2" t="s">
         <v>115</v>
       </c>
-      <c r="CG2" t="s">
+      <c r="CL2" t="s">
         <v>116</v>
       </c>
-      <c r="CH2" t="s">
+      <c r="CM2" t="s">
         <v>117</v>
       </c>
-      <c r="CI2" t="s">
-        <v>94</v>
-      </c>
-      <c r="CJ2" t="s">
+      <c r="CN2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CO2" t="s">
         <v>118</v>
       </c>
-      <c r="CK2" t="s">
+      <c r="CP2" t="s">
         <v>110</v>
       </c>
-      <c r="CL2" t="s">
+      <c r="CQ2" t="s">
         <v>109</v>
       </c>
-      <c r="CM2" t="s">
+      <c r="CR2" t="s">
         <v>119</v>
       </c>
-      <c r="CN2" t="s">
-        <v>94</v>
-      </c>
-      <c r="CO2" t="s">
+      <c r="CS2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CT2" t="s">
         <v>119</v>
       </c>
-      <c r="CP2" t="s">
+      <c r="CU2" t="s">
         <v>120</v>
       </c>
-      <c r="CQ2" t="s">
-        <v>94</v>
-      </c>
-      <c r="CR2" t="s">
+      <c r="CV2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CW2" t="s">
         <v>93</v>
       </c>
-      <c r="CS2" t="s">
+      <c r="CX2" t="s">
         <v>121</v>
       </c>
-      <c r="CT2" t="s">
-        <v>94</v>
-      </c>
-      <c r="CU2" t="s">
+      <c r="CY2" t="s">
+        <v>94</v>
+      </c>
+      <c r="CZ2" t="s">
         <v>122</v>
       </c>
-      <c r="CV2" t="s">
+      <c r="DA2" t="s">
         <v>123</v>
       </c>
-      <c r="CW2" t="s">
+      <c r="DB2" t="s">
         <v>124</v>
       </c>
-      <c r="CX2" t="s">
-        <v>94</v>
-      </c>
-      <c r="CY2" t="s">
+      <c r="DC2" t="s">
+        <v>94</v>
+      </c>
+      <c r="DD2" t="s">
         <v>125</v>
       </c>
-      <c r="CZ2" t="s">
+      <c r="DE2" t="s">
         <v>126</v>
       </c>
-      <c r="DA2" t="s">
+      <c r="DF2" t="s">
         <v>127</v>
       </c>
-      <c r="DB2" t="s">
+      <c r="DG2" t="s">
         <v>128</v>
       </c>
-      <c r="DC2" t="s">
+      <c r="DH2" t="s">
         <v>129</v>
       </c>
-      <c r="DD2" t="s">
+      <c r="DI2" t="s">
         <v>130</v>
       </c>
-      <c r="DE2" t="s">
+      <c r="DJ2" t="s">
         <v>131</v>
       </c>
-      <c r="DF2" t="s">
+      <c r="DK2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:116" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="E3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F3" t="s">
+        <v>106</v>
+      </c>
+      <c r="H3" t="s">
+        <v>106</v>
+      </c>
+      <c r="I3" t="s">
+        <v>106</v>
+      </c>
+      <c r="J3" t="s">
+        <v>106</v>
+      </c>
+      <c r="K3" t="s">
+        <v>106</v>
+      </c>
+      <c r="L3">
+        <v>30</v>
+      </c>
+      <c r="M3">
+        <v>100</v>
+      </c>
+      <c r="N3" t="s">
+        <v>89</v>
+      </c>
+      <c r="O3" t="s">
+        <v>93</v>
+      </c>
+      <c r="P3" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>91</v>
+      </c>
+      <c r="R3">
+        <v>10</v>
+      </c>
+      <c r="S3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T3" t="s">
+        <v>91</v>
+      </c>
+      <c r="U3" t="s">
+        <v>91</v>
+      </c>
+      <c r="V3" t="s">
+        <v>91</v>
+      </c>
+      <c r="W3" t="s">
+        <v>91</v>
+      </c>
+      <c r="X3" t="s">
+        <v>91</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>93</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>140</v>
+      </c>
+      <c r="AA3">
+        <v>2900</v>
+      </c>
+      <c r="AB3">
+        <v>6000</v>
+      </c>
+      <c r="AC3">
+        <v>80</v>
+      </c>
+      <c r="AD3">
+        <v>90</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>91</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>91</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>91</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>91</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>106</v>
+      </c>
+      <c r="AP3" t="s">
+        <v>157</v>
+      </c>
+      <c r="AQ3">
+        <v>30122025</v>
+      </c>
+      <c r="AR3" t="s">
+        <v>93</v>
+      </c>
+      <c r="AS3" t="s">
+        <v>161</v>
+      </c>
+      <c r="AT3" t="s">
+        <v>94</v>
+      </c>
+      <c r="AU3" t="s">
+        <v>95</v>
+      </c>
+      <c r="AV3" t="s">
+        <v>96</v>
+      </c>
+      <c r="AW3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AX3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AY3" t="s">
+        <v>94</v>
+      </c>
+      <c r="AZ3" t="s">
+        <v>99</v>
+      </c>
+      <c r="BA3" t="s">
+        <v>100</v>
+      </c>
+      <c r="BB3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BC3" t="s">
+        <v>101</v>
+      </c>
+      <c r="BD3" t="s">
+        <v>102</v>
+      </c>
+      <c r="BE3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BF3" t="s">
+        <v>103</v>
+      </c>
+      <c r="BG3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BH3" t="s">
+        <v>104</v>
+      </c>
+      <c r="BI3" t="s">
+        <v>105</v>
+      </c>
+      <c r="BJ3" t="s">
+        <v>133</v>
+      </c>
+      <c r="BK3" t="s">
+        <v>93</v>
+      </c>
+      <c r="BL3" t="s">
+        <v>93</v>
+      </c>
+      <c r="BM3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BN3" t="s">
+        <v>138</v>
+      </c>
+      <c r="BO3" t="s">
+        <v>106</v>
+      </c>
+      <c r="BP3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BQ3" t="s">
+        <v>91</v>
+      </c>
+      <c r="BR3" t="s">
+        <v>91</v>
+      </c>
+      <c r="BS3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BT3" t="s">
+        <v>107</v>
+      </c>
+      <c r="BU3" t="s">
+        <v>108</v>
+      </c>
+      <c r="BV3" t="s">
+        <v>91</v>
+      </c>
+      <c r="BW3" t="s">
+        <v>91</v>
+      </c>
+      <c r="BX3" t="s">
+        <v>91</v>
+      </c>
+      <c r="BY3" t="s">
+        <v>91</v>
+      </c>
+      <c r="BZ3" t="s">
+        <v>94</v>
+      </c>
+      <c r="CA3" t="s">
+        <v>109</v>
+      </c>
+      <c r="CB3" t="s">
+        <v>94</v>
+      </c>
+      <c r="CC3" t="s">
+        <v>110</v>
+      </c>
+      <c r="CD3" t="s">
+        <v>110</v>
+      </c>
+      <c r="CE3" t="s">
+        <v>111</v>
+      </c>
+      <c r="CF3" t="s">
+        <v>112</v>
+      </c>
+      <c r="CG3" t="s">
+        <v>94</v>
+      </c>
+      <c r="CH3" t="s">
+        <v>113</v>
+      </c>
+      <c r="CI3" t="s">
+        <v>114</v>
+      </c>
+      <c r="CJ3" t="s">
+        <v>94</v>
+      </c>
+      <c r="CK3" t="s">
+        <v>115</v>
+      </c>
+      <c r="CL3" t="s">
+        <v>116</v>
+      </c>
+      <c r="CM3" t="s">
+        <v>117</v>
+      </c>
+      <c r="CN3" t="s">
+        <v>94</v>
+      </c>
+      <c r="CO3" t="s">
+        <v>118</v>
+      </c>
+      <c r="CP3" t="s">
+        <v>110</v>
+      </c>
+      <c r="CQ3" t="s">
+        <v>109</v>
+      </c>
+      <c r="CR3" t="s">
+        <v>119</v>
+      </c>
+      <c r="CS3" t="s">
+        <v>94</v>
+      </c>
+      <c r="CT3" t="s">
+        <v>119</v>
+      </c>
+      <c r="CU3" t="s">
+        <v>120</v>
+      </c>
+      <c r="CV3" t="s">
+        <v>94</v>
+      </c>
+      <c r="CW3" t="s">
+        <v>93</v>
+      </c>
+      <c r="CX3" t="s">
+        <v>121</v>
+      </c>
+      <c r="CY3" t="s">
+        <v>94</v>
+      </c>
+      <c r="CZ3" t="s">
+        <v>122</v>
+      </c>
+      <c r="DA3" t="s">
+        <v>123</v>
+      </c>
+      <c r="DB3" t="s">
+        <v>124</v>
+      </c>
+      <c r="DC3" t="s">
+        <v>94</v>
+      </c>
+      <c r="DD3" t="s">
+        <v>125</v>
+      </c>
+      <c r="DE3" t="s">
+        <v>126</v>
+      </c>
+      <c r="DF3" t="s">
+        <v>127</v>
+      </c>
+      <c r="DG3" t="s">
+        <v>128</v>
+      </c>
+      <c r="DH3" t="s">
+        <v>129</v>
+      </c>
+      <c r="DI3" t="s">
+        <v>130</v>
+      </c>
+      <c r="DJ3" t="s">
+        <v>131</v>
+      </c>
+      <c r="DK3" t="s">
         <v>93</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="44">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2 O2:S2 BQ2:BT2 BL2:BM2 BJ2 Z2 AD2 AF2 AH2 AJ2" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q3 T2:X3 BV2:BY3 BQ2:BR3 BO2:BO3 AE2:AE3 AI2:AI3 AK2:AK3 AM2:AM3 AO2:AO3 F2:F3" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E3" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2 DE2 DB2" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2 AT2 AW2 AZ2 BB2 BH2 BK2 BN2 BU2 BW2 CB2 CE2 CI2 CN2 CQ2 CT2 CX2" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S3 DJ2:DJ3 DG2:DG3" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AT2:AT3 AY2:AY3 BB2:BB3 BE2:BE3 BG2:BG3 BM2:BM3 BP2:BP3 BS2:BS3 BZ2:BZ3 CB2:CB3 CG2:CG3 CJ2:CJ3 CN2:CN3 CS2:CS3 CV2:CV3 CY2:CY3 DC2:DC3" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y2:Y3" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AP2" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2:AU3" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2:AV3" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AR2" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW2:AW3" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AZ2:AZ3" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BA2:BA3" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX2" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BC2:BC3" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AY2" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BD2:BD3" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BA2" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BF2:BF3" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BC2" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH2:BH3" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BD2" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2:BI3" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BE2" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BJ2:BJ3" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Sesuai Umur,Ada kemungkinan penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BF2" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BK2:BK3" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BG2" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2:BL3" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Normal,Curiga kelainan pupil putih pada anak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BT2:BT3 H2:K3" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU2:BU3" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2:CK3" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2:CL3" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2:CM3" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CW2:CW3" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CX2:CX3" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CU2" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CZ2:CZ3" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DA2:DA3" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CW2" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DB2:DB3" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CY2" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DD2:DD3" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CZ2" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DE2:DE3" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DA2" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DF2:DF3" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DC2" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DH2:DH3" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DD2" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DI2:DI3" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DF2" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DK2:DK3" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{00000000-0002-0000-0000-000027000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N3" xr:uid="{00000000-0002-0000-0000-000027000000}">
       <formula1>"Berdiri,Telentang"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2" xr:uid="{00000000-0002-0000-0000-000028000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O3" xr:uid="{00000000-0002-0000-0000-000028000000}">
       <formula1>"Makrosefali,Normal,Mikrosefali"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2" xr:uid="{00000000-0002-0000-0000-000029000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P3" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"Perkembangan sesuai usia,Perkembangan meragukan,Perkembangan curiga adanya penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AS2" xr:uid="{8CF71D70-E85F-9946-A33A-2D9580913A62}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX2:AX3" xr:uid="{8CF71D70-E85F-9946-A33A-2D9580913A62}">
       <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
         <mc:Choice Requires="x12ac">
           <x12ac:list>Mtb not detected (Neg),"Mtb detected, Rif resistance not detected (Rif Sen)","Mtb detected, Rif resistance detected (Rif Res)","MTB detected, Rif Resistance Indeterminate (Rif Indet)",Invalid,Error,No Result</x12ac:list>
@@ -1881,22 +2463,22 @@
         </mc:Fallback>
       </mc:AlternateContent>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2" xr:uid="{6581135A-9ACF-CC48-9D5E-ECD150302CDE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BN2:BN3" xr:uid="{6581135A-9ACF-CC48-9D5E-ECD150302CDE}">
       <formula1>"Tidak ada,1,2,3,&gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2" xr:uid="{C8F9D09B-6ED1-1641-81FF-EFC972969A8B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Z2:Z3" xr:uid="{C8F9D09B-6ED1-1641-81FF-EFC972969A8B}">
       <formula1>"Sudah,Belum"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA2:AC2 AE2 AG2 AI2" xr:uid="{8053A0D4-04B2-4C40-B539-974DDB07ADD7}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AF2:AH3 AJ2:AJ3 AL2:AL3 AN2:AN3" xr:uid="{8053A0D4-04B2-4C40-B539-974DDB07ADD7}">
       <formula1>"Positif,Negatif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2" xr:uid="{268DC933-A25C-DE45-9BA6-2A40B37E78EB}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AP2:AP3" xr:uid="{268DC933-A25C-DE45-9BA6-2A40B37E78EB}">
       <formula1>"Normal,Bayi Kuning Kramer 1-3,Bayi Kuning Kramer &gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM2" xr:uid="{CB08F77E-49BC-544C-8574-4FEDEA492356}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AR2:AR3" xr:uid="{CB08F77E-49BC-544C-8574-4FEDEA492356}">
       <formula1>"Normal,Bayi Kuning Kramer 1,Bayi Kuning Kramer 2,Bayi Kuning Kramer 3,Bayi Kuning Kramer 4,Bayi Kuning Kramer 5"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2" xr:uid="{D7812175-EA41-8345-9FD2-DBDE71A78328}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AS2:AS3" xr:uid="{D7812175-EA41-8345-9FD2-DBDE71A78328}">
       <formula1>"&gt;3 Normal,&lt;=3 Pucat"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: screening logic for examination status
</commit_message>
<xml_diff>
--- a/dataset/anak.xlsx
+++ b/dataset/anak.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9ECE863-5B8E-1C43-BD4D-1D1CF6118F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB578C2-B9A6-4A4F-8569-01EE5072980A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="19520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -195,7 +195,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="197">
   <si>
     <t>batas_awal</t>
   </si>
@@ -767,13 +767,25 @@
     <t>AFIFUDDIN MUHAJIR</t>
   </si>
   <si>
-    <t>2026-06-04</t>
-  </si>
-  <si>
-    <t>2026-06-10</t>
-  </si>
-  <si>
-    <t>ABYASA NARAYAN PRADIPTA</t>
+    <t>SHERYL MEILYTHA NABILA ZAFA</t>
+  </si>
+  <si>
+    <t>2026-06-17</t>
+  </si>
+  <si>
+    <t>2026-06-15</t>
+  </si>
+  <si>
+    <t>Telentang</t>
+  </si>
+  <si>
+    <t>Tidak dilakukan</t>
+  </si>
+  <si>
+    <t>Non Reaktif</t>
+  </si>
+  <si>
+    <t>Bukan kusta</t>
   </si>
 </sst>
 </file>
@@ -2452,143 +2464,530 @@
     </row>
     <row r="4" spans="1:136" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>191</v>
       </c>
       <c r="C4" t="s">
-        <v>192</v>
+        <v>190</v>
+      </c>
+      <c r="E4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F4" t="s">
+        <v>140</v>
+      </c>
+      <c r="H4" t="s">
+        <v>140</v>
+      </c>
+      <c r="I4" t="s">
+        <v>140</v>
+      </c>
+      <c r="J4" t="s">
+        <v>140</v>
+      </c>
+      <c r="K4" t="s">
+        <v>140</v>
+      </c>
+      <c r="L4" t="s">
+        <v>144</v>
+      </c>
+      <c r="M4" t="s">
+        <v>144</v>
+      </c>
+      <c r="N4" t="s">
+        <v>146</v>
+      </c>
+      <c r="O4" t="s">
+        <v>146</v>
+      </c>
+      <c r="P4" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>146</v>
+      </c>
+      <c r="R4" t="s">
+        <v>146</v>
+      </c>
+      <c r="S4" t="s">
+        <v>146</v>
+      </c>
+      <c r="T4" t="s">
+        <v>146</v>
+      </c>
+      <c r="U4" t="s">
+        <v>146</v>
+      </c>
+      <c r="V4" t="s">
+        <v>146</v>
+      </c>
+      <c r="W4" t="s">
+        <v>146</v>
+      </c>
+      <c r="X4" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>146</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>146</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>146</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>146</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>146</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>146</v>
+      </c>
+      <c r="AF4">
+        <v>3</v>
+      </c>
+      <c r="AG4">
+        <v>58</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>193</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>142</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>143</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>144</v>
+      </c>
+      <c r="AL4">
+        <v>10</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>145</v>
+      </c>
+      <c r="AN4" t="s">
+        <v>140</v>
+      </c>
+      <c r="AO4" t="s">
+        <v>140</v>
+      </c>
+      <c r="AP4" t="s">
+        <v>140</v>
+      </c>
+      <c r="AQ4" t="s">
+        <v>140</v>
+      </c>
+      <c r="AR4" t="s">
+        <v>140</v>
+      </c>
+      <c r="AS4" t="s">
+        <v>142</v>
+      </c>
+      <c r="AT4" t="s">
+        <v>146</v>
+      </c>
+      <c r="AU4">
+        <v>2900</v>
+      </c>
+      <c r="AV4">
+        <v>3000</v>
+      </c>
+      <c r="AW4">
+        <v>80</v>
+      </c>
+      <c r="AX4">
+        <v>90</v>
+      </c>
+      <c r="AY4" t="s">
+        <v>144</v>
+      </c>
+      <c r="AZ4" t="s">
+        <v>147</v>
+      </c>
+      <c r="BA4" t="s">
+        <v>147</v>
+      </c>
+      <c r="BB4" t="s">
+        <v>147</v>
+      </c>
+      <c r="BC4" t="s">
+        <v>144</v>
+      </c>
+      <c r="BD4" t="s">
+        <v>147</v>
+      </c>
+      <c r="BE4" t="s">
+        <v>144</v>
+      </c>
+      <c r="BF4" t="s">
+        <v>147</v>
+      </c>
+      <c r="BG4" t="s">
+        <v>144</v>
+      </c>
+      <c r="BH4" t="s">
+        <v>147</v>
+      </c>
+      <c r="BI4" t="s">
+        <v>140</v>
+      </c>
+      <c r="BJ4" t="s">
+        <v>142</v>
+      </c>
+      <c r="BK4">
+        <v>17062026</v>
+      </c>
+      <c r="BL4" t="s">
+        <v>142</v>
+      </c>
+      <c r="BM4" t="s">
+        <v>149</v>
+      </c>
+      <c r="BN4" t="s">
+        <v>150</v>
+      </c>
+      <c r="BO4" t="s">
+        <v>163</v>
+      </c>
+      <c r="BQ4" t="s">
+        <v>194</v>
+      </c>
+      <c r="BR4" t="s">
+        <v>154</v>
+      </c>
+      <c r="BS4" t="s">
+        <v>150</v>
+      </c>
+      <c r="BT4" t="s">
+        <v>159</v>
+      </c>
+      <c r="BU4" t="s">
+        <v>195</v>
+      </c>
+      <c r="BV4" t="s">
+        <v>150</v>
+      </c>
+      <c r="BW4" t="s">
+        <v>159</v>
+      </c>
+      <c r="BX4" t="s">
+        <v>196</v>
+      </c>
+      <c r="BY4" t="s">
+        <v>150</v>
+      </c>
+      <c r="BZ4" t="s">
+        <v>159</v>
+      </c>
+      <c r="CA4" t="s">
+        <v>150</v>
+      </c>
+      <c r="CB4" t="s">
+        <v>160</v>
+      </c>
+      <c r="CC4" t="s">
+        <v>161</v>
+      </c>
+      <c r="CD4" t="s">
+        <v>162</v>
+      </c>
+      <c r="CE4" t="s">
+        <v>142</v>
+      </c>
+      <c r="CF4" t="s">
+        <v>142</v>
+      </c>
+      <c r="CG4" t="s">
+        <v>150</v>
+      </c>
+      <c r="CH4" t="s">
+        <v>163</v>
+      </c>
+      <c r="CI4" t="s">
+        <v>140</v>
+      </c>
+      <c r="CJ4" t="s">
+        <v>150</v>
+      </c>
+      <c r="CK4" t="s">
+        <v>140</v>
+      </c>
+      <c r="CL4" t="s">
+        <v>140</v>
+      </c>
+      <c r="CM4" t="s">
+        <v>150</v>
+      </c>
+      <c r="CN4" t="s">
+        <v>140</v>
+      </c>
+      <c r="CO4" t="s">
+        <v>165</v>
+      </c>
+      <c r="CP4" t="s">
+        <v>140</v>
+      </c>
+      <c r="CQ4" t="s">
+        <v>140</v>
+      </c>
+      <c r="CR4" t="s">
+        <v>140</v>
+      </c>
+      <c r="CS4" t="s">
+        <v>140</v>
+      </c>
+      <c r="CT4" t="s">
+        <v>150</v>
+      </c>
+      <c r="CU4">
+        <v>99</v>
+      </c>
+      <c r="CV4" t="s">
+        <v>150</v>
+      </c>
+      <c r="CW4" t="s">
+        <v>167</v>
+      </c>
+      <c r="CX4" t="s">
+        <v>167</v>
+      </c>
+      <c r="CY4" t="s">
+        <v>168</v>
+      </c>
+      <c r="CZ4" t="s">
+        <v>169</v>
+      </c>
+      <c r="DA4" t="s">
+        <v>150</v>
+      </c>
+      <c r="DB4" t="s">
+        <v>170</v>
+      </c>
+      <c r="DC4" t="s">
+        <v>171</v>
+      </c>
+      <c r="DD4" t="s">
+        <v>150</v>
+      </c>
+      <c r="DE4" t="s">
+        <v>172</v>
+      </c>
+      <c r="DF4" t="s">
+        <v>173</v>
+      </c>
+      <c r="DG4" t="s">
+        <v>174</v>
+      </c>
+      <c r="DH4" t="s">
+        <v>150</v>
+      </c>
+      <c r="DI4" t="s">
+        <v>175</v>
+      </c>
+      <c r="DJ4" t="s">
+        <v>167</v>
+      </c>
+      <c r="DK4" t="s">
+        <v>166</v>
+      </c>
+      <c r="DL4" t="s">
+        <v>176</v>
+      </c>
+      <c r="DM4" t="s">
+        <v>150</v>
+      </c>
+      <c r="DN4" t="s">
+        <v>176</v>
+      </c>
+      <c r="DO4" t="s">
+        <v>177</v>
+      </c>
+      <c r="DP4" t="s">
+        <v>150</v>
+      </c>
+      <c r="DQ4" t="s">
+        <v>142</v>
+      </c>
+      <c r="DR4" t="s">
+        <v>178</v>
+      </c>
+      <c r="DS4" t="s">
+        <v>150</v>
+      </c>
+      <c r="DT4" t="s">
+        <v>179</v>
+      </c>
+      <c r="DU4" t="s">
+        <v>180</v>
+      </c>
+      <c r="DV4" t="s">
+        <v>147</v>
+      </c>
+      <c r="DW4" t="s">
+        <v>150</v>
+      </c>
+      <c r="DX4" t="s">
+        <v>181</v>
+      </c>
+      <c r="DY4" t="s">
+        <v>182</v>
+      </c>
+      <c r="DZ4" t="s">
+        <v>183</v>
+      </c>
+      <c r="EA4" t="s">
+        <v>184</v>
+      </c>
+      <c r="EB4" t="s">
+        <v>185</v>
+      </c>
+      <c r="EC4" t="s">
+        <v>186</v>
+      </c>
+      <c r="ED4" t="s">
+        <v>187</v>
+      </c>
+      <c r="EE4" t="s">
+        <v>142</v>
       </c>
       <c r="EF4" s="4"/>
     </row>
   </sheetData>
   <dataValidations count="43">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F3 L3:M3 AK2:AK3 AN2:AR3 AY2:AY3 BC2:BC3 BE2:BE3 BG2:BG3 BI2:BI3 CI2:CI3 CK2:CL3 CP2:CS3" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F4 L3:M4 AK2:AK4 AN2:AR4 AY2:AY4 BC2:BC4 BE2:BE4 BG2:BG4 BI2:BI4 CI2:CI4 CK2:CL4 CP2:CS4" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E3" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E4" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM2:AM3 BR2:BR3 EA2:EA3 ED2:ED3" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BN2:BN3 BS2:BS3 BV2:BV3 BY2:BY3 CA2:CA3 CG2:CG3 CJ2:CJ3 CM2:CM3 CT2:CT3 CV2:CV3 DA2:DA3 DD2:DD3 DH2:DH3 DM2:DM3 DP2:DP3 DS2:DS3 DW2:DW3" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM2:AM4 BR2:BR4 EA2:EA4 ED2:ED4" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BN2:BN4 BS2:BS4 BV2:BV4 BY2:BY4 CA2:CA4 CG2:CG4 CJ2:CJ4 CM2:CM4 CT2:CT4 CV2:CV4 DA2:DA4 DD2:DD4 DH2:DH4 DM2:DM4 DP2:DP4 DS2:DS4 DW2:DW4" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"True,False"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AS2:AS3" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AS2:AS4" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2:BO3" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2:BO4" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2:BP3" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2:BP4" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ2:BQ3" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ2:BQ4" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BT2:BT3" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BT2:BT4" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU2:BU3" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU2:BU4" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BW2:BW3" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BW2:BW4" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2:BX3" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2:BX4" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2:BZ3" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2:BZ4" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2:CB3" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2:CB4" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2:CC3" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2:CC4" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2:CD3" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2:CD4" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Sesuai Umur,Ada kemungkinan penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CE2:CE3" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CE2:CE4" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2:CF3" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2:CF4" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Normal,Curiga kelainan pupil putih pada anak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:K3 L2:AE2 CN2:CN3" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:K4 L2:AE2 CN2:CN4" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2:CO3" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2:CO4" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"&lt;20 bungkus per tahun,20-30 bungkus per tahun,&gt;30 bungkus per tahun"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DE2:DE3" xr:uid="{00000000-0002-0000-0000-000014000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DE2:DE4" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"HBsAg Non Reaktif,HBsAg Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DF2:DF3" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DF2:DF4" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"Anti HCV Non Reaktif,Anti HCV Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DG2:DG3" xr:uid="{00000000-0002-0000-0000-000016000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DG2:DG4" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"VL HCV RNA Negatif,VL HCV RNA Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DQ2:DQ3" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DQ2:DQ4" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Normal,Abnormal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DR2:DR3" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DR2:DR4" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"Normal,Abnormal ST Depresi,Abnormal T Inversi,Abnormal Hipertrofi Ventrikel Kiri,Abnormal Atrial Fibrilasi,Abnormal Q-Patologis,Abnormal ST Elevasi,Abnormal Gambaran Abnormal Lainnya"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DT2:DT3" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DT2:DT4" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"Bersedia,Menolak,Tidak tahu"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DU2:DU3" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DU2:DU4" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"Ditemukan benjolan,Tidak ditemukan benjolan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DV2:DV3" xr:uid="{00000000-0002-0000-0000-00001B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DV2:DV4" xr:uid="{00000000-0002-0000-0000-00001B000000}">
       <formula1>"Negatif,Positif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DX2:DX3" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DX2:DX4" xr:uid="{00000000-0002-0000-0000-00001C000000}">
       <formula1>"Memiliki diagnosis kanker &gt;5 tahun yang lalu,Memiliki diagnosis kanker &lt;5 tahun yang lalu,Tidak pernah didiagnosis menderita kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DY2:DY3" xr:uid="{00000000-0002-0000-0000-00001D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DY2:DY4" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>"Memiliki keluarga yang terdiagnosis kanker paru,Memiliki keluarga yang terdiagnosis kanker lain,Tidak ada keluarga yang terdiagnosis kanker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2:DZ3" xr:uid="{00000000-0002-0000-0000-00001E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DZ2:DZ4" xr:uid="{00000000-0002-0000-0000-00001E000000}">
       <formula1>"Perokok aktif (dalam 1 tahun ini masih merokok),Perokok/bekas perokok berhenti &lt;10 tahun lalu,Perokok pasif dari lingkungan rumah/tempat kerja,Tidak pernah merokok"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EB2:EB3" xr:uid="{00000000-0002-0000-0000-00001F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EB2:EB4" xr:uid="{00000000-0002-0000-0000-00001F000000}">
       <formula1>"Memiliki tempat tinggal berpotensi tinggi,Tidak yakin memiliki tempat tinggal berpotensi tinggi,Tidak memiliki tempat tinggal berpotensi tinggi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2:EC3" xr:uid="{00000000-0002-0000-0000-000020000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EC2:EC4" xr:uid="{00000000-0002-0000-0000-000020000000}">
       <formula1>"Memiliki lingkungan dalam rumah yang tidak sehat,Tidak yakin memiliki lingkungan dalam rumah yang tidak sehat,Memiliki lingkungan dalam rumah yang sehat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EE2:EE3" xr:uid="{00000000-0002-0000-0000-000021000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="EE2:EE4" xr:uid="{00000000-0002-0000-0000-000021000000}">
       <formula1>"Normal,Tidak Normal"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH2:AH3" xr:uid="{00000000-0002-0000-0000-000022000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH2:AH4" xr:uid="{00000000-0002-0000-0000-000022000000}">
       <formula1>"Berdiri,Telentang"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2:AI3" xr:uid="{00000000-0002-0000-0000-000023000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2:AI4" xr:uid="{00000000-0002-0000-0000-000023000000}">
       <formula1>"Makrosefali,Normal,Mikrosefali"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ3" xr:uid="{00000000-0002-0000-0000-000024000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ4" xr:uid="{00000000-0002-0000-0000-000024000000}">
       <formula1>"Perkembangan sesuai usia,Perkembangan meragukan,Perkembangan curiga adanya penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2:CH3" xr:uid="{00000000-0002-0000-0000-000025000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2:CH4" xr:uid="{00000000-0002-0000-0000-000025000000}">
       <formula1>"Tidak ada,1,2,3,&gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:AE3 AT2:AT3" xr:uid="{00000000-0002-0000-0000-000026000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:AE4 AT2:AT4" xr:uid="{00000000-0002-0000-0000-000026000000}">
       <formula1>"Sudah,Belum"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AZ2:BB3 BD2:BD3 BF2:BF3 BH2:BH3" xr:uid="{00000000-0002-0000-0000-000027000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AZ2:BB4 BD2:BD4 BF2:BF4 BH2:BH4" xr:uid="{00000000-0002-0000-0000-000027000000}">
       <formula1>"Positif,Negatif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BJ2:BJ3" xr:uid="{00000000-0002-0000-0000-000028000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BJ2:BJ4" xr:uid="{00000000-0002-0000-0000-000028000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1-3,Bayi Kuning Kramer &gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2:BL3" xr:uid="{00000000-0002-0000-0000-000029000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2:BL4" xr:uid="{00000000-0002-0000-0000-000029000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1,Bayi Kuning Kramer 2,Bayi Kuning Kramer 3,Bayi Kuning Kramer 4,Bayi Kuning Kramer 5"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BM2:BM3" xr:uid="{00000000-0002-0000-0000-00002A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BM2:BM4" xr:uid="{00000000-0002-0000-0000-00002A000000}">
       <formula1>"&gt;3 Normal,&lt;=3 Pucat"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
update dataset excel files
</commit_message>
<xml_diff>
--- a/dataset/anak.xlsx
+++ b/dataset/anak.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/Downloads/dist/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B37D5B3E-FA75-B54B-A5FE-A3EA8E2DDA38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE21BE9F-3992-DF4A-8E32-7378AF947F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4500" yWindow="-21000" windowWidth="36000" windowHeight="19520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: stage 4 fixing skrining-filtering, doing excel modification for anak and screening nakes
</commit_message>
<xml_diff>
--- a/dataset/anak.xlsx
+++ b/dataset/anak.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC938DA8-5369-5344-89C0-ECCFE8E36FCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69689F7C-0C0C-1545-BFBC-F83AFA9E82E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4500" yWindow="-21000" windowWidth="36000" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -100,7 +100,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="BA1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -115,7 +115,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BQ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="CB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -130,33 +130,49 @@
         </r>
       </text>
     </comment>
-    <comment ref="BU1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="CG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
+            <color rgb="FF000000"/>
             <rFont val="Aptos Narrow"/>
             <family val="2"/>
-            <scheme val="minor"/>
           </rPr>
-          <t>Microsoft Office User:
-wajib diisi apabila Suspek Frambusia</t>
+          <t xml:space="preserve">Microsoft Office User:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t>wajib diisi apabila Suspek Frambusia</t>
         </r>
       </text>
     </comment>
-    <comment ref="BW1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="CJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
             <sz val="12"/>
-            <color theme="1"/>
+            <color rgb="FF000000"/>
             <rFont val="Aptos Narrow"/>
             <family val="2"/>
-            <scheme val="minor"/>
           </rPr>
-          <t>Microsoft Office User:
-wajib diisi apabila bercak_putih Meragukan</t>
+          <t xml:space="preserve">Microsoft Office User:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
+          </rPr>
+          <t>wajib diisi apabila bercak_putih Meragukan</t>
         </r>
       </text>
     </comment>
@@ -165,7 +181,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="136">
   <si>
     <t>batas_awal</t>
   </si>
@@ -525,13 +541,61 @@
   </si>
   <si>
     <t>skrining_imunisasi_rutin_balita</t>
+  </si>
+  <si>
+    <t>skrining_pertumbuhan</t>
+  </si>
+  <si>
+    <t>skrining_kpsp</t>
+  </si>
+  <si>
+    <t>skrining_m_chat_1</t>
+  </si>
+  <si>
+    <t>skrining_m_chat_2</t>
+  </si>
+  <si>
+    <t>skrining_risiko_tb_anak</t>
+  </si>
+  <si>
+    <t>skrining_tb_anak</t>
+  </si>
+  <si>
+    <t>skrining_imunisasi_hepatitis_b</t>
+  </si>
+  <si>
+    <t>skrining_berat_lahir</t>
+  </si>
+  <si>
+    <t>skrining_jantung_bawaan</t>
+  </si>
+  <si>
+    <t>skrining_shk</t>
+  </si>
+  <si>
+    <t>skrining_gizi_anak_sekolah</t>
+  </si>
+  <si>
+    <t>skrining_periksa_gigi_anak</t>
+  </si>
+  <si>
+    <t>skrining_telinga_mata_anak_sekolah</t>
+  </si>
+  <si>
+    <t>skrining_skabies</t>
+  </si>
+  <si>
+    <t>skrining_kusta</t>
+  </si>
+  <si>
+    <t>skrining_frambusia</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -558,6 +622,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -608,7 +678,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -618,6 +688,7 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Dark Mode" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -953,7 +1024,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CE5"/>
+  <dimension ref="A1:CU5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -980,48 +1051,66 @@
     <col min="25" max="25" width="24.5" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="29" bestFit="1" customWidth="1"/>
     <col min="27" max="33" width="29" customWidth="1"/>
-    <col min="34" max="35" width="14.33203125" customWidth="1"/>
-    <col min="36" max="36" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="19" bestFit="1" customWidth="1"/>
-    <col min="38" max="40" width="19" customWidth="1"/>
-    <col min="41" max="41" width="25" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="14.83203125" customWidth="1"/>
-    <col min="48" max="48" width="28.83203125" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="10" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="16" bestFit="1" customWidth="1"/>
-    <col min="52" max="53" width="13.6640625" customWidth="1"/>
-    <col min="54" max="54" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="55" max="56" width="13.6640625" customWidth="1"/>
-    <col min="57" max="57" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="58" max="62" width="22.5" customWidth="1"/>
-    <col min="63" max="63" width="35.83203125" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="22.5" customWidth="1"/>
-    <col min="65" max="65" width="22.5" style="1" customWidth="1"/>
-    <col min="66" max="67" width="22.5" customWidth="1"/>
-    <col min="68" max="68" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="22.83203125" customWidth="1"/>
-    <col min="72" max="72" width="16.1640625" customWidth="1"/>
-    <col min="73" max="73" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="74" max="75" width="12.33203125" customWidth="1"/>
-    <col min="76" max="76" width="14.1640625" customWidth="1"/>
-    <col min="77" max="77" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="23.6640625" customWidth="1"/>
-    <col min="79" max="79" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="20" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="19.5" style="6" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="23.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="36" max="37" width="14.33203125" customWidth="1"/>
+    <col min="38" max="38" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="19" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="29" style="6" customWidth="1"/>
+    <col min="41" max="41" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="29" style="6" customWidth="1"/>
+    <col min="43" max="43" width="19" customWidth="1"/>
+    <col min="44" max="44" width="29" style="6" customWidth="1"/>
+    <col min="45" max="45" width="19" customWidth="1"/>
+    <col min="46" max="46" width="19" style="6" customWidth="1"/>
+    <col min="47" max="47" width="25" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="14.83203125" customWidth="1"/>
+    <col min="54" max="54" width="26.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="28.83203125" style="6" customWidth="1"/>
+    <col min="57" max="57" width="10" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="22.1640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="16" bestFit="1" customWidth="1"/>
+    <col min="61" max="62" width="13.6640625" customWidth="1"/>
+    <col min="63" max="63" width="13.6640625" style="6" customWidth="1"/>
+    <col min="64" max="64" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="65" max="66" width="13.6640625" customWidth="1"/>
+    <col min="67" max="67" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="68" max="72" width="22.5" customWidth="1"/>
+    <col min="73" max="73" width="35.83203125" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="22.5" customWidth="1"/>
+    <col min="75" max="75" width="22.5" style="1" customWidth="1"/>
+    <col min="76" max="77" width="22.5" customWidth="1"/>
+    <col min="78" max="78" width="22.5" style="6" customWidth="1"/>
+    <col min="79" max="79" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="22.83203125" customWidth="1"/>
+    <col min="83" max="83" width="22.83203125" style="6" customWidth="1"/>
+    <col min="84" max="84" width="16.1640625" customWidth="1"/>
+    <col min="85" max="85" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="19.83203125" style="6" customWidth="1"/>
+    <col min="87" max="88" width="12.33203125" customWidth="1"/>
+    <col min="89" max="89" width="12.33203125" style="6" customWidth="1"/>
+    <col min="90" max="90" width="14.1640625" customWidth="1"/>
+    <col min="91" max="91" width="14.1640625" style="6" customWidth="1"/>
+    <col min="92" max="92" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="23.6640625" customWidth="1"/>
+    <col min="94" max="94" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="23.1640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:83" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:99" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1121,158 +1210,206 @@
       <c r="AG1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AH1" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="AI1" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="AJ1" t="s">
         <v>30</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AK1" t="s">
         <v>31</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AL1" t="s">
         <v>32</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AM1" t="s">
         <v>33</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AN1" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="AO1" t="s">
         <v>34</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AP1" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="AQ1" t="s">
         <v>35</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AR1" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="AS1" t="s">
         <v>36</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AT1" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="AU1" t="s">
         <v>37</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AV1" t="s">
         <v>38</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AW1" t="s">
         <v>39</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AX1" t="s">
         <v>40</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AY1" t="s">
         <v>41</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AZ1" t="s">
         <v>42</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="BA1" t="s">
         <v>43</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="BB1" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="BC1" t="s">
         <v>44</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="BD1" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="BE1" t="s">
         <v>45</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="BF1" t="s">
         <v>46</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="BG1" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="BH1" t="s">
         <v>47</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BI1" t="s">
         <v>48</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BJ1" t="s">
         <v>49</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BK1" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="BL1" t="s">
         <v>50</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BM1" t="s">
         <v>51</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BN1" t="s">
         <v>52</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BO1" t="s">
         <v>53</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BP1" t="s">
         <v>54</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BQ1" t="s">
         <v>55</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BR1" t="s">
         <v>56</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BS1" t="s">
         <v>57</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BT1" t="s">
         <v>58</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BU1" t="s">
         <v>59</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BV1" t="s">
         <v>60</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BW1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BX1" t="s">
         <v>62</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BY1" t="s">
         <v>63</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BZ1" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="CA1" t="s">
         <v>64</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="CB1" t="s">
         <v>65</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="CC1" t="s">
         <v>66</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="CD1" t="s">
         <v>67</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="CE1" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="CF1" t="s">
         <v>68</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="CG1" t="s">
         <v>69</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="CH1" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="CI1" t="s">
         <v>70</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="CJ1" t="s">
         <v>71</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CK1" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="CL1" t="s">
         <v>72</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CM1" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="CN1" t="s">
         <v>73</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CO1" t="s">
         <v>74</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CP1" t="s">
         <v>75</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CQ1" t="s">
         <v>76</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CR1" t="s">
         <v>77</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CS1" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="CT1" t="s">
         <v>78</v>
       </c>
-      <c r="CE1" t="s">
+      <c r="CU1" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:83" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:99" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>80</v>
       </c>
@@ -1297,158 +1434,206 @@
       <c r="M2" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="AH2">
+      <c r="AH2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AJ2">
         <v>5</v>
       </c>
-      <c r="AI2">
+      <c r="AK2">
         <v>100</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AL2" t="s">
         <v>85</v>
       </c>
-      <c r="AK2" t="s">
+      <c r="AM2" t="s">
         <v>86</v>
       </c>
-      <c r="AL2" t="s">
+      <c r="AN2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AO2" t="s">
         <v>87</v>
       </c>
-      <c r="AM2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AN2">
+      <c r="AP2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AR2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AS2">
         <v>10</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AT2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AU2" t="s">
         <v>89</v>
       </c>
-      <c r="AP2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AS2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AT2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AU2" t="s">
+      <c r="AV2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AW2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AX2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AY2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AZ2" t="s">
+        <v>88</v>
+      </c>
+      <c r="BA2" t="s">
         <v>86</v>
       </c>
-      <c r="AV2" t="s">
-        <v>90</v>
-      </c>
-      <c r="AW2">
+      <c r="BB2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BC2" t="s">
+        <v>90</v>
+      </c>
+      <c r="BD2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BE2">
         <v>2900</v>
       </c>
-      <c r="AX2">
+      <c r="BF2">
         <v>6000</v>
       </c>
-      <c r="AY2">
+      <c r="BG2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BH2">
         <v>80</v>
       </c>
-      <c r="AZ2">
-        <v>90</v>
-      </c>
-      <c r="BA2" t="s">
-        <v>88</v>
-      </c>
-      <c r="BB2" t="s">
+      <c r="BI2">
+        <v>90</v>
+      </c>
+      <c r="BJ2" t="s">
+        <v>88</v>
+      </c>
+      <c r="BK2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BL2" t="s">
         <v>91</v>
       </c>
-      <c r="BC2" t="s">
+      <c r="BM2" t="s">
         <v>91</v>
       </c>
-      <c r="BD2" t="s">
+      <c r="BN2" t="s">
         <v>91</v>
       </c>
-      <c r="BE2" t="s">
-        <v>88</v>
-      </c>
-      <c r="BF2" t="s">
+      <c r="BO2" t="s">
+        <v>88</v>
+      </c>
+      <c r="BP2" t="s">
         <v>91</v>
       </c>
-      <c r="BG2" t="s">
-        <v>88</v>
-      </c>
-      <c r="BH2" t="s">
+      <c r="BQ2" t="s">
+        <v>88</v>
+      </c>
+      <c r="BR2" t="s">
         <v>91</v>
       </c>
-      <c r="BI2" t="s">
-        <v>88</v>
-      </c>
-      <c r="BJ2" t="s">
+      <c r="BS2" t="s">
+        <v>88</v>
+      </c>
+      <c r="BT2" t="s">
         <v>91</v>
       </c>
-      <c r="BK2" t="s">
-        <v>84</v>
-      </c>
-      <c r="BL2" t="s">
+      <c r="BU2" t="s">
+        <v>84</v>
+      </c>
+      <c r="BV2" t="s">
         <v>92</v>
       </c>
-      <c r="BM2" s="1" t="s">
+      <c r="BW2" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="BN2" t="s">
+      <c r="BX2" t="s">
         <v>86</v>
       </c>
-      <c r="BO2" t="s">
+      <c r="BY2" t="s">
         <v>94</v>
       </c>
-      <c r="BP2" t="s">
+      <c r="BZ2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CA2" t="s">
         <v>95</v>
       </c>
-      <c r="BQ2" t="s">
+      <c r="CB2" t="s">
         <v>96</v>
       </c>
-      <c r="BR2" t="s">
+      <c r="CC2" t="s">
         <v>97</v>
       </c>
-      <c r="BS2" t="s">
+      <c r="CD2" t="s">
         <v>98</v>
       </c>
-      <c r="BT2" t="s">
+      <c r="CE2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CF2" t="s">
         <v>99</v>
       </c>
-      <c r="BU2" t="s">
+      <c r="CG2" t="s">
         <v>100</v>
       </c>
-      <c r="BV2" t="s">
+      <c r="CH2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CI2" t="s">
         <v>101</v>
       </c>
-      <c r="BW2" t="s">
+      <c r="CJ2" t="s">
         <v>102</v>
       </c>
-      <c r="BX2" t="s">
+      <c r="CK2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CL2" t="s">
         <v>99</v>
       </c>
-      <c r="BY2" t="s">
+      <c r="CM2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CN2" t="s">
         <v>103</v>
       </c>
-      <c r="BZ2" t="s">
+      <c r="CO2" t="s">
         <v>104</v>
       </c>
-      <c r="CA2" t="s">
+      <c r="CP2" t="s">
         <v>105</v>
       </c>
-      <c r="CB2" t="s">
+      <c r="CQ2" t="s">
         <v>86</v>
       </c>
-      <c r="CC2" t="s">
+      <c r="CR2" t="s">
         <v>86</v>
       </c>
-      <c r="CD2" t="s">
+      <c r="CS2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CT2" t="s">
         <v>95</v>
       </c>
-      <c r="CE2" t="s">
+      <c r="CU2" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="3" spans="1:83" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:99" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>80</v>
       </c>
@@ -1545,158 +1730,206 @@
       <c r="AG3" t="s">
         <v>90</v>
       </c>
-      <c r="AH3">
+      <c r="AH3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AJ3">
         <v>5</v>
       </c>
-      <c r="AI3">
+      <c r="AK3">
         <v>100</v>
       </c>
-      <c r="AJ3" t="s">
+      <c r="AL3" t="s">
         <v>85</v>
       </c>
-      <c r="AK3" t="s">
+      <c r="AM3" t="s">
         <v>86</v>
       </c>
-      <c r="AL3" t="s">
+      <c r="AN3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AO3" t="s">
         <v>87</v>
       </c>
-      <c r="AM3" t="s">
-        <v>88</v>
-      </c>
-      <c r="AN3">
+      <c r="AP3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AQ3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AR3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AS3">
         <v>10</v>
       </c>
-      <c r="AO3" t="s">
+      <c r="AT3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AU3" t="s">
         <v>89</v>
       </c>
-      <c r="AP3" t="s">
-        <v>88</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>88</v>
-      </c>
-      <c r="AR3" t="s">
-        <v>88</v>
-      </c>
-      <c r="AS3" t="s">
-        <v>88</v>
-      </c>
-      <c r="AT3" t="s">
-        <v>88</v>
-      </c>
-      <c r="AU3" t="s">
+      <c r="AV3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AW3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AX3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AY3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AZ3" t="s">
+        <v>88</v>
+      </c>
+      <c r="BA3" t="s">
         <v>86</v>
       </c>
-      <c r="AV3" t="s">
-        <v>90</v>
-      </c>
-      <c r="AW3">
+      <c r="BB3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BC3" t="s">
+        <v>90</v>
+      </c>
+      <c r="BD3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BE3">
         <v>2900</v>
       </c>
-      <c r="AX3">
+      <c r="BF3">
         <v>6000</v>
       </c>
-      <c r="AY3">
+      <c r="BG3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BH3">
         <v>80</v>
       </c>
-      <c r="AZ3">
-        <v>90</v>
-      </c>
-      <c r="BA3" t="s">
-        <v>88</v>
-      </c>
-      <c r="BB3" t="s">
+      <c r="BI3">
+        <v>90</v>
+      </c>
+      <c r="BJ3" t="s">
+        <v>88</v>
+      </c>
+      <c r="BK3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BL3" t="s">
         <v>91</v>
       </c>
-      <c r="BC3" t="s">
+      <c r="BM3" t="s">
         <v>91</v>
       </c>
-      <c r="BD3" t="s">
+      <c r="BN3" t="s">
         <v>91</v>
       </c>
-      <c r="BE3" t="s">
-        <v>88</v>
-      </c>
-      <c r="BF3" t="s">
+      <c r="BO3" t="s">
+        <v>88</v>
+      </c>
+      <c r="BP3" t="s">
         <v>91</v>
       </c>
-      <c r="BG3" t="s">
-        <v>88</v>
-      </c>
-      <c r="BH3" t="s">
+      <c r="BQ3" t="s">
+        <v>88</v>
+      </c>
+      <c r="BR3" t="s">
         <v>91</v>
       </c>
-      <c r="BI3" t="s">
-        <v>88</v>
-      </c>
-      <c r="BJ3" t="s">
+      <c r="BS3" t="s">
+        <v>88</v>
+      </c>
+      <c r="BT3" t="s">
         <v>91</v>
       </c>
-      <c r="BK3" t="s">
-        <v>84</v>
-      </c>
-      <c r="BL3" t="s">
+      <c r="BU3" t="s">
+        <v>84</v>
+      </c>
+      <c r="BV3" t="s">
         <v>92</v>
       </c>
-      <c r="BM3" s="1" t="s">
+      <c r="BW3" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="BN3" t="s">
+      <c r="BX3" t="s">
         <v>86</v>
       </c>
-      <c r="BO3" t="s">
+      <c r="BY3" t="s">
         <v>94</v>
       </c>
-      <c r="BP3" t="s">
+      <c r="BZ3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CA3" t="s">
         <v>95</v>
       </c>
-      <c r="BQ3" t="s">
+      <c r="CB3" t="s">
         <v>96</v>
       </c>
-      <c r="BR3" t="s">
+      <c r="CC3" t="s">
         <v>97</v>
       </c>
-      <c r="BS3" t="s">
+      <c r="CD3" t="s">
         <v>98</v>
       </c>
-      <c r="BT3" t="s">
+      <c r="CE3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CF3" t="s">
         <v>99</v>
       </c>
-      <c r="BU3" t="s">
+      <c r="CG3" t="s">
         <v>100</v>
       </c>
-      <c r="BV3" t="s">
+      <c r="CH3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CI3" t="s">
         <v>101</v>
       </c>
-      <c r="BW3" t="s">
+      <c r="CJ3" t="s">
         <v>102</v>
       </c>
-      <c r="BX3" t="s">
+      <c r="CK3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CL3" t="s">
         <v>99</v>
       </c>
-      <c r="BY3" t="s">
+      <c r="CM3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CN3" t="s">
         <v>103</v>
       </c>
-      <c r="BZ3" t="s">
+      <c r="CO3" t="s">
         <v>104</v>
       </c>
-      <c r="CA3" t="s">
+      <c r="CP3" t="s">
         <v>105</v>
       </c>
-      <c r="CB3" t="s">
+      <c r="CQ3" t="s">
         <v>86</v>
       </c>
-      <c r="CC3" t="s">
+      <c r="CR3" t="s">
         <v>86</v>
       </c>
-      <c r="CD3" t="s">
+      <c r="CS3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CT3" t="s">
         <v>95</v>
       </c>
-      <c r="CE3" t="s">
+      <c r="CU3" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="4" spans="1:83" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:99" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>108</v>
       </c>
@@ -1793,155 +2026,203 @@
       <c r="AG4" t="s">
         <v>90</v>
       </c>
-      <c r="AH4">
+      <c r="AH4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AJ4">
         <v>5</v>
       </c>
-      <c r="AI4">
+      <c r="AK4">
         <v>58</v>
       </c>
-      <c r="AJ4" t="s">
+      <c r="AL4" t="s">
         <v>111</v>
       </c>
-      <c r="AK4" t="s">
+      <c r="AM4" t="s">
         <v>86</v>
       </c>
-      <c r="AL4" t="s">
+      <c r="AN4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AO4" t="s">
         <v>87</v>
       </c>
-      <c r="AM4" t="s">
-        <v>88</v>
-      </c>
-      <c r="AN4">
+      <c r="AP4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AQ4" t="s">
+        <v>88</v>
+      </c>
+      <c r="AR4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AS4">
         <v>10</v>
       </c>
-      <c r="AO4" t="s">
+      <c r="AT4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AU4" t="s">
         <v>89</v>
       </c>
-      <c r="AP4" t="s">
-        <v>84</v>
-      </c>
-      <c r="AQ4" t="s">
-        <v>84</v>
-      </c>
-      <c r="AR4" t="s">
-        <v>84</v>
-      </c>
-      <c r="AS4" t="s">
-        <v>84</v>
-      </c>
-      <c r="AT4" t="s">
-        <v>84</v>
-      </c>
-      <c r="AU4" t="s">
+      <c r="AV4" t="s">
+        <v>84</v>
+      </c>
+      <c r="AW4" t="s">
+        <v>84</v>
+      </c>
+      <c r="AX4" t="s">
+        <v>84</v>
+      </c>
+      <c r="AY4" t="s">
+        <v>84</v>
+      </c>
+      <c r="AZ4" t="s">
+        <v>84</v>
+      </c>
+      <c r="BA4" t="s">
         <v>86</v>
       </c>
-      <c r="AV4" t="s">
-        <v>90</v>
-      </c>
-      <c r="AW4">
+      <c r="BB4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BC4" t="s">
+        <v>90</v>
+      </c>
+      <c r="BD4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BE4">
         <v>2900</v>
       </c>
-      <c r="AX4">
+      <c r="BF4">
         <v>3000</v>
       </c>
-      <c r="AY4">
+      <c r="BG4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BH4">
         <v>80</v>
       </c>
-      <c r="AZ4">
-        <v>90</v>
-      </c>
-      <c r="BA4" t="s">
-        <v>88</v>
-      </c>
-      <c r="BB4" t="s">
+      <c r="BI4">
+        <v>90</v>
+      </c>
+      <c r="BJ4" t="s">
+        <v>88</v>
+      </c>
+      <c r="BK4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BL4" t="s">
         <v>91</v>
       </c>
-      <c r="BC4" t="s">
+      <c r="BM4" t="s">
         <v>91</v>
       </c>
-      <c r="BD4" t="s">
+      <c r="BN4" t="s">
         <v>91</v>
       </c>
-      <c r="BE4" t="s">
-        <v>88</v>
-      </c>
-      <c r="BF4" t="s">
+      <c r="BO4" t="s">
+        <v>88</v>
+      </c>
+      <c r="BP4" t="s">
         <v>91</v>
       </c>
-      <c r="BG4" t="s">
-        <v>88</v>
-      </c>
-      <c r="BH4" t="s">
+      <c r="BQ4" t="s">
+        <v>88</v>
+      </c>
+      <c r="BR4" t="s">
         <v>91</v>
       </c>
-      <c r="BI4" t="s">
-        <v>88</v>
-      </c>
-      <c r="BJ4" t="s">
+      <c r="BS4" t="s">
+        <v>88</v>
+      </c>
+      <c r="BT4" t="s">
         <v>91</v>
       </c>
-      <c r="BK4" t="s">
-        <v>84</v>
-      </c>
-      <c r="BL4" t="s">
+      <c r="BU4" t="s">
+        <v>84</v>
+      </c>
+      <c r="BV4" t="s">
         <v>86</v>
       </c>
-      <c r="BM4" s="1" t="s">
+      <c r="BW4" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BX4" t="s">
         <v>86</v>
       </c>
-      <c r="BO4" t="s">
+      <c r="BY4" t="s">
         <v>94</v>
       </c>
-      <c r="BP4" t="s">
+      <c r="BZ4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CA4" t="s">
         <v>95</v>
       </c>
-      <c r="BR4" t="s">
+      <c r="CC4" t="s">
         <v>112</v>
       </c>
-      <c r="BS4" t="s">
+      <c r="CD4" t="s">
         <v>98</v>
       </c>
-      <c r="BT4" t="s">
+      <c r="CE4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CF4" t="s">
         <v>99</v>
       </c>
-      <c r="BU4" t="s">
+      <c r="CG4" t="s">
         <v>100</v>
       </c>
-      <c r="BV4" t="s">
+      <c r="CH4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CI4" t="s">
         <v>99</v>
       </c>
-      <c r="BW4" t="s">
+      <c r="CJ4" t="s">
         <v>113</v>
       </c>
-      <c r="BX4" t="s">
+      <c r="CK4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CL4" t="s">
         <v>99</v>
       </c>
-      <c r="BY4" t="s">
+      <c r="CM4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CN4" t="s">
         <v>103</v>
       </c>
-      <c r="BZ4" t="s">
+      <c r="CO4" t="s">
         <v>104</v>
       </c>
-      <c r="CA4" t="s">
+      <c r="CP4" t="s">
         <v>105</v>
       </c>
-      <c r="CB4" t="s">
+      <c r="CQ4" t="s">
         <v>86</v>
       </c>
-      <c r="CC4" t="s">
+      <c r="CR4" t="s">
         <v>86</v>
       </c>
-      <c r="CD4" t="s">
+      <c r="CS4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CT4" t="s">
         <v>95</v>
       </c>
-      <c r="CE4" s="4" t="s">
+      <c r="CU4" s="4" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="5" spans="1:83" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:99" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>114</v>
       </c>
@@ -2038,233 +2319,281 @@
       <c r="AG5" t="s">
         <v>90</v>
       </c>
-      <c r="AH5">
+      <c r="AH5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AJ5">
         <v>5</v>
       </c>
-      <c r="AI5">
+      <c r="AK5">
         <v>58</v>
       </c>
-      <c r="AJ5" t="s">
+      <c r="AL5" t="s">
         <v>111</v>
       </c>
-      <c r="AK5" t="s">
+      <c r="AM5" t="s">
         <v>86</v>
       </c>
-      <c r="AL5" t="s">
+      <c r="AN5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AO5" t="s">
         <v>87</v>
       </c>
-      <c r="AM5" t="s">
-        <v>88</v>
-      </c>
-      <c r="AN5">
+      <c r="AP5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>88</v>
+      </c>
+      <c r="AR5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AS5">
         <v>10</v>
       </c>
-      <c r="AO5" t="s">
+      <c r="AT5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AU5" t="s">
         <v>89</v>
       </c>
-      <c r="AP5" t="s">
-        <v>84</v>
-      </c>
-      <c r="AQ5" t="s">
-        <v>84</v>
-      </c>
-      <c r="AR5" t="s">
-        <v>84</v>
-      </c>
-      <c r="AS5" t="s">
-        <v>84</v>
-      </c>
-      <c r="AT5" t="s">
-        <v>84</v>
-      </c>
-      <c r="AU5" t="s">
+      <c r="AV5" t="s">
+        <v>84</v>
+      </c>
+      <c r="AW5" t="s">
+        <v>84</v>
+      </c>
+      <c r="AX5" t="s">
+        <v>84</v>
+      </c>
+      <c r="AY5" t="s">
+        <v>84</v>
+      </c>
+      <c r="AZ5" t="s">
+        <v>84</v>
+      </c>
+      <c r="BA5" t="s">
         <v>86</v>
       </c>
-      <c r="AV5" t="s">
-        <v>90</v>
-      </c>
-      <c r="AW5">
+      <c r="BB5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BC5" t="s">
+        <v>90</v>
+      </c>
+      <c r="BD5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BE5">
         <v>2900</v>
       </c>
-      <c r="AX5">
+      <c r="BF5">
         <v>3000</v>
       </c>
-      <c r="AY5">
+      <c r="BG5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BH5">
         <v>80</v>
       </c>
-      <c r="AZ5">
-        <v>90</v>
-      </c>
-      <c r="BA5" t="s">
-        <v>88</v>
-      </c>
-      <c r="BB5" t="s">
+      <c r="BI5">
+        <v>90</v>
+      </c>
+      <c r="BJ5" t="s">
+        <v>88</v>
+      </c>
+      <c r="BK5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BL5" t="s">
         <v>91</v>
       </c>
-      <c r="BC5" t="s">
+      <c r="BM5" t="s">
         <v>91</v>
       </c>
-      <c r="BD5" t="s">
+      <c r="BN5" t="s">
         <v>91</v>
       </c>
-      <c r="BE5" t="s">
-        <v>88</v>
-      </c>
-      <c r="BF5" t="s">
+      <c r="BO5" t="s">
+        <v>88</v>
+      </c>
+      <c r="BP5" t="s">
         <v>91</v>
       </c>
-      <c r="BG5" t="s">
-        <v>88</v>
-      </c>
-      <c r="BH5" t="s">
+      <c r="BQ5" t="s">
+        <v>88</v>
+      </c>
+      <c r="BR5" t="s">
         <v>91</v>
       </c>
-      <c r="BI5" t="s">
-        <v>88</v>
-      </c>
-      <c r="BJ5" t="s">
+      <c r="BS5" t="s">
+        <v>88</v>
+      </c>
+      <c r="BT5" t="s">
         <v>91</v>
       </c>
-      <c r="BK5" t="s">
-        <v>84</v>
-      </c>
-      <c r="BL5" t="s">
+      <c r="BU5" t="s">
+        <v>84</v>
+      </c>
+      <c r="BV5" t="s">
         <v>86</v>
       </c>
-      <c r="BM5" s="1" t="s">
+      <c r="BW5" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="BN5" t="s">
+      <c r="BX5" t="s">
         <v>86</v>
       </c>
-      <c r="BO5" t="s">
+      <c r="BY5" t="s">
         <v>94</v>
       </c>
-      <c r="BP5" t="s">
+      <c r="BZ5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CA5" t="s">
         <v>95</v>
       </c>
-      <c r="BR5" t="s">
+      <c r="CC5" t="s">
         <v>112</v>
       </c>
-      <c r="BS5" t="s">
+      <c r="CD5" t="s">
         <v>98</v>
       </c>
-      <c r="BT5" t="s">
+      <c r="CE5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CF5" t="s">
         <v>99</v>
       </c>
-      <c r="BU5" t="s">
+      <c r="CG5" t="s">
         <v>100</v>
       </c>
-      <c r="BV5" t="s">
+      <c r="CH5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CI5" t="s">
         <v>99</v>
       </c>
-      <c r="BW5" t="s">
+      <c r="CJ5" t="s">
         <v>113</v>
       </c>
-      <c r="BX5" t="s">
+      <c r="CK5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CL5" t="s">
         <v>99</v>
       </c>
-      <c r="BY5" t="s">
+      <c r="CM5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CN5" t="s">
         <v>103</v>
       </c>
-      <c r="BZ5" t="s">
+      <c r="CO5" t="s">
         <v>104</v>
       </c>
-      <c r="CA5" t="s">
+      <c r="CP5" t="s">
         <v>105</v>
       </c>
-      <c r="CB5" t="s">
+      <c r="CQ5" t="s">
         <v>86</v>
       </c>
-      <c r="CC5" t="s">
+      <c r="CR5" t="s">
         <v>86</v>
       </c>
-      <c r="CD5" t="s">
+      <c r="CS5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CT5" t="s">
         <v>95</v>
       </c>
-      <c r="CE5" t="s">
+      <c r="CU5" t="s">
         <v>106</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="27">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:O5 AM2:AM5 AP2:AT5 BA2:BA5 BE2:BE5 BG2:BG5 BI2:BI5 BK2:BK5 D2:D14 F2:G5 M2:M5" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:O5 AN2:AN5 AV2:AZ5 BG2:BG5 BO2:BO5 BQ2:BQ5 BS2:BS5 BU2:BU5 D2:D14 F2:G5 M2:M5 BJ2:BK5 AP2:AR5 AT2:AT5 BZ2:BZ5 BB2:BB5 BD2:BD5 AH2:AI5 CS2:CS5 CM2:CM5 CK2:CK5 CH2:CH5 CE2:CE5" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E5" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2:AO5 BS2:BS5" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2:AU5" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2:AU5 CD2:CD5" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BA2:BA5" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2:BP5" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA2:CA5" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BQ2:BQ5" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2:CB5" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2:BR5" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2:CC5" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BT2:BT5" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2:CF5" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU2:BU5" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2:CG5" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BV2:BV5" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2:CI5" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BW2:BW5" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2:CJ5" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2:BX5" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2:CL5" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BY2:BY5" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2:CN5" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2:BZ5" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2:CO5" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA2:CA5" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2:CP5" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Sesuai Umur,Ada kemungkinan penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2:CB5" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2:CQ5" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2:CC5" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2:CR5" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Curiga kelainan pupil putih pada anak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:AG2 I2:L5" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:L5 N2:AG2" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ5" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2:AL5" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"Berdiri,Telentang"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AK2:AK5" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM2:AM5" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"Makrosefali,Normal,Mikrosefali"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AL2:AL5" xr:uid="{00000000-0002-0000-0000-000014000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2:AO5" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"Perkembangan sesuai usia,Perkembangan meragukan,Perkembangan curiga adanya penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2:CD5" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2:CT5" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"Tidak ada,1,2,3,&gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P3:AG5 AV2:AV5" xr:uid="{00000000-0002-0000-0000-000016000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P3:AG5 BC2:BC5" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"Sudah,Belum"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BB2:BD5 BF2:BF5 BH2:BH5 BJ2:BJ5" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2:BN5 BP2:BP5 BR2:BR5 BT2:BT5" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Positif,Negatif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2:BL5" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BV2:BV5" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1-3,Bayi Kuning Kramer &gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BN2:BN5" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2:BX5" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1,Bayi Kuning Kramer 2,Bayi Kuning Kramer 3,Bayi Kuning Kramer 4,Bayi Kuning Kramer 5"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BO2:BO5" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BY2:BY5" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"&gt;3 Normal,&lt;=3 Pucat"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: stage 6 fixing skrining-filtering, doing modification for screening nakes and add little bit change on anak
</commit_message>
<xml_diff>
--- a/dataset/anak.xlsx
+++ b/dataset/anak.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69689F7C-0C0C-1545-BFBC-F83AFA9E82E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BA0E03A-DBB2-BF4A-B198-33B4502F6631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -115,7 +115,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="CF1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -130,7 +130,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="CK1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -153,7 +153,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CJ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="CN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -181,7 +181,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="140">
   <si>
     <t>batas_awal</t>
   </si>
@@ -589,6 +589,18 @@
   </si>
   <si>
     <t>skrining_frambusia</t>
+  </si>
+  <si>
+    <t>skrining_warna_kulit_dan_tinja</t>
+  </si>
+  <si>
+    <t>skrining_hasil_kramer</t>
+  </si>
+  <si>
+    <t>skrining_warna_kulit_dan_tinja_28</t>
+  </si>
+  <si>
+    <t>skrining_konfirmasi_shk</t>
   </si>
 </sst>
 </file>
@@ -1024,7 +1036,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CU5"/>
+  <dimension ref="A1:CY5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
@@ -1081,36 +1093,40 @@
     <col min="63" max="63" width="13.6640625" style="6" customWidth="1"/>
     <col min="64" max="64" width="6.1640625" bestFit="1" customWidth="1"/>
     <col min="65" max="66" width="13.6640625" customWidth="1"/>
-    <col min="67" max="67" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="68" max="72" width="22.5" customWidth="1"/>
-    <col min="73" max="73" width="35.83203125" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="22.5" customWidth="1"/>
-    <col min="75" max="75" width="22.5" style="1" customWidth="1"/>
-    <col min="76" max="77" width="22.5" customWidth="1"/>
+    <col min="67" max="67" width="20.83203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="69" max="73" width="22.5" customWidth="1"/>
+    <col min="74" max="74" width="26.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="35.83203125" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="35.83203125" style="6" customWidth="1"/>
+    <col min="77" max="77" width="22.5" customWidth="1"/>
     <col min="78" max="78" width="22.5" style="6" customWidth="1"/>
-    <col min="79" max="79" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="22.83203125" customWidth="1"/>
-    <col min="83" max="83" width="22.83203125" style="6" customWidth="1"/>
-    <col min="84" max="84" width="16.1640625" customWidth="1"/>
-    <col min="85" max="85" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="19.83203125" style="6" customWidth="1"/>
-    <col min="87" max="88" width="12.33203125" customWidth="1"/>
-    <col min="89" max="89" width="12.33203125" style="6" customWidth="1"/>
-    <col min="90" max="90" width="14.1640625" customWidth="1"/>
-    <col min="91" max="91" width="14.1640625" style="6" customWidth="1"/>
-    <col min="92" max="92" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="23.6640625" customWidth="1"/>
-    <col min="94" max="94" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="23.1640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="20" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="22.5" style="1" customWidth="1"/>
+    <col min="80" max="81" width="22.5" customWidth="1"/>
+    <col min="82" max="82" width="22.5" style="6" customWidth="1"/>
+    <col min="83" max="83" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="22.83203125" customWidth="1"/>
+    <col min="87" max="87" width="22.83203125" style="6" customWidth="1"/>
+    <col min="88" max="88" width="16.1640625" customWidth="1"/>
+    <col min="89" max="89" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="19.83203125" style="6" customWidth="1"/>
+    <col min="91" max="92" width="12.33203125" customWidth="1"/>
+    <col min="93" max="93" width="12.33203125" style="6" customWidth="1"/>
+    <col min="94" max="94" width="14.1640625" customWidth="1"/>
+    <col min="95" max="95" width="14.1640625" style="6" customWidth="1"/>
+    <col min="96" max="96" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="23.6640625" customWidth="1"/>
+    <col min="98" max="98" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="23.1640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:99" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:103" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1309,107 +1325,119 @@
       <c r="BN1" t="s">
         <v>52</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BO1" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP1" t="s">
         <v>53</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BQ1" t="s">
         <v>54</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BR1" t="s">
         <v>55</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BS1" t="s">
         <v>56</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BT1" t="s">
         <v>57</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BU1" t="s">
         <v>58</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BV1" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="BW1" t="s">
         <v>59</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="BX1" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="BY1" t="s">
         <v>60</v>
       </c>
-      <c r="BW1" s="1" t="s">
+      <c r="BZ1" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="CA1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CB1" t="s">
         <v>62</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CC1" t="s">
         <v>63</v>
       </c>
-      <c r="BZ1" s="6" t="s">
+      <c r="CD1" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CE1" t="s">
         <v>64</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CF1" t="s">
         <v>65</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CG1" t="s">
         <v>66</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CH1" t="s">
         <v>67</v>
       </c>
-      <c r="CE1" s="6" t="s">
+      <c r="CI1" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CJ1" t="s">
         <v>68</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CK1" t="s">
         <v>69</v>
       </c>
-      <c r="CH1" s="6" t="s">
+      <c r="CL1" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CM1" t="s">
         <v>70</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CN1" t="s">
         <v>71</v>
       </c>
-      <c r="CK1" s="6" t="s">
+      <c r="CO1" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CP1" t="s">
         <v>72</v>
       </c>
-      <c r="CM1" s="6" t="s">
+      <c r="CQ1" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CR1" t="s">
         <v>73</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CS1" t="s">
         <v>74</v>
       </c>
-      <c r="CP1" t="s">
+      <c r="CT1" t="s">
         <v>75</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="CU1" t="s">
         <v>76</v>
       </c>
-      <c r="CR1" t="s">
+      <c r="CV1" t="s">
         <v>77</v>
       </c>
-      <c r="CS1" s="6" t="s">
+      <c r="CW1" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="CX1" t="s">
         <v>78</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="CY1" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:99" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:103" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>80</v>
       </c>
@@ -1533,107 +1561,119 @@
       <c r="BN2" t="s">
         <v>91</v>
       </c>
-      <c r="BO2" t="s">
+      <c r="BO2" s="6" t="s">
         <v>88</v>
       </c>
       <c r="BP2" t="s">
+        <v>88</v>
+      </c>
+      <c r="BQ2" t="s">
         <v>91</v>
       </c>
-      <c r="BQ2" t="s">
-        <v>88</v>
-      </c>
       <c r="BR2" t="s">
+        <v>88</v>
+      </c>
+      <c r="BS2" t="s">
         <v>91</v>
       </c>
-      <c r="BS2" t="s">
-        <v>88</v>
-      </c>
       <c r="BT2" t="s">
+        <v>88</v>
+      </c>
+      <c r="BU2" t="s">
         <v>91</v>
       </c>
-      <c r="BU2" t="s">
-        <v>84</v>
-      </c>
-      <c r="BV2" t="s">
+      <c r="BV2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BW2" t="s">
+        <v>84</v>
+      </c>
+      <c r="BX2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BY2" t="s">
         <v>92</v>
       </c>
-      <c r="BW2" s="1" t="s">
+      <c r="BZ2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CA2" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="BX2" t="s">
+      <c r="CB2" t="s">
         <v>86</v>
       </c>
-      <c r="BY2" t="s">
+      <c r="CC2" t="s">
         <v>94</v>
       </c>
-      <c r="BZ2" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CA2" t="s">
+      <c r="CD2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CE2" t="s">
         <v>95</v>
       </c>
-      <c r="CB2" t="s">
+      <c r="CF2" t="s">
         <v>96</v>
       </c>
-      <c r="CC2" t="s">
+      <c r="CG2" t="s">
         <v>97</v>
       </c>
-      <c r="CD2" t="s">
+      <c r="CH2" t="s">
         <v>98</v>
       </c>
-      <c r="CE2" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CF2" t="s">
+      <c r="CI2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CJ2" t="s">
         <v>99</v>
       </c>
-      <c r="CG2" t="s">
+      <c r="CK2" t="s">
         <v>100</v>
       </c>
-      <c r="CH2" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CI2" t="s">
+      <c r="CL2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CM2" t="s">
         <v>101</v>
       </c>
-      <c r="CJ2" t="s">
+      <c r="CN2" t="s">
         <v>102</v>
       </c>
-      <c r="CK2" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CL2" t="s">
+      <c r="CO2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CP2" t="s">
         <v>99</v>
       </c>
-      <c r="CM2" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CN2" t="s">
+      <c r="CQ2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CR2" t="s">
         <v>103</v>
       </c>
-      <c r="CO2" t="s">
+      <c r="CS2" t="s">
         <v>104</v>
       </c>
-      <c r="CP2" t="s">
+      <c r="CT2" t="s">
         <v>105</v>
       </c>
-      <c r="CQ2" t="s">
+      <c r="CU2" t="s">
         <v>86</v>
       </c>
-      <c r="CR2" t="s">
+      <c r="CV2" t="s">
         <v>86</v>
       </c>
-      <c r="CS2" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CT2" t="s">
+      <c r="CW2" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CX2" t="s">
         <v>95</v>
       </c>
-      <c r="CU2" t="s">
+      <c r="CY2" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="3" spans="1:99" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:103" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>80</v>
       </c>
@@ -1829,107 +1869,119 @@
       <c r="BN3" t="s">
         <v>91</v>
       </c>
-      <c r="BO3" t="s">
+      <c r="BO3" s="6" t="s">
         <v>88</v>
       </c>
       <c r="BP3" t="s">
+        <v>88</v>
+      </c>
+      <c r="BQ3" t="s">
         <v>91</v>
       </c>
-      <c r="BQ3" t="s">
-        <v>88</v>
-      </c>
       <c r="BR3" t="s">
+        <v>88</v>
+      </c>
+      <c r="BS3" t="s">
         <v>91</v>
       </c>
-      <c r="BS3" t="s">
-        <v>88</v>
-      </c>
       <c r="BT3" t="s">
+        <v>88</v>
+      </c>
+      <c r="BU3" t="s">
         <v>91</v>
       </c>
-      <c r="BU3" t="s">
-        <v>84</v>
-      </c>
-      <c r="BV3" t="s">
+      <c r="BV3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BW3" t="s">
+        <v>84</v>
+      </c>
+      <c r="BX3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BY3" t="s">
         <v>92</v>
       </c>
-      <c r="BW3" s="1" t="s">
+      <c r="BZ3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CA3" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="BX3" t="s">
+      <c r="CB3" t="s">
         <v>86</v>
       </c>
-      <c r="BY3" t="s">
+      <c r="CC3" t="s">
         <v>94</v>
       </c>
-      <c r="BZ3" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CA3" t="s">
+      <c r="CD3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CE3" t="s">
         <v>95</v>
       </c>
-      <c r="CB3" t="s">
+      <c r="CF3" t="s">
         <v>96</v>
       </c>
-      <c r="CC3" t="s">
+      <c r="CG3" t="s">
         <v>97</v>
       </c>
-      <c r="CD3" t="s">
+      <c r="CH3" t="s">
         <v>98</v>
       </c>
-      <c r="CE3" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CF3" t="s">
+      <c r="CI3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CJ3" t="s">
         <v>99</v>
       </c>
-      <c r="CG3" t="s">
+      <c r="CK3" t="s">
         <v>100</v>
       </c>
-      <c r="CH3" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CI3" t="s">
+      <c r="CL3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CM3" t="s">
         <v>101</v>
       </c>
-      <c r="CJ3" t="s">
+      <c r="CN3" t="s">
         <v>102</v>
       </c>
-      <c r="CK3" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CL3" t="s">
+      <c r="CO3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CP3" t="s">
         <v>99</v>
       </c>
-      <c r="CM3" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CN3" t="s">
+      <c r="CQ3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CR3" t="s">
         <v>103</v>
       </c>
-      <c r="CO3" t="s">
+      <c r="CS3" t="s">
         <v>104</v>
       </c>
-      <c r="CP3" t="s">
+      <c r="CT3" t="s">
         <v>105</v>
       </c>
-      <c r="CQ3" t="s">
+      <c r="CU3" t="s">
         <v>86</v>
       </c>
-      <c r="CR3" t="s">
+      <c r="CV3" t="s">
         <v>86</v>
       </c>
-      <c r="CS3" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CT3" t="s">
+      <c r="CW3" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CX3" t="s">
         <v>95</v>
       </c>
-      <c r="CU3" t="s">
+      <c r="CY3" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="4" spans="1:99" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:103" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>108</v>
       </c>
@@ -2125,104 +2177,116 @@
       <c r="BN4" t="s">
         <v>91</v>
       </c>
-      <c r="BO4" t="s">
+      <c r="BO4" s="6" t="s">
         <v>88</v>
       </c>
       <c r="BP4" t="s">
+        <v>88</v>
+      </c>
+      <c r="BQ4" t="s">
         <v>91</v>
       </c>
-      <c r="BQ4" t="s">
-        <v>88</v>
-      </c>
       <c r="BR4" t="s">
+        <v>88</v>
+      </c>
+      <c r="BS4" t="s">
         <v>91</v>
       </c>
-      <c r="BS4" t="s">
-        <v>88</v>
-      </c>
       <c r="BT4" t="s">
+        <v>88</v>
+      </c>
+      <c r="BU4" t="s">
         <v>91</v>
       </c>
-      <c r="BU4" t="s">
-        <v>84</v>
-      </c>
-      <c r="BV4" t="s">
+      <c r="BV4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BW4" t="s">
+        <v>84</v>
+      </c>
+      <c r="BX4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BY4" t="s">
         <v>86</v>
       </c>
-      <c r="BW4" s="1" t="s">
+      <c r="BZ4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CA4" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="BX4" t="s">
+      <c r="CB4" t="s">
         <v>86</v>
       </c>
-      <c r="BY4" t="s">
+      <c r="CC4" t="s">
         <v>94</v>
       </c>
-      <c r="BZ4" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CA4" t="s">
+      <c r="CD4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CE4" t="s">
         <v>95</v>
       </c>
-      <c r="CC4" t="s">
+      <c r="CG4" t="s">
         <v>112</v>
       </c>
-      <c r="CD4" t="s">
+      <c r="CH4" t="s">
         <v>98</v>
       </c>
-      <c r="CE4" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CF4" t="s">
+      <c r="CI4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CJ4" t="s">
         <v>99</v>
       </c>
-      <c r="CG4" t="s">
+      <c r="CK4" t="s">
         <v>100</v>
       </c>
-      <c r="CH4" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CI4" t="s">
+      <c r="CL4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CM4" t="s">
         <v>99</v>
       </c>
-      <c r="CJ4" t="s">
+      <c r="CN4" t="s">
         <v>113</v>
       </c>
-      <c r="CK4" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CL4" t="s">
+      <c r="CO4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CP4" t="s">
         <v>99</v>
       </c>
-      <c r="CM4" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CN4" t="s">
+      <c r="CQ4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CR4" t="s">
         <v>103</v>
       </c>
-      <c r="CO4" t="s">
+      <c r="CS4" t="s">
         <v>104</v>
       </c>
-      <c r="CP4" t="s">
+      <c r="CT4" t="s">
         <v>105</v>
       </c>
-      <c r="CQ4" t="s">
+      <c r="CU4" t="s">
         <v>86</v>
       </c>
-      <c r="CR4" t="s">
+      <c r="CV4" t="s">
         <v>86</v>
       </c>
-      <c r="CS4" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CT4" t="s">
+      <c r="CW4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CX4" t="s">
         <v>95</v>
       </c>
-      <c r="CU4" s="4" t="s">
+      <c r="CY4" s="4" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="5" spans="1:99" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:103" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>114</v>
       </c>
@@ -2418,152 +2482,164 @@
       <c r="BN5" t="s">
         <v>91</v>
       </c>
-      <c r="BO5" t="s">
+      <c r="BO5" s="6" t="s">
         <v>88</v>
       </c>
       <c r="BP5" t="s">
+        <v>88</v>
+      </c>
+      <c r="BQ5" t="s">
         <v>91</v>
       </c>
-      <c r="BQ5" t="s">
-        <v>88</v>
-      </c>
       <c r="BR5" t="s">
+        <v>88</v>
+      </c>
+      <c r="BS5" t="s">
         <v>91</v>
       </c>
-      <c r="BS5" t="s">
-        <v>88</v>
-      </c>
       <c r="BT5" t="s">
+        <v>88</v>
+      </c>
+      <c r="BU5" t="s">
         <v>91</v>
       </c>
-      <c r="BU5" t="s">
-        <v>84</v>
-      </c>
-      <c r="BV5" t="s">
+      <c r="BV5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BW5" t="s">
+        <v>84</v>
+      </c>
+      <c r="BX5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="BY5" t="s">
         <v>86</v>
       </c>
-      <c r="BW5" s="1" t="s">
+      <c r="BZ5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CA5" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="BX5" t="s">
+      <c r="CB5" t="s">
         <v>86</v>
       </c>
-      <c r="BY5" t="s">
+      <c r="CC5" t="s">
         <v>94</v>
       </c>
-      <c r="BZ5" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CA5" t="s">
+      <c r="CD5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CE5" t="s">
         <v>95</v>
       </c>
-      <c r="CC5" t="s">
+      <c r="CG5" t="s">
         <v>112</v>
       </c>
-      <c r="CD5" t="s">
+      <c r="CH5" t="s">
         <v>98</v>
       </c>
-      <c r="CE5" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CF5" t="s">
+      <c r="CI5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CJ5" t="s">
         <v>99</v>
       </c>
-      <c r="CG5" t="s">
+      <c r="CK5" t="s">
         <v>100</v>
       </c>
-      <c r="CH5" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CI5" t="s">
+      <c r="CL5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CM5" t="s">
         <v>99</v>
       </c>
-      <c r="CJ5" t="s">
+      <c r="CN5" t="s">
         <v>113</v>
       </c>
-      <c r="CK5" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CL5" t="s">
+      <c r="CO5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CP5" t="s">
         <v>99</v>
       </c>
-      <c r="CM5" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CN5" t="s">
+      <c r="CQ5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CR5" t="s">
         <v>103</v>
       </c>
-      <c r="CO5" t="s">
+      <c r="CS5" t="s">
         <v>104</v>
       </c>
-      <c r="CP5" t="s">
+      <c r="CT5" t="s">
         <v>105</v>
       </c>
-      <c r="CQ5" t="s">
+      <c r="CU5" t="s">
         <v>86</v>
       </c>
-      <c r="CR5" t="s">
+      <c r="CV5" t="s">
         <v>86</v>
       </c>
-      <c r="CS5" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="CT5" t="s">
+      <c r="CW5" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="CX5" t="s">
         <v>95</v>
       </c>
-      <c r="CU5" t="s">
+      <c r="CY5" t="s">
         <v>106</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="27">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:O5 AN2:AN5 AV2:AZ5 BG2:BG5 BO2:BO5 BQ2:BQ5 BS2:BS5 BU2:BU5 D2:D14 F2:G5 M2:M5 BJ2:BK5 AP2:AR5 AT2:AT5 BZ2:BZ5 BB2:BB5 BD2:BD5 AH2:AI5 CS2:CS5 CM2:CM5 CK2:CK5 CH2:CH5 CE2:CE5" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:O5 AN2:AN5 AV2:AZ5 BG2:BG5 BR2:BR5 BT2:BT5 D2:D14 F2:G5 M2:M5 BJ2:BK5 AP2:AR5 AT2:AT5 CD2:CD5 BB2:BB5 BD2:BD5 AH2:AI5 CW2:CW5 CQ2:CQ5 CO2:CO5 CL2:CL5 CI2:CI5 BV2:BX5 BZ2:BZ5 BO2:BP5" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E5" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2:AU5 CD2:CD5" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AU2:AU5 CH2:CH5" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BA2:BA5" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CA2:CA5" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CE2:CE5" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2:CB5" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2:CF5" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2:CC5" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2:CG5" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2:CF5" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2:CJ5" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2:CG5" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2:CK5" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2:CI5" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2:CM5" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2:CJ5" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2:CN5" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2:CL5" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2:CP5" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2:CN5" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2:CR5" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2:CO5" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2:CS5" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2:CP5" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2:CT5" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Sesuai Umur,Ada kemungkinan penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2:CQ5" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CU2:CU5" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CR2:CR5" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2:CV5" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Curiga kelainan pupil putih pada anak"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:L5 N2:AG2" xr:uid="{00000000-0002-0000-0000-000011000000}">
@@ -2578,22 +2654,22 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2:AO5" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"Perkembangan sesuai usia,Perkembangan meragukan,Perkembangan curiga adanya penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2:CT5" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CX2:CX5" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"Tidak ada,1,2,3,&gt;3"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P3:AG5 BC2:BC5" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"Sudah,Belum"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2:BN5 BP2:BP5 BR2:BR5 BT2:BT5" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BU2:BU5 BQ2:BQ5 BS2:BS5 BL2:BN5" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Positif,Negatif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BV2:BV5" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BY2:BY5" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1-3,Bayi Kuning Kramer &gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2:BX5" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2:CB5" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1,Bayi Kuning Kramer 2,Bayi Kuning Kramer 3,Bayi Kuning Kramer 4,Bayi Kuning Kramer 5"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BY2:BY5" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2:CC5" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"&gt;3 Normal,&lt;=3 Pucat"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: update dataset files for anak, dewasa, lansia, and remaja
</commit_message>
<xml_diff>
--- a/dataset/anak.xlsx
+++ b/dataset/anak.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3F6D452-0F0D-F34A-825C-2F6921FF0740}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F29E86-7B5B-7A48-842D-763B89F63E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
     <author>Microsoft Office User</author>
   </authors>
   <commentList>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="K1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -40,7 +40,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -55,7 +55,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -70,7 +70,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
@@ -93,7 +93,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="O1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
       <text>
         <r>
           <rPr>
@@ -108,7 +108,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BB1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+    <comment ref="BD1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
       <text>
         <r>
           <rPr>
@@ -123,7 +123,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CG1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+    <comment ref="CI1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
       <text>
         <r>
           <rPr>
@@ -138,7 +138,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CL1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+    <comment ref="CN1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
       <text>
         <r>
           <rPr>
@@ -161,7 +161,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="CO1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="CQ1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="133">
   <si>
     <t>batas_awal</t>
   </si>
@@ -579,13 +579,22 @@
   </si>
   <si>
     <t>skrining_konfirmasi_shk</t>
+  </si>
+  <si>
+    <t>cari_by_nik</t>
+  </si>
+  <si>
+    <t>nik</t>
+  </si>
+  <si>
+    <t>3512082302650001</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -619,8 +628,15 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF343434"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -636,6 +652,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -676,11 +698,11 @@
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Dark Mode" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -1016,452 +1038,454 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CY4"/>
+  <dimension ref="A1:DA5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.5" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="13.83203125" style="8" customWidth="1"/>
-    <col min="12" max="12" width="21.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="23.83203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="27.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="23.83203125" style="8" customWidth="1"/>
-    <col min="17" max="17" width="29" style="8" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="23.83203125" style="8" customWidth="1"/>
-    <col min="19" max="19" width="22.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="22.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="23.83203125" style="8" customWidth="1"/>
-    <col min="23" max="23" width="27.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="27.1640625" style="8" customWidth="1"/>
-    <col min="26" max="26" width="24.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="29" style="8" bestFit="1" customWidth="1"/>
-    <col min="28" max="34" width="29" style="8" customWidth="1"/>
-    <col min="35" max="35" width="19.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="23.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="37" max="38" width="14.33203125" style="8" customWidth="1"/>
-    <col min="39" max="39" width="16.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="19" style="8" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="29" style="8" customWidth="1"/>
-    <col min="42" max="42" width="23.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="29" style="8" customWidth="1"/>
-    <col min="44" max="44" width="19" style="8" customWidth="1"/>
-    <col min="45" max="45" width="29" style="8" customWidth="1"/>
-    <col min="46" max="47" width="19" style="8" customWidth="1"/>
-    <col min="48" max="48" width="25" style="8" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="8.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="19.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="4.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="23.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="14.83203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="14.83203125" style="8" customWidth="1"/>
-    <col min="55" max="55" width="26.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="28.83203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="28.83203125" style="8" customWidth="1"/>
-    <col min="58" max="58" width="10" style="8" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="13.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="22.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="16" style="8" bestFit="1" customWidth="1"/>
-    <col min="62" max="64" width="13.6640625" style="8" customWidth="1"/>
-    <col min="65" max="65" width="6.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="66" max="67" width="13.6640625" style="8" customWidth="1"/>
-    <col min="68" max="68" width="20.83203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="22.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="70" max="74" width="22.5" style="8" customWidth="1"/>
-    <col min="75" max="75" width="26.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="35.83203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="35.83203125" style="8" customWidth="1"/>
-    <col min="78" max="79" width="22.5" style="8" customWidth="1"/>
-    <col min="80" max="80" width="22.5" style="7" customWidth="1"/>
-    <col min="81" max="83" width="22.5" style="8" customWidth="1"/>
-    <col min="84" max="84" width="21.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="11.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="22.83203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="87" max="88" width="22.83203125" style="8" customWidth="1"/>
-    <col min="89" max="89" width="16.1640625" style="8" customWidth="1"/>
-    <col min="90" max="90" width="19.83203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="19.83203125" style="8" customWidth="1"/>
-    <col min="92" max="94" width="12.33203125" style="8" customWidth="1"/>
-    <col min="95" max="96" width="14.1640625" style="8" customWidth="1"/>
-    <col min="97" max="97" width="23.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="23.6640625" style="8" customWidth="1"/>
-    <col min="99" max="99" width="14.83203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="18.83203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="10.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="23.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="16.5" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="18.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="13.83203125" customWidth="1"/>
+    <col min="14" max="14" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="27.1640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="23.83203125" customWidth="1"/>
+    <col min="19" max="19" width="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="23.83203125" customWidth="1"/>
+    <col min="21" max="21" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="23.83203125" customWidth="1"/>
+    <col min="25" max="25" width="27.1640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="27.1640625" customWidth="1"/>
+    <col min="28" max="28" width="24.5" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="36" width="29" customWidth="1"/>
+    <col min="37" max="37" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="39" max="40" width="14.33203125" customWidth="1"/>
+    <col min="41" max="41" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="19" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="29" customWidth="1"/>
+    <col min="44" max="44" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="29" customWidth="1"/>
+    <col min="46" max="46" width="19" customWidth="1"/>
+    <col min="47" max="47" width="29" customWidth="1"/>
+    <col min="48" max="49" width="19" customWidth="1"/>
+    <col min="50" max="50" width="25" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="14.83203125" customWidth="1"/>
+    <col min="57" max="57" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="28.83203125" customWidth="1"/>
+    <col min="60" max="60" width="10" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="22.1640625" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="16" bestFit="1" customWidth="1"/>
+    <col min="64" max="66" width="13.6640625" customWidth="1"/>
+    <col min="67" max="67" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="68" max="69" width="13.6640625" customWidth="1"/>
+    <col min="70" max="70" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="72" max="76" width="22.5" customWidth="1"/>
+    <col min="77" max="77" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="35.83203125" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="35.83203125" customWidth="1"/>
+    <col min="80" max="81" width="22.5" customWidth="1"/>
+    <col min="82" max="82" width="22.5" style="1" customWidth="1"/>
+    <col min="83" max="85" width="22.5" customWidth="1"/>
+    <col min="86" max="86" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="89" max="90" width="22.83203125" customWidth="1"/>
+    <col min="91" max="91" width="16.1640625" customWidth="1"/>
+    <col min="92" max="92" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="19.83203125" customWidth="1"/>
+    <col min="94" max="96" width="12.33203125" customWidth="1"/>
+    <col min="97" max="98" width="14.1640625" customWidth="1"/>
+    <col min="99" max="99" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="23.6640625" customWidth="1"/>
+    <col min="101" max="101" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="105" max="105" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:103" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:105" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>79</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>6</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>7</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>8</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>9</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
         <v>10</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>11</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="S1" t="s">
         <v>12</v>
       </c>
-      <c r="R1" t="s">
+      <c r="T1" t="s">
         <v>13</v>
       </c>
-      <c r="S1" t="s">
+      <c r="U1" t="s">
         <v>14</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AC1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AD1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AF1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AG1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AH1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="AG1" s="3" t="s">
+      <c r="AI1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="AH1" s="3" t="s">
+      <c r="AJ1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AI1" s="6" t="s">
+      <c r="AK1" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="AJ1" s="6" t="s">
+      <c r="AL1" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AM1" t="s">
         <v>30</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AN1" t="s">
         <v>31</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AO1" t="s">
         <v>32</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AP1" t="s">
         <v>33</v>
       </c>
-      <c r="AO1" s="6" t="s">
+      <c r="AQ1" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AR1" t="s">
         <v>34</v>
       </c>
-      <c r="AQ1" s="6" t="s">
+      <c r="AS1" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AT1" t="s">
         <v>35</v>
       </c>
-      <c r="AS1" s="6" t="s">
+      <c r="AU1" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AV1" t="s">
         <v>36</v>
       </c>
-      <c r="AU1" s="5" t="s">
+      <c r="AW1" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AX1" t="s">
         <v>37</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AY1" t="s">
         <v>38</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AZ1" t="s">
         <v>39</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="BA1" t="s">
         <v>40</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BB1" t="s">
         <v>41</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BC1" t="s">
         <v>42</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BD1" t="s">
         <v>43</v>
       </c>
-      <c r="BC1" s="5" t="s">
+      <c r="BE1" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BF1" t="s">
         <v>44</v>
       </c>
-      <c r="BE1" s="5" t="s">
+      <c r="BG1" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BH1" t="s">
         <v>45</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BI1" t="s">
         <v>46</v>
       </c>
-      <c r="BH1" s="5" t="s">
+      <c r="BJ1" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BK1" t="s">
         <v>47</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BL1" t="s">
         <v>48</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BM1" t="s">
         <v>49</v>
       </c>
-      <c r="BL1" s="5" t="s">
+      <c r="BN1" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BO1" t="s">
         <v>50</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BP1" t="s">
         <v>51</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BQ1" t="s">
         <v>52</v>
       </c>
-      <c r="BP1" s="5" t="s">
+      <c r="BR1" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BS1" t="s">
         <v>53</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BT1" t="s">
         <v>54</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BU1" t="s">
         <v>55</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="BV1" t="s">
         <v>56</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="BW1" t="s">
         <v>57</v>
       </c>
-      <c r="BV1" t="s">
+      <c r="BX1" t="s">
         <v>58</v>
       </c>
-      <c r="BW1" s="5" t="s">
+      <c r="BY1" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="BZ1" t="s">
         <v>59</v>
       </c>
-      <c r="BY1" s="5" t="s">
+      <c r="CA1" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CB1" t="s">
         <v>60</v>
       </c>
-      <c r="CA1" s="5" t="s">
+      <c r="CC1" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="CB1" s="1" t="s">
+      <c r="CD1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="CC1" t="s">
+      <c r="CE1" t="s">
         <v>62</v>
       </c>
-      <c r="CD1" t="s">
+      <c r="CF1" t="s">
         <v>63</v>
       </c>
-      <c r="CE1" s="5" t="s">
+      <c r="CG1" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="CF1" t="s">
+      <c r="CH1" t="s">
         <v>64</v>
       </c>
-      <c r="CG1" t="s">
+      <c r="CI1" t="s">
         <v>65</v>
       </c>
-      <c r="CH1" t="s">
+      <c r="CJ1" t="s">
         <v>66</v>
       </c>
-      <c r="CI1" t="s">
+      <c r="CK1" t="s">
         <v>67</v>
       </c>
-      <c r="CJ1" s="5" t="s">
+      <c r="CL1" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="CM1" t="s">
         <v>68</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CN1" t="s">
         <v>69</v>
       </c>
-      <c r="CM1" s="5" t="s">
+      <c r="CO1" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="CP1" t="s">
         <v>70</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="CQ1" t="s">
         <v>71</v>
       </c>
-      <c r="CP1" s="5" t="s">
+      <c r="CR1" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="CQ1" t="s">
+      <c r="CS1" t="s">
         <v>72</v>
       </c>
-      <c r="CR1" s="5" t="s">
+      <c r="CT1" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="CS1" t="s">
+      <c r="CU1" t="s">
         <v>73</v>
       </c>
-      <c r="CT1" t="s">
+      <c r="CV1" t="s">
         <v>74</v>
       </c>
-      <c r="CU1" t="s">
+      <c r="CW1" t="s">
         <v>75</v>
       </c>
-      <c r="CV1" t="s">
+      <c r="CX1" t="s">
         <v>76</v>
       </c>
-      <c r="CW1" t="s">
+      <c r="CY1" t="s">
         <v>77</v>
       </c>
-      <c r="CX1" s="5" t="s">
+      <c r="CZ1" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="CY1" t="s">
+      <c r="DA1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:103" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:105" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="8"/>
+      <c r="E2" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>105</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="G2" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H2" t="s">
         <v>82</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H2" t="s">
-        <v>83</v>
-      </c>
-      <c r="I2"/>
+      <c r="I2" s="4" t="s">
+        <v>87</v>
+      </c>
       <c r="J2" t="s">
         <v>83</v>
       </c>
-      <c r="K2" t="s">
-        <v>83</v>
-      </c>
       <c r="L2" t="s">
         <v>83</v>
       </c>
       <c r="M2" t="s">
         <v>83</v>
       </c>
-      <c r="N2" s="4" t="s">
-        <v>87</v>
+      <c r="N2" t="s">
+        <v>83</v>
       </c>
       <c r="O2" t="s">
-        <v>87</v>
-      </c>
-      <c r="P2" t="s">
+        <v>83</v>
+      </c>
+      <c r="P2" s="4" t="s">
         <v>87</v>
       </c>
       <c r="Q2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="R2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="S2" t="s">
         <v>89</v>
@@ -1511,54 +1535,54 @@
       <c r="AH2" t="s">
         <v>89</v>
       </c>
-      <c r="AI2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="AJ2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="AK2">
+      <c r="AI2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AK2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="AL2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="AM2">
         <v>5</v>
       </c>
-      <c r="AL2">
+      <c r="AN2">
         <v>100</v>
       </c>
-      <c r="AM2" t="s">
+      <c r="AO2" t="s">
         <v>84</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AP2" t="s">
         <v>85</v>
       </c>
-      <c r="AO2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="AP2" t="s">
+      <c r="AQ2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="AR2" t="s">
         <v>86</v>
       </c>
-      <c r="AQ2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>87</v>
-      </c>
       <c r="AS2" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="AT2">
+      <c r="AT2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AU2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="AV2">
         <v>10</v>
       </c>
-      <c r="AU2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="AV2" t="s">
+      <c r="AW2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="AX2" t="s">
         <v>88</v>
       </c>
-      <c r="AW2" t="s">
-        <v>87</v>
-      </c>
-      <c r="AX2" t="s">
-        <v>87</v>
-      </c>
       <c r="AY2" t="s">
         <v>87</v>
       </c>
@@ -1569,55 +1593,55 @@
         <v>87</v>
       </c>
       <c r="BB2" t="s">
+        <v>87</v>
+      </c>
+      <c r="BC2" t="s">
+        <v>87</v>
+      </c>
+      <c r="BD2" t="s">
         <v>85</v>
       </c>
-      <c r="BC2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="BD2" t="s">
+      <c r="BE2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="BF2" t="s">
         <v>89</v>
       </c>
-      <c r="BE2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="BF2">
+      <c r="BG2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="BH2">
         <v>2900</v>
       </c>
-      <c r="BG2">
+      <c r="BI2">
         <v>6000</v>
       </c>
-      <c r="BH2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="BI2">
+      <c r="BJ2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="BK2">
         <v>80</v>
       </c>
-      <c r="BJ2">
+      <c r="BL2">
         <v>90</v>
       </c>
-      <c r="BK2" t="s">
-        <v>87</v>
-      </c>
-      <c r="BL2" s="5" t="s">
-        <v>87</v>
-      </c>
       <c r="BM2" t="s">
-        <v>90</v>
-      </c>
-      <c r="BN2" t="s">
-        <v>90</v>
+        <v>87</v>
+      </c>
+      <c r="BN2" s="5" t="s">
+        <v>87</v>
       </c>
       <c r="BO2" t="s">
         <v>90</v>
       </c>
-      <c r="BP2" s="5" t="s">
-        <v>87</v>
+      <c r="BP2" t="s">
+        <v>90</v>
       </c>
       <c r="BQ2" t="s">
-        <v>87</v>
-      </c>
-      <c r="BR2" t="s">
         <v>90</v>
+      </c>
+      <c r="BR2" s="5" t="s">
+        <v>87</v>
       </c>
       <c r="BS2" t="s">
         <v>87</v>
@@ -1631,182 +1655,198 @@
       <c r="BV2" t="s">
         <v>90</v>
       </c>
-      <c r="BW2" s="5" t="s">
+      <c r="BW2" t="s">
         <v>87</v>
       </c>
       <c r="BX2" t="s">
+        <v>90</v>
+      </c>
+      <c r="BY2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="BZ2" t="s">
         <v>83</v>
       </c>
-      <c r="BY2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="BZ2" t="s">
+      <c r="CA2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="CB2" t="s">
         <v>91</v>
       </c>
-      <c r="CA2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="CB2" s="1" t="s">
+      <c r="CC2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="CD2" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="CC2" t="s">
+      <c r="CE2" t="s">
         <v>85</v>
       </c>
-      <c r="CD2" t="s">
+      <c r="CF2" t="s">
         <v>93</v>
       </c>
-      <c r="CE2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="CF2" t="s">
+      <c r="CG2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="CH2" t="s">
         <v>94</v>
       </c>
-      <c r="CG2" t="s">
+      <c r="CI2" t="s">
         <v>95</v>
       </c>
-      <c r="CH2" t="s">
+      <c r="CJ2" t="s">
         <v>96</v>
       </c>
-      <c r="CI2" t="s">
+      <c r="CK2" t="s">
         <v>97</v>
       </c>
-      <c r="CJ2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="CK2" t="s">
+      <c r="CL2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="CM2" t="s">
         <v>98</v>
       </c>
-      <c r="CL2" t="s">
+      <c r="CN2" t="s">
         <v>99</v>
       </c>
-      <c r="CM2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="CN2" t="s">
+      <c r="CO2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="CP2" t="s">
         <v>100</v>
       </c>
-      <c r="CO2" t="s">
+      <c r="CQ2" t="s">
         <v>101</v>
       </c>
-      <c r="CP2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="CQ2" t="s">
+      <c r="CR2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="CS2" t="s">
         <v>98</v>
       </c>
-      <c r="CR2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="CS2" t="s">
+      <c r="CT2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="CU2" t="s">
         <v>102</v>
       </c>
-      <c r="CT2" t="s">
+      <c r="CV2" t="s">
         <v>103</v>
       </c>
-      <c r="CU2" t="s">
+      <c r="CW2" t="s">
         <v>104</v>
       </c>
-      <c r="CV2" t="s">
+      <c r="CX2" t="s">
         <v>85</v>
       </c>
-      <c r="CW2" t="s">
+      <c r="CY2" t="s">
         <v>85</v>
       </c>
-      <c r="CX2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="CY2" t="s">
+      <c r="CZ2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="DA2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="3" spans="1:103" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D3" s="9"/>
-      <c r="G3" s="7"/>
-      <c r="N3" s="7"/>
+    <row r="3" spans="1:105" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D3" s="8"/>
+      <c r="F3" s="7"/>
+      <c r="I3" s="1"/>
+      <c r="P3" s="1"/>
     </row>
-    <row r="4" spans="1:103" x14ac:dyDescent="0.2">
-      <c r="G4" s="7"/>
-      <c r="N4" s="7"/>
+    <row r="4" spans="1:105" x14ac:dyDescent="0.2">
+      <c r="C4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="I4" s="1"/>
+      <c r="P4" s="1"/>
+    </row>
+    <row r="5" spans="1:105" ht="18" x14ac:dyDescent="0.2">
+      <c r="D5" s="9"/>
     </row>
   </sheetData>
   <dataValidations count="27">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BP2:BQ4 CA2:CA4 BW2:BY4 CJ2:CJ4 CM2:CM4 CP2:CP4 CR2:CR4 CX2:CX4 AI2:AJ4 BE2:BE4 BC2:BC4 CE2:CE4 AU2:AU4 AQ2:AS4 BK2:BL4 N2:P4 G2:H4 E2:E13 BU2:BU4 BS2:BS4 BH2:BH4 AW2:BA4 AO2:AO4" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BR2:BS4 CC2:CC4 BY2:CA4 CL2:CL4 CO2:CO4 CR2:CR4 CT2:CT4 CZ2:CZ4 AK2:AL4 BG2:BG4 BE2:BE4 CG2:CG4 AW2:AW4 AS2:AU4 BM2:BN4 P2:R4 I2:J4 G2:G13 BW2:BW4 BU2:BU4 BJ2:BJ4 AY2:BC4 AQ2:AQ4" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:AH4 BD2:BD4" xr:uid="{00000000-0002-0000-0000-000016000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:AJ4 BF2:BF4" xr:uid="{00000000-0002-0000-0000-000016000000}">
       <formula1>"Sudah,Belum"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F4" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H4" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Non disabilitas,Penyandang disabilitas"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV2:AV4 CI2:CI4" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BB2:BB4" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX2:AX4 CK2:CK4" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BD2:BD4" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Normal,Abnormal TBC,Abnormal non TBC"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2:CF4" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2:CH4" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Riwayat kontak serumah,Riwayat kontak erat,Tidak ada,Tidak diketahui"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CG2:CG4" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CI2:CI4" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Bakteriologis,Klinis"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CH2:CH4" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CJ2:CJ4" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"TCM,BTA,NPOC,Tidak dilakukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CK2:CK4" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CM2:CM4" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"Suspek frambusia,Bukan frambusia,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CL2:CL4" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2:CN4" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"Reaktif,Non Reaktif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CN2:CN4" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CP2:CP4" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CO2:CO4" xr:uid="{00000000-0002-0000-0000-00000A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2:CQ4" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Kusta,Bukan kusta,Meragukan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CQ2:CQ4" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2:CS4" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>"Skabies,Bukan Skabies,Meragukan,Tidak Ada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CS2:CS4" xr:uid="{00000000-0002-0000-0000-00000C000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CU2:CU4" xr:uid="{00000000-0002-0000-0000-00000C000000}">
       <formula1>"Tidak ada serumen impaksi,Ada serumen impaksi"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CT2:CT4" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2:CV4" xr:uid="{00000000-0002-0000-0000-00000D000000}">
       <formula1>"Tidak ada infeksi telinga,Ada infeksi telinga"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CU2:CU4" xr:uid="{00000000-0002-0000-0000-00000E000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CW2:CW4" xr:uid="{00000000-0002-0000-0000-00000E000000}">
       <formula1>"Sesuai Umur,Ada kemungkinan penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CV2:CV4" xr:uid="{00000000-0002-0000-0000-00000F000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CX2:CX4" xr:uid="{00000000-0002-0000-0000-00000F000000}">
       <formula1>"Normal,Curiga kelainan mata"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CW2:CW4" xr:uid="{00000000-0002-0000-0000-000010000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CY2:CY4" xr:uid="{00000000-0002-0000-0000-000010000000}">
       <formula1>"Normal,Curiga kelainan pupil putih pada anak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:M4" xr:uid="{00000000-0002-0000-0000-000011000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:O4" xr:uid="{00000000-0002-0000-0000-000011000000}">
       <formula1>"Iya,Tidak"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AM2:AM4" xr:uid="{00000000-0002-0000-0000-000012000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AO2:AO4" xr:uid="{00000000-0002-0000-0000-000012000000}">
       <formula1>"Berdiri,Telentang"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN2:AN4" xr:uid="{00000000-0002-0000-0000-000013000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AP2:AP4" xr:uid="{00000000-0002-0000-0000-000013000000}">
       <formula1>"Makrosefali,Normal,Mikrosefali"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AP2:AP4" xr:uid="{00000000-0002-0000-0000-000014000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AR2:AR4" xr:uid="{00000000-0002-0000-0000-000014000000}">
       <formula1>"Perkembangan sesuai usia,Perkembangan meragukan,Perkembangan curiga adanya penyimpangan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CY2:CY4" xr:uid="{00000000-0002-0000-0000-000015000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="DA2:DA4" xr:uid="{00000000-0002-0000-0000-000015000000}">
       <formula1>"Tidak ada,1,2,3,&gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BV2:BV4 BM2:BO4 BT2:BT4 BR2:BR4" xr:uid="{00000000-0002-0000-0000-000017000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BX2:BX4 BO2:BQ4 BV2:BV4 BT2:BT4" xr:uid="{00000000-0002-0000-0000-000017000000}">
       <formula1>"Positif,Negatif"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ2:BZ4" xr:uid="{00000000-0002-0000-0000-000018000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CB2:CB4" xr:uid="{00000000-0002-0000-0000-000018000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1-3,Bayi Kuning Kramer &gt;3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CC2:CC4" xr:uid="{00000000-0002-0000-0000-000019000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CE2:CE4" xr:uid="{00000000-0002-0000-0000-000019000000}">
       <formula1>"Normal,Bayi Kuning Kramer 1,Bayi Kuning Kramer 2,Bayi Kuning Kramer 3,Bayi Kuning Kramer 4,Bayi Kuning Kramer 5"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CD2:CD4" xr:uid="{00000000-0002-0000-0000-00001A000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="CF2:CF4" xr:uid="{00000000-0002-0000-0000-00001A000000}">
       <formula1>"&gt;3 Normal,&lt;=3 Pucat"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>